<commit_message>
Testování výstupů a zpracovani dat z KN.
</commit_message>
<xml_diff>
--- a/GIS2/vystup.xlsx
+++ b/GIS2/vystup.xlsx
@@ -472,7 +472,7 @@
     </row>
     <row r="2">
       <c r="A2" t="n">
-        <v>55</v>
+        <v>661</v>
       </c>
       <c r="B2" t="inlineStr">
         <is>
@@ -486,17 +486,17 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>69/26</t>
+          <t>st. 110</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>Říčany-Radošovice</t>
+          <t>Nová Ves u Prahy</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>č. 69/26 Říčany-Radošovice</t>
+          <t>stavební č. 110 Nová Ves u Prahy</t>
         </is>
       </c>
       <c r="G2" t="n">
@@ -510,11 +510,11 @@
     </row>
     <row r="3">
       <c r="A3" t="n">
-        <v>56</v>
+        <v>662</v>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>budova</t>
+          <t>parcela</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -524,17 +524,17 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>st. 736</t>
+          <t>172/40</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>Říčany-Radošovice</t>
+          <t>Nová Ves u Prahy</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>stavební č. 736 Říčany-Radošovice (součástí je stavba č.p. 366, čst obce Radošovice)</t>
+          <t>č. 172/40 Nová Ves u Prahy</t>
         </is>
       </c>
       <c r="G3" t="n">
@@ -542,17 +542,17 @@
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>č. + KU</t>
+          <t>číslo a KU za ním</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="n">
-        <v>57</v>
+        <v>663</v>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>parcela</t>
+          <t>budova</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -562,17 +562,17 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>92/13</t>
+          <t>st. 602</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>Říčany-Radošovice</t>
+          <t>Nová Ves u Prahy</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>č. 92/13 Říčany-Radošovice</t>
+          <t>stavební č. 602 Nová Ves u Prahy (součástí je stavba č.p. 519, čst obce Nová Ves)</t>
         </is>
       </c>
       <c r="G4" t="n">
@@ -580,13 +580,13 @@
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>číslo a KU za ním</t>
+          <t>č. + KU</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="n">
-        <v>58</v>
+        <v>664</v>
       </c>
       <c r="B5" t="inlineStr">
         <is>
@@ -600,17 +600,17 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>561/6</t>
+          <t>173/122</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>Říčany-Radošovice</t>
+          <t>Nová Ves u Prahy</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>č. 561/6 Říčany-Radošovice</t>
+          <t>č. 173/122 Nová Ves u Prahy</t>
         </is>
       </c>
       <c r="G5" t="n">
@@ -624,7 +624,7 @@
     </row>
     <row r="6">
       <c r="A6" t="n">
-        <v>63</v>
+        <v>665</v>
       </c>
       <c r="B6" t="inlineStr">
         <is>
@@ -638,17 +638,17 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>263/2</t>
+          <t>173/127</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>Těptín</t>
+          <t>Nová Ves u Prahy</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>č. 263/2 Těptín</t>
+          <t>č. 173/127 Nová Ves u Prahy</t>
         </is>
       </c>
       <c r="G6" t="n">
@@ -662,11 +662,11 @@
     </row>
     <row r="7">
       <c r="A7" t="n">
-        <v>64</v>
+        <v>16796</v>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>parcela</t>
+          <t>budova</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
@@ -676,17 +676,17 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>516/3</t>
+          <t>st. 323</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>Těptín</t>
+          <t>Nová Ves u Prahy</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>č. 516/3 Těptín</t>
+          <t>stavební č. 323 Nová Ves u Prahy (součástí je stavba č.p. 247, čst obce Nová Ves)</t>
         </is>
       </c>
       <c r="G7" t="n">
@@ -694,17 +694,17 @@
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>číslo a KU za ním</t>
+          <t>č. + KU</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="n">
-        <v>65</v>
+        <v>16797</v>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>jednotka</t>
+          <t>parcela</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
@@ -714,17 +714,17 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>st. 1105</t>
+          <t>95/66</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>Těptín</t>
+          <t>Nová Ves u Prahy</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>jednotka č. 280014, byt v budově č.p. 28, část obce Kamenice, na parcele st. 1105 Těptín, podíl na společných částech domu a pozemku 381/6380</t>
+          <t>č. 95/66 Nová Ves u Prahy</t>
         </is>
       </c>
       <c r="G8" t="n">
@@ -732,17 +732,17 @@
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>jednotka na parcele s prefixem st. + KU</t>
+          <t>číslo a KU za ním</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="n">
-        <v>66</v>
+        <v>16798</v>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>parcela</t>
+          <t>jednotka</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -752,17 +752,17 @@
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>619/1</t>
+          <t>st. 298</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>Těptín</t>
+          <t>Nová Ves u Prahy</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>č. 619/1 Těptín</t>
+          <t>jednotka č. 2650083, byt v budově č.p. 265, část obce Nová Ves, na parcele st. 298 Nová Ves u Prahy, podíl na společných částech domu a pozemku 620/1984</t>
         </is>
       </c>
       <c r="G9" t="n">
@@ -770,13 +770,13 @@
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>číslo a KU za ním</t>
+          <t>jednotka na parcele s prefixem st. + KU</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="n">
-        <v>67</v>
+        <v>16799</v>
       </c>
       <c r="B10" t="inlineStr">
         <is>
@@ -790,17 +790,17 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>725/28</t>
+          <t>95/218</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>Těptín</t>
+          <t>Nová Ves u Prahy</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>č. 725/28 Těptín</t>
+          <t>č. 95/218 Nová Ves u Prahy</t>
         </is>
       </c>
       <c r="G10" t="n">
@@ -814,11 +814,11 @@
     </row>
     <row r="11">
       <c r="A11" t="n">
-        <v>68</v>
+        <v>16800</v>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>budova</t>
+          <t>parcela</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
@@ -828,17 +828,17 @@
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>st. 1603</t>
+          <t>95/131</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>Těptín</t>
+          <t>Nová Ves u Prahy</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>stavební č. 1603 Těptín (součástí je stavba č.p. 2833, čst obce Těptín)</t>
+          <t>č. 95/131 Nová Ves u Prahy</t>
         </is>
       </c>
       <c r="G11" t="n">
@@ -846,7 +846,7 @@
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>č. + KU</t>
+          <t>číslo a KU za ním</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Upravena FCE na hledani kodu ku v Praze pres kombinaci obec + ku
</commit_message>
<xml_diff>
--- a/GIS2/vystup.xlsx
+++ b/GIS2/vystup.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H11"/>
+  <dimension ref="A1:H64"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -472,7 +472,7 @@
     </row>
     <row r="2">
       <c r="A2" t="n">
-        <v>661</v>
+        <v>58842</v>
       </c>
       <c r="B2" t="inlineStr">
         <is>
@@ -481,22 +481,22 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Praha-východ</t>
+          <t>Hlavní město Praha</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>st. 110</t>
+          <t>1044/2</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>Nová Ves u Prahy</t>
+          <t>Libuš</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>stavební č. 110 Nová Ves u Prahy</t>
+          <t>č. 1044/2 Libuš</t>
         </is>
       </c>
       <c r="G2" t="n">
@@ -510,31 +510,31 @@
     </row>
     <row r="3">
       <c r="A3" t="n">
-        <v>662</v>
+        <v>58841</v>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>parcela</t>
+          <t>budova</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Praha-východ</t>
+          <t>Hlavní město Praha</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>172/40</t>
+          <t>1044/4</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>Nová Ves u Prahy</t>
+          <t>Libuš</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>č. 172/40 Nová Ves u Prahy</t>
+          <t>č. 1044/4 Libuš (součástí je stavba č.p. 957, čst obce Libuš)</t>
         </is>
       </c>
       <c r="G3" t="n">
@@ -542,37 +542,37 @@
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>číslo a KU za ním</t>
+          <t>č. + KU</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="n">
-        <v>663</v>
+        <v>58840</v>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>budova</t>
+          <t>parcela</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Praha-východ</t>
+          <t>Hlavní město Praha</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>st. 602</t>
+          <t>1087/2</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>Nová Ves u Prahy</t>
+          <t>Libuš</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>stavební č. 602 Nová Ves u Prahy (součástí je stavba č.p. 519, čst obce Nová Ves)</t>
+          <t>č. 1087/2 Libuš</t>
         </is>
       </c>
       <c r="G4" t="n">
@@ -580,13 +580,13 @@
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>č. + KU</t>
+          <t>číslo a KU za ním</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="n">
-        <v>664</v>
+        <v>58839</v>
       </c>
       <c r="B5" t="inlineStr">
         <is>
@@ -595,22 +595,22 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Praha-východ</t>
+          <t>Hlavní město Praha</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>173/122</t>
+          <t>1088</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>Nová Ves u Prahy</t>
+          <t>Libuš</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>č. 173/122 Nová Ves u Prahy</t>
+          <t>č. 1088 Libuš</t>
         </is>
       </c>
       <c r="G5" t="n">
@@ -624,31 +624,31 @@
     </row>
     <row r="6">
       <c r="A6" t="n">
-        <v>665</v>
+        <v>58838</v>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>parcela</t>
+          <t>budova</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Praha-východ</t>
+          <t>Hlavní město Praha</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>173/127</t>
+          <t>1087/1</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>Nová Ves u Prahy</t>
+          <t>Libuš</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>č. 173/127 Nová Ves u Prahy</t>
+          <t>č. 1087/1 Libuš (součástí je stavba č.p. 435, čst obce Libuš)</t>
         </is>
       </c>
       <c r="G6" t="n">
@@ -656,37 +656,37 @@
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>číslo a KU za ním</t>
+          <t>č. + KU</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="n">
-        <v>16796</v>
+        <v>58837</v>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>budova</t>
+          <t>parcela</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Praha-východ</t>
+          <t>Hlavní město Praha</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>st. 323</t>
+          <t>546/1</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>Nová Ves u Prahy</t>
+          <t>Libuš</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>stavební č. 323 Nová Ves u Prahy (součástí je stavba č.p. 247, čst obce Nová Ves)</t>
+          <t>č. 546/1 Libuš</t>
         </is>
       </c>
       <c r="G7" t="n">
@@ -694,13 +694,13 @@
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>č. + KU</t>
+          <t>číslo a KU za ním</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="n">
-        <v>16797</v>
+        <v>58836</v>
       </c>
       <c r="B8" t="inlineStr">
         <is>
@@ -709,22 +709,22 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Praha-východ</t>
+          <t>Hlavní město Praha</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>95/66</t>
+          <t>546/3</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>Nová Ves u Prahy</t>
+          <t>Libuš</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>č. 95/66 Nová Ves u Prahy</t>
+          <t>č. 546/3 Libuš</t>
         </is>
       </c>
       <c r="G8" t="n">
@@ -738,31 +738,31 @@
     </row>
     <row r="9">
       <c r="A9" t="n">
-        <v>16798</v>
+        <v>58835</v>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>jednotka</t>
+          <t>budova</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Praha-východ</t>
+          <t>Hlavní město Praha</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>st. 298</t>
+          <t>546/2</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>Nová Ves u Prahy</t>
+          <t>Libuš</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>jednotka č. 2650083, byt v budově č.p. 265, část obce Nová Ves, na parcele st. 298 Nová Ves u Prahy, podíl na společných částech domu a pozemku 620/1984</t>
+          <t>č. 546/2 Libuš (součástí je stavba budova bez čp/če, jiná stavba)</t>
         </is>
       </c>
       <c r="G9" t="n">
@@ -770,37 +770,37 @@
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>jednotka na parcele s prefixem st. + KU</t>
+          <t>č. + KU</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="n">
-        <v>16799</v>
+        <v>58834</v>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>parcela</t>
+          <t>budova</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Praha-východ</t>
+          <t>Hlavní město Praha</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>95/218</t>
+          <t>546/4</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>Nová Ves u Prahy</t>
+          <t>Libuš</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>č. 95/218 Nová Ves u Prahy</t>
+          <t>č. 546/4 Libuš (součástí je stavba budova bez čp/če, jiná stavba)</t>
         </is>
       </c>
       <c r="G10" t="n">
@@ -808,13 +808,13 @@
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>číslo a KU za ním</t>
+          <t>č. + KU</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="n">
-        <v>16800</v>
+        <v>58833</v>
       </c>
       <c r="B11" t="inlineStr">
         <is>
@@ -823,28 +823,2042 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Praha-východ</t>
+          <t>Hlavní město Praha</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>95/131</t>
+          <t>835/84</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>Nová Ves u Prahy</t>
+          <t>Písnice</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>č. 95/131 Nová Ves u Prahy</t>
+          <t>č. 835/84 Písnice</t>
         </is>
       </c>
       <c r="G11" t="n">
         <v>1</v>
       </c>
       <c r="H11" t="inlineStr">
+        <is>
+          <t>číslo a KU za ním</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="n">
+        <v>58832</v>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>parcela</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>Hlavní město Praha</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>761</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>Písnice</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>č. 761 Písnice</t>
+        </is>
+      </c>
+      <c r="G12" t="n">
+        <v>1</v>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>číslo a KU za ním</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="n">
+        <v>58831</v>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>budova</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>Hlavní město Praha</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>760</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>Písnice</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>č. 760 Písnice (součástí je stavba č.p. 329, čst obce Písnice)</t>
+        </is>
+      </c>
+      <c r="G13" t="n">
+        <v>1</v>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>č. + KU</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="n">
+        <v>58830</v>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>jednotka</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>Hlavní město Praha</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>910/2</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>Písnice</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>jednotka č. 3660007, byt v budově č.p. 361, 362, 363, 364, 365, 366, část obce Písnice, na parcele 910/2 Písnice (*), 910/3 Písnice (*), 910/4 Písnice (*), 910/5 Písnice (*), 910/6 Písnice (*), 910/7 Písnice, podíl na společných částech domu a pozemku 106/10000</t>
+        </is>
+      </c>
+      <c r="G14" t="n">
+        <v>1</v>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>jednotka na parcele bez prefixu st. + KU</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="n">
+        <v>58830</v>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>jednotka</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>Hlavní město Praha</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>910/3</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>Písnice</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>jednotka č. 3660007, byt v budově č.p. 361, 362, 363, 364, 365, 366, část obce Písnice, na parcele 910/2 Písnice (*), 910/3 Písnice (*), 910/4 Písnice (*), 910/5 Písnice (*), 910/6 Písnice (*), 910/7 Písnice, podíl na společných částech domu a pozemku 106/10000</t>
+        </is>
+      </c>
+      <c r="G15" t="n">
+        <v>1</v>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>více parcel oddělených čárkou</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="n">
+        <v>58830</v>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>jednotka</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>Hlavní město Praha</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>910/4</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>Písnice</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>jednotka č. 3660007, byt v budově č.p. 361, 362, 363, 364, 365, 366, část obce Písnice, na parcele 910/2 Písnice (*), 910/3 Písnice (*), 910/4 Písnice (*), 910/5 Písnice (*), 910/6 Písnice (*), 910/7 Písnice, podíl na společných částech domu a pozemku 106/10000</t>
+        </is>
+      </c>
+      <c r="G16" t="n">
+        <v>1</v>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>více parcel oddělených čárkou</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="n">
+        <v>58830</v>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>jednotka</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>Hlavní město Praha</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>910/5</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>Písnice</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>jednotka č. 3660007, byt v budově č.p. 361, 362, 363, 364, 365, 366, část obce Písnice, na parcele 910/2 Písnice (*), 910/3 Písnice (*), 910/4 Písnice (*), 910/5 Písnice (*), 910/6 Písnice (*), 910/7 Písnice, podíl na společných částech domu a pozemku 106/10000</t>
+        </is>
+      </c>
+      <c r="G17" t="n">
+        <v>1</v>
+      </c>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>více parcel oddělených čárkou</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="n">
+        <v>58830</v>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>jednotka</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>Hlavní město Praha</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>910/6</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>Písnice</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>jednotka č. 3660007, byt v budově č.p. 361, 362, 363, 364, 365, 366, část obce Písnice, na parcele 910/2 Písnice (*), 910/3 Písnice (*), 910/4 Písnice (*), 910/5 Písnice (*), 910/6 Písnice (*), 910/7 Písnice, podíl na společných částech domu a pozemku 106/10000</t>
+        </is>
+      </c>
+      <c r="G18" t="n">
+        <v>1</v>
+      </c>
+      <c r="H18" t="inlineStr">
+        <is>
+          <t>více parcel oddělených čárkou</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="n">
+        <v>58830</v>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>jednotka</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>Hlavní město Praha</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>910/7</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>Písnice</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>jednotka č. 3660007, byt v budově č.p. 361, 362, 363, 364, 365, 366, část obce Písnice, na parcele 910/2 Písnice (*), 910/3 Písnice (*), 910/4 Písnice (*), 910/5 Písnice (*), 910/6 Písnice (*), 910/7 Písnice, podíl na společných částech domu a pozemku 106/10000</t>
+        </is>
+      </c>
+      <c r="G19" t="n">
+        <v>1</v>
+      </c>
+      <c r="H19" t="inlineStr">
+        <is>
+          <t>více parcel oddělených čárkou</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="n">
+        <v>58829</v>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>parcela</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>Havlíčkův Brod</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>2197/2</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>Ledeč nad Sázavou</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>č. 2197/2 Ledeč nad Sázavou</t>
+        </is>
+      </c>
+      <c r="G20" t="n">
+        <v>1</v>
+      </c>
+      <c r="H20" t="inlineStr">
+        <is>
+          <t>číslo a KU za ním</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="n">
+        <v>58828</v>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>budova</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>Havlíčkův Brod</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>st. 500</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>Ledeč nad Sázavou</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>stavební č. 500 Ledeč nad Sázavou (součástí je stavba č.p. 117, čst obce Horní Ledeč)</t>
+        </is>
+      </c>
+      <c r="G21" t="n">
+        <v>1</v>
+      </c>
+      <c r="H21" t="inlineStr">
+        <is>
+          <t>č. + KU</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="n">
+        <v>58827</v>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>jednotka</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>Havlíčkův Brod</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>st. 825</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>Ledeč nad Sázavou</t>
+        </is>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>jednotka č. 6450002, byt v budově č.p. 645, 646, část obce Ledeč nad Sázavou, na parcele st. 825 Ledeč nad Sázavou, podíl na společných částech domu a pozemku 237/12278</t>
+        </is>
+      </c>
+      <c r="G22" t="n">
+        <v>1</v>
+      </c>
+      <c r="H22" t="inlineStr">
+        <is>
+          <t>jednotka na parcele s prefixem st. + KU</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="n">
+        <v>58826</v>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>parcela</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>Havlíčkův Brod</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>2090/24</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>Ledeč nad Sázavou</t>
+        </is>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>č. 2090/24 Ledeč nad Sázavou</t>
+        </is>
+      </c>
+      <c r="G23" t="n">
+        <v>1</v>
+      </c>
+      <c r="H23" t="inlineStr">
+        <is>
+          <t>číslo a KU za ním</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="n">
+        <v>58825</v>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>jednotka</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>Havlíčkův Brod</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>st. 614</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>Ledeč nad Sázavou</t>
+        </is>
+      </c>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>jednotka č. 5540005, byt v budově č.p. 553, 554, část obce Ledeč nad Sázavou, na parcele st. 614 Ledeč nad Sázavou, podíl na společných částech domu a pozemku 629/8741</t>
+        </is>
+      </c>
+      <c r="G24" t="n">
+        <v>1</v>
+      </c>
+      <c r="H24" t="inlineStr">
+        <is>
+          <t>jednotka na parcele s prefixem st. + KU</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="n">
+        <v>58824</v>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>jednotka</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>Havlíčkův Brod</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>st. 722</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>Ledeč nad Sázavou</t>
+        </is>
+      </c>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>jednotka č. 6700007, byt v budově č.p. 670, část obce Ledeč nad Sázavou, na parcele st. 722 Ledeč nad Sázavou, podíl na společných částech domu a pozemku 52/1000</t>
+        </is>
+      </c>
+      <c r="G25" t="n">
+        <v>1</v>
+      </c>
+      <c r="H25" t="inlineStr">
+        <is>
+          <t>jednotka na parcele s prefixem st. + KU</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="n">
+        <v>58823</v>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>parcela</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>Havlíčkův Brod</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>823/5</t>
+        </is>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>Ledeč nad Sázavou</t>
+        </is>
+      </c>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>č. 823/5 Ledeč nad Sázavou</t>
+        </is>
+      </c>
+      <c r="G26" t="n">
+        <v>1</v>
+      </c>
+      <c r="H26" t="inlineStr">
+        <is>
+          <t>číslo a KU za ním</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="n">
+        <v>58822</v>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>parcela</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>Havlíčkův Brod</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>823/25</t>
+        </is>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>Ledeč nad Sázavou</t>
+        </is>
+      </c>
+      <c r="F27" t="inlineStr">
+        <is>
+          <t>č. 823/25 Ledeč nad Sázavou</t>
+        </is>
+      </c>
+      <c r="G27" t="n">
+        <v>1</v>
+      </c>
+      <c r="H27" t="inlineStr">
+        <is>
+          <t>číslo a KU za ním</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="n">
+        <v>58821</v>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>parcela</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>Havlíčkův Brod</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>823/32</t>
+        </is>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>Ledeč nad Sázavou</t>
+        </is>
+      </c>
+      <c r="F28" t="inlineStr">
+        <is>
+          <t>č. 823/32 Ledeč nad Sázavou</t>
+        </is>
+      </c>
+      <c r="G28" t="n">
+        <v>1</v>
+      </c>
+      <c r="H28" t="inlineStr">
+        <is>
+          <t>číslo a KU za ním</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="n">
+        <v>58820</v>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>budova</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>Havlíčkův Brod</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>st. 1640</t>
+        </is>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>Ledeč nad Sázavou</t>
+        </is>
+      </c>
+      <c r="F29" t="inlineStr">
+        <is>
+          <t>stavební č. 1640 Ledeč nad Sázavou (součástí je stavba budova bez čp/če, garáž)</t>
+        </is>
+      </c>
+      <c r="G29" t="n">
+        <v>1</v>
+      </c>
+      <c r="H29" t="inlineStr">
+        <is>
+          <t>č. + KU</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="n">
+        <v>58819</v>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>budova</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>Havlíčkův Brod</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>st. 710/2</t>
+        </is>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>Ledeč nad Sázavou</t>
+        </is>
+      </c>
+      <c r="F30" t="inlineStr">
+        <is>
+          <t>stavební č. 710/2 Ledeč nad Sázavou (součástí je stavba budova bez čp/če, jiná stavba)</t>
+        </is>
+      </c>
+      <c r="G30" t="n">
+        <v>1</v>
+      </c>
+      <c r="H30" t="inlineStr">
+        <is>
+          <t>č. + KU</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="n">
+        <v>58818</v>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>budova</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>Havlíčkův Brod</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>st. 710/1</t>
+        </is>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>Ledeč nad Sázavou</t>
+        </is>
+      </c>
+      <c r="F31" t="inlineStr">
+        <is>
+          <t>stavební č. 710/1 Ledeč nad Sázavou (součástí je stavba č.p. 674, čst obce Ledeč nad Sázavou)</t>
+        </is>
+      </c>
+      <c r="G31" t="n">
+        <v>1</v>
+      </c>
+      <c r="H31" t="inlineStr">
+        <is>
+          <t>č. + KU</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="n">
+        <v>58817</v>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>parcela</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>Havlíčkův Brod</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>964</t>
+        </is>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>Ledeč nad Sázavou</t>
+        </is>
+      </c>
+      <c r="F32" t="inlineStr">
+        <is>
+          <t>č. 964 Ledeč nad Sázavou</t>
+        </is>
+      </c>
+      <c r="G32" t="n">
+        <v>1</v>
+      </c>
+      <c r="H32" t="inlineStr">
+        <is>
+          <t>číslo a KU za ním</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="n">
+        <v>58816</v>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>jednotka</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>Havlíčkův Brod</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>st. 601</t>
+        </is>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>Ledeč nad Sázavou</t>
+        </is>
+      </c>
+      <c r="F33" t="inlineStr">
+        <is>
+          <t>jednotka č. 5560004, byt v budově č.p. 557, 555, 556, část obce Ledeč nad Sázavou, na parcele st. 601 Ledeč nad Sázavou, podíl na společných částech domu a pozemku 519/9693</t>
+        </is>
+      </c>
+      <c r="G33" t="n">
+        <v>1</v>
+      </c>
+      <c r="H33" t="inlineStr">
+        <is>
+          <t>jednotka na parcele s prefixem st. + KU</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="n">
+        <v>58815</v>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>jednotka</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>Hlavní město Praha</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>429/48</t>
+        </is>
+      </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>Libuš</t>
+        </is>
+      </c>
+      <c r="F34" t="inlineStr">
+        <is>
+          <t>jednotka č. 9860006, garáž v budově č.p. 986, část obce Libuš, na parcele 429/48 Libuš, podíl na společných částech domu a pozemku 184814/679789</t>
+        </is>
+      </c>
+      <c r="G34" t="n">
+        <v>1</v>
+      </c>
+      <c r="H34" t="inlineStr">
+        <is>
+          <t>jednotka na parcele bez prefixu st. + KU</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="n">
+        <v>58814</v>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>jednotka</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>Hlavní město Praha</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>429/48</t>
+        </is>
+      </c>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>Libuš</t>
+        </is>
+      </c>
+      <c r="F35" t="inlineStr">
+        <is>
+          <t>jednotka č. 9860410, byt v budově č.p. 986, část obce Libuš, na parcele 429/48 Libuš, podíl na společných částech domu a pozemku 5732/679789</t>
+        </is>
+      </c>
+      <c r="G35" t="n">
+        <v>1</v>
+      </c>
+      <c r="H35" t="inlineStr">
+        <is>
+          <t>jednotka na parcele bez prefixu st. + KU</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="n">
+        <v>58813</v>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>parcela</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>Hlavní město Praha</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>1123/116</t>
+        </is>
+      </c>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>Libuš</t>
+        </is>
+      </c>
+      <c r="F36" t="inlineStr">
+        <is>
+          <t>č. 1123/116 Libuš</t>
+        </is>
+      </c>
+      <c r="G36" t="n">
+        <v>1</v>
+      </c>
+      <c r="H36" t="inlineStr">
+        <is>
+          <t>číslo a KU za ním</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="n">
+        <v>58812</v>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>parcela</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>Hlavní město Praha</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>1123/76</t>
+        </is>
+      </c>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>Libuš</t>
+        </is>
+      </c>
+      <c r="F37" t="inlineStr">
+        <is>
+          <t>č. 1123/76 Libuš</t>
+        </is>
+      </c>
+      <c r="G37" t="n">
+        <v>1</v>
+      </c>
+      <c r="H37" t="inlineStr">
+        <is>
+          <t>číslo a KU za ním</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="n">
+        <v>58811</v>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>parcela</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>Hlavní město Praha</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>1123/73</t>
+        </is>
+      </c>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>Libuš</t>
+        </is>
+      </c>
+      <c r="F38" t="inlineStr">
+        <is>
+          <t>č. 1123/73 Libuš</t>
+        </is>
+      </c>
+      <c r="G38" t="n">
+        <v>1</v>
+      </c>
+      <c r="H38" t="inlineStr">
+        <is>
+          <t>číslo a KU za ním</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="n">
+        <v>58810</v>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>parcela</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>Hlavní město Praha</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>1123/120</t>
+        </is>
+      </c>
+      <c r="E39" t="inlineStr">
+        <is>
+          <t>Libuš</t>
+        </is>
+      </c>
+      <c r="F39" t="inlineStr">
+        <is>
+          <t>č. 1123/120 Libuš</t>
+        </is>
+      </c>
+      <c r="G39" t="n">
+        <v>1</v>
+      </c>
+      <c r="H39" t="inlineStr">
+        <is>
+          <t>číslo a KU za ním</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="n">
+        <v>58809</v>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>parcela</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>Hlavní město Praha</t>
+        </is>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>1123/118</t>
+        </is>
+      </c>
+      <c r="E40" t="inlineStr">
+        <is>
+          <t>Libuš</t>
+        </is>
+      </c>
+      <c r="F40" t="inlineStr">
+        <is>
+          <t>č. 1123/118 Libuš</t>
+        </is>
+      </c>
+      <c r="G40" t="n">
+        <v>1</v>
+      </c>
+      <c r="H40" t="inlineStr">
+        <is>
+          <t>číslo a KU za ním</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="n">
+        <v>58808</v>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>parcela</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>Hlavní město Praha</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>1123/119</t>
+        </is>
+      </c>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>Libuš</t>
+        </is>
+      </c>
+      <c r="F41" t="inlineStr">
+        <is>
+          <t>č. 1123/119 Libuš</t>
+        </is>
+      </c>
+      <c r="G41" t="n">
+        <v>1</v>
+      </c>
+      <c r="H41" t="inlineStr">
+        <is>
+          <t>číslo a KU za ním</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="n">
+        <v>58807</v>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>parcela</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>Hlavní město Praha</t>
+        </is>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>1123/117</t>
+        </is>
+      </c>
+      <c r="E42" t="inlineStr">
+        <is>
+          <t>Libuš</t>
+        </is>
+      </c>
+      <c r="F42" t="inlineStr">
+        <is>
+          <t>č. 1123/117 Libuš</t>
+        </is>
+      </c>
+      <c r="G42" t="n">
+        <v>1</v>
+      </c>
+      <c r="H42" t="inlineStr">
+        <is>
+          <t>číslo a KU za ním</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="n">
+        <v>58806</v>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>parcela</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>Hlavní město Praha</t>
+        </is>
+      </c>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>2382/8</t>
+        </is>
+      </c>
+      <c r="E43" t="inlineStr">
+        <is>
+          <t>Kunratice</t>
+        </is>
+      </c>
+      <c r="F43" t="inlineStr">
+        <is>
+          <t>č. 2382/8 Kunratice</t>
+        </is>
+      </c>
+      <c r="G43" t="n">
+        <v>1</v>
+      </c>
+      <c r="H43" t="inlineStr">
+        <is>
+          <t>číslo a KU za ním</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="n">
+        <v>58805</v>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>parcela</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>Hlavní město Praha</t>
+        </is>
+      </c>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t>2342/27</t>
+        </is>
+      </c>
+      <c r="E44" t="inlineStr">
+        <is>
+          <t>Kunratice</t>
+        </is>
+      </c>
+      <c r="F44" t="inlineStr">
+        <is>
+          <t>č. 2342/27 Kunratice</t>
+        </is>
+      </c>
+      <c r="G44" t="n">
+        <v>1</v>
+      </c>
+      <c r="H44" t="inlineStr">
+        <is>
+          <t>číslo a KU za ním</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="n">
+        <v>58804</v>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>parcela</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>Hlavní město Praha</t>
+        </is>
+      </c>
+      <c r="D45" t="inlineStr">
+        <is>
+          <t>2342/30</t>
+        </is>
+      </c>
+      <c r="E45" t="inlineStr">
+        <is>
+          <t>Kunratice</t>
+        </is>
+      </c>
+      <c r="F45" t="inlineStr">
+        <is>
+          <t>č. 2342/30 Kunratice</t>
+        </is>
+      </c>
+      <c r="G45" t="n">
+        <v>1</v>
+      </c>
+      <c r="H45" t="inlineStr">
+        <is>
+          <t>číslo a KU za ním</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="n">
+        <v>58803</v>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>parcela</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>Hlavní město Praha</t>
+        </is>
+      </c>
+      <c r="D46" t="inlineStr">
+        <is>
+          <t>2342/28</t>
+        </is>
+      </c>
+      <c r="E46" t="inlineStr">
+        <is>
+          <t>Kunratice</t>
+        </is>
+      </c>
+      <c r="F46" t="inlineStr">
+        <is>
+          <t>č. 2342/28 Kunratice</t>
+        </is>
+      </c>
+      <c r="G46" t="n">
+        <v>1</v>
+      </c>
+      <c r="H46" t="inlineStr">
+        <is>
+          <t>číslo a KU za ním</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="n">
+        <v>58802</v>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>parcela</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>Hlavní město Praha</t>
+        </is>
+      </c>
+      <c r="D47" t="inlineStr">
+        <is>
+          <t>2342/29</t>
+        </is>
+      </c>
+      <c r="E47" t="inlineStr">
+        <is>
+          <t>Kunratice</t>
+        </is>
+      </c>
+      <c r="F47" t="inlineStr">
+        <is>
+          <t>č. 2342/29 Kunratice</t>
+        </is>
+      </c>
+      <c r="G47" t="n">
+        <v>1</v>
+      </c>
+      <c r="H47" t="inlineStr">
+        <is>
+          <t>číslo a KU za ním</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="n">
+        <v>58801</v>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>budova</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>Hlavní město Praha</t>
+        </is>
+      </c>
+      <c r="D48" t="inlineStr">
+        <is>
+          <t>2342/31</t>
+        </is>
+      </c>
+      <c r="E48" t="inlineStr">
+        <is>
+          <t>Kunratice</t>
+        </is>
+      </c>
+      <c r="F48" t="inlineStr">
+        <is>
+          <t>č. 2342/31 Kunratice</t>
+        </is>
+      </c>
+      <c r="G48" t="n">
+        <v>1</v>
+      </c>
+      <c r="H48" t="inlineStr">
+        <is>
+          <t>č. + KU</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="n">
+        <v>58800</v>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>jednotka</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>Hlavní město Praha</t>
+        </is>
+      </c>
+      <c r="D49" t="inlineStr">
+        <is>
+          <t>2342/27</t>
+        </is>
+      </c>
+      <c r="E49" t="inlineStr">
+        <is>
+          <t>Kunratice</t>
+        </is>
+      </c>
+      <c r="F49" t="inlineStr">
+        <is>
+          <t>jednotka č. 11500902, garáž v budově č.p. 1152, 1148, 1149, 1150, 1151, část obce Kunratice, na parcele 2342/27 Kunratice, 2342/28 Kunratice, 2342/29 Kunratice, 2342/30 Kunratice, 2342/31 Kunratice, podíl na společných částech domu a pozemku 17/7754</t>
+        </is>
+      </c>
+      <c r="G49" t="n">
+        <v>1</v>
+      </c>
+      <c r="H49" t="inlineStr">
+        <is>
+          <t>jednotka na parcele bez prefixu st. + KU</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="n">
+        <v>58800</v>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>jednotka</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>Hlavní město Praha</t>
+        </is>
+      </c>
+      <c r="D50" t="inlineStr">
+        <is>
+          <t>2342/28</t>
+        </is>
+      </c>
+      <c r="E50" t="inlineStr">
+        <is>
+          <t>Kunratice</t>
+        </is>
+      </c>
+      <c r="F50" t="inlineStr">
+        <is>
+          <t>jednotka č. 11500902, garáž v budově č.p. 1152, 1148, 1149, 1150, 1151, část obce Kunratice, na parcele 2342/27 Kunratice, 2342/28 Kunratice, 2342/29 Kunratice, 2342/30 Kunratice, 2342/31 Kunratice, podíl na společných částech domu a pozemku 17/7754</t>
+        </is>
+      </c>
+      <c r="G50" t="n">
+        <v>1</v>
+      </c>
+      <c r="H50" t="inlineStr">
+        <is>
+          <t>více parcel oddělených čárkou</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="n">
+        <v>58800</v>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>jednotka</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>Hlavní město Praha</t>
+        </is>
+      </c>
+      <c r="D51" t="inlineStr">
+        <is>
+          <t>2342/29</t>
+        </is>
+      </c>
+      <c r="E51" t="inlineStr">
+        <is>
+          <t>Kunratice</t>
+        </is>
+      </c>
+      <c r="F51" t="inlineStr">
+        <is>
+          <t>jednotka č. 11500902, garáž v budově č.p. 1152, 1148, 1149, 1150, 1151, část obce Kunratice, na parcele 2342/27 Kunratice, 2342/28 Kunratice, 2342/29 Kunratice, 2342/30 Kunratice, 2342/31 Kunratice, podíl na společných částech domu a pozemku 17/7754</t>
+        </is>
+      </c>
+      <c r="G51" t="n">
+        <v>1</v>
+      </c>
+      <c r="H51" t="inlineStr">
+        <is>
+          <t>více parcel oddělených čárkou</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="n">
+        <v>58800</v>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>jednotka</t>
+        </is>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>Hlavní město Praha</t>
+        </is>
+      </c>
+      <c r="D52" t="inlineStr">
+        <is>
+          <t>2342/30</t>
+        </is>
+      </c>
+      <c r="E52" t="inlineStr">
+        <is>
+          <t>Kunratice</t>
+        </is>
+      </c>
+      <c r="F52" t="inlineStr">
+        <is>
+          <t>jednotka č. 11500902, garáž v budově č.p. 1152, 1148, 1149, 1150, 1151, část obce Kunratice, na parcele 2342/27 Kunratice, 2342/28 Kunratice, 2342/29 Kunratice, 2342/30 Kunratice, 2342/31 Kunratice, podíl na společných částech domu a pozemku 17/7754</t>
+        </is>
+      </c>
+      <c r="G52" t="n">
+        <v>1</v>
+      </c>
+      <c r="H52" t="inlineStr">
+        <is>
+          <t>více parcel oddělených čárkou</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="n">
+        <v>58800</v>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>jednotka</t>
+        </is>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>Hlavní město Praha</t>
+        </is>
+      </c>
+      <c r="D53" t="inlineStr">
+        <is>
+          <t>2342/31</t>
+        </is>
+      </c>
+      <c r="E53" t="inlineStr">
+        <is>
+          <t>Kunratice</t>
+        </is>
+      </c>
+      <c r="F53" t="inlineStr">
+        <is>
+          <t>jednotka č. 11500902, garáž v budově č.p. 1152, 1148, 1149, 1150, 1151, část obce Kunratice, na parcele 2342/27 Kunratice, 2342/28 Kunratice, 2342/29 Kunratice, 2342/30 Kunratice, 2342/31 Kunratice, podíl na společných částech domu a pozemku 17/7754</t>
+        </is>
+      </c>
+      <c r="G53" t="n">
+        <v>1</v>
+      </c>
+      <c r="H53" t="inlineStr">
+        <is>
+          <t>více parcel oddělených čárkou</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="n">
+        <v>58799</v>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>jednotka</t>
+        </is>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>Hlavní město Praha</t>
+        </is>
+      </c>
+      <c r="D54" t="inlineStr">
+        <is>
+          <t>2342/27</t>
+        </is>
+      </c>
+      <c r="E54" t="inlineStr">
+        <is>
+          <t>Kunratice</t>
+        </is>
+      </c>
+      <c r="F54" t="inlineStr">
+        <is>
+          <t>jednotka č. 11500061, byt v budově č.p. 1152, 1148, 1149, 1150, 1151, část obce Kunratice, na parcele 2342/27 Kunratice, 2342/28 Kunratice, 2342/29 Kunratice, 2342/30 Kunratice, 2342/31 Kunratice, podíl na společných částech domu a pozemku 82/7754</t>
+        </is>
+      </c>
+      <c r="G54" t="n">
+        <v>1</v>
+      </c>
+      <c r="H54" t="inlineStr">
+        <is>
+          <t>jednotka na parcele bez prefixu st. + KU</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="n">
+        <v>58799</v>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>jednotka</t>
+        </is>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>Hlavní město Praha</t>
+        </is>
+      </c>
+      <c r="D55" t="inlineStr">
+        <is>
+          <t>2342/28</t>
+        </is>
+      </c>
+      <c r="E55" t="inlineStr">
+        <is>
+          <t>Kunratice</t>
+        </is>
+      </c>
+      <c r="F55" t="inlineStr">
+        <is>
+          <t>jednotka č. 11500061, byt v budově č.p. 1152, 1148, 1149, 1150, 1151, část obce Kunratice, na parcele 2342/27 Kunratice, 2342/28 Kunratice, 2342/29 Kunratice, 2342/30 Kunratice, 2342/31 Kunratice, podíl na společných částech domu a pozemku 82/7754</t>
+        </is>
+      </c>
+      <c r="G55" t="n">
+        <v>1</v>
+      </c>
+      <c r="H55" t="inlineStr">
+        <is>
+          <t>více parcel oddělených čárkou</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="n">
+        <v>58799</v>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>jednotka</t>
+        </is>
+      </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>Hlavní město Praha</t>
+        </is>
+      </c>
+      <c r="D56" t="inlineStr">
+        <is>
+          <t>2342/29</t>
+        </is>
+      </c>
+      <c r="E56" t="inlineStr">
+        <is>
+          <t>Kunratice</t>
+        </is>
+      </c>
+      <c r="F56" t="inlineStr">
+        <is>
+          <t>jednotka č. 11500061, byt v budově č.p. 1152, 1148, 1149, 1150, 1151, část obce Kunratice, na parcele 2342/27 Kunratice, 2342/28 Kunratice, 2342/29 Kunratice, 2342/30 Kunratice, 2342/31 Kunratice, podíl na společných částech domu a pozemku 82/7754</t>
+        </is>
+      </c>
+      <c r="G56" t="n">
+        <v>1</v>
+      </c>
+      <c r="H56" t="inlineStr">
+        <is>
+          <t>více parcel oddělených čárkou</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="n">
+        <v>58799</v>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>jednotka</t>
+        </is>
+      </c>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>Hlavní město Praha</t>
+        </is>
+      </c>
+      <c r="D57" t="inlineStr">
+        <is>
+          <t>2342/30</t>
+        </is>
+      </c>
+      <c r="E57" t="inlineStr">
+        <is>
+          <t>Kunratice</t>
+        </is>
+      </c>
+      <c r="F57" t="inlineStr">
+        <is>
+          <t>jednotka č. 11500061, byt v budově č.p. 1152, 1148, 1149, 1150, 1151, část obce Kunratice, na parcele 2342/27 Kunratice, 2342/28 Kunratice, 2342/29 Kunratice, 2342/30 Kunratice, 2342/31 Kunratice, podíl na společných částech domu a pozemku 82/7754</t>
+        </is>
+      </c>
+      <c r="G57" t="n">
+        <v>1</v>
+      </c>
+      <c r="H57" t="inlineStr">
+        <is>
+          <t>více parcel oddělených čárkou</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="n">
+        <v>58799</v>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>jednotka</t>
+        </is>
+      </c>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>Hlavní město Praha</t>
+        </is>
+      </c>
+      <c r="D58" t="inlineStr">
+        <is>
+          <t>2342/31</t>
+        </is>
+      </c>
+      <c r="E58" t="inlineStr">
+        <is>
+          <t>Kunratice</t>
+        </is>
+      </c>
+      <c r="F58" t="inlineStr">
+        <is>
+          <t>jednotka č. 11500061, byt v budově č.p. 1152, 1148, 1149, 1150, 1151, část obce Kunratice, na parcele 2342/27 Kunratice, 2342/28 Kunratice, 2342/29 Kunratice, 2342/30 Kunratice, 2342/31 Kunratice, podíl na společných částech domu a pozemku 82/7754</t>
+        </is>
+      </c>
+      <c r="G58" t="n">
+        <v>1</v>
+      </c>
+      <c r="H58" t="inlineStr">
+        <is>
+          <t>více parcel oddělených čárkou</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="n">
+        <v>58798</v>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>parcela</t>
+        </is>
+      </c>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>Hlavní město Praha</t>
+        </is>
+      </c>
+      <c r="D59" t="inlineStr">
+        <is>
+          <t>1433/13</t>
+        </is>
+      </c>
+      <c r="E59" t="inlineStr">
+        <is>
+          <t>Kunratice</t>
+        </is>
+      </c>
+      <c r="F59" t="inlineStr">
+        <is>
+          <t>č. 1433/13 Kunratice</t>
+        </is>
+      </c>
+      <c r="G59" t="n">
+        <v>1</v>
+      </c>
+      <c r="H59" t="inlineStr">
+        <is>
+          <t>číslo a KU za ním</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="n">
+        <v>58797</v>
+      </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>parcela</t>
+        </is>
+      </c>
+      <c r="C60" t="inlineStr">
+        <is>
+          <t>Hlavní město Praha</t>
+        </is>
+      </c>
+      <c r="D60" t="inlineStr">
+        <is>
+          <t>1433/12</t>
+        </is>
+      </c>
+      <c r="E60" t="inlineStr">
+        <is>
+          <t>Kunratice</t>
+        </is>
+      </c>
+      <c r="F60" t="inlineStr">
+        <is>
+          <t>č. 1433/12 Kunratice</t>
+        </is>
+      </c>
+      <c r="G60" t="n">
+        <v>1</v>
+      </c>
+      <c r="H60" t="inlineStr">
+        <is>
+          <t>číslo a KU za ním</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="n">
+        <v>58796</v>
+      </c>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>parcela</t>
+        </is>
+      </c>
+      <c r="C61" t="inlineStr">
+        <is>
+          <t>Hlavní město Praha</t>
+        </is>
+      </c>
+      <c r="D61" t="inlineStr">
+        <is>
+          <t>59/12</t>
+        </is>
+      </c>
+      <c r="E61" t="inlineStr">
+        <is>
+          <t>Kunratice</t>
+        </is>
+      </c>
+      <c r="F61" t="inlineStr">
+        <is>
+          <t>č. 59/12 Kunratice</t>
+        </is>
+      </c>
+      <c r="G61" t="n">
+        <v>1</v>
+      </c>
+      <c r="H61" t="inlineStr">
+        <is>
+          <t>číslo a KU za ním</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="n">
+        <v>58795</v>
+      </c>
+      <c r="B62" t="inlineStr">
+        <is>
+          <t>budova</t>
+        </is>
+      </c>
+      <c r="C62" t="inlineStr">
+        <is>
+          <t>Hlavní město Praha</t>
+        </is>
+      </c>
+      <c r="D62" t="inlineStr">
+        <is>
+          <t>59/45</t>
+        </is>
+      </c>
+      <c r="E62" t="inlineStr">
+        <is>
+          <t>Kunratice</t>
+        </is>
+      </c>
+      <c r="F62" t="inlineStr">
+        <is>
+          <t>č. 59/45 Kunratice (součástí je stavba č.p. 1045, čst obce Kunratice)</t>
+        </is>
+      </c>
+      <c r="G62" t="n">
+        <v>1</v>
+      </c>
+      <c r="H62" t="inlineStr">
+        <is>
+          <t>č. + KU</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="n">
+        <v>58794</v>
+      </c>
+      <c r="B63" t="inlineStr">
+        <is>
+          <t>budova</t>
+        </is>
+      </c>
+      <c r="C63" t="inlineStr">
+        <is>
+          <t>Hlavní město Praha</t>
+        </is>
+      </c>
+      <c r="D63" t="inlineStr">
+        <is>
+          <t>267/9</t>
+        </is>
+      </c>
+      <c r="E63" t="inlineStr">
+        <is>
+          <t>Kunratice</t>
+        </is>
+      </c>
+      <c r="F63" t="inlineStr">
+        <is>
+          <t>budova bez čp/če, jiná stavba, na parcele 267/9 Kunratice</t>
+        </is>
+      </c>
+      <c r="G63" t="n">
+        <v>1</v>
+      </c>
+      <c r="H63" t="inlineStr">
+        <is>
+          <t>budova na parcele č.</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="n">
+        <v>58793</v>
+      </c>
+      <c r="B64" t="inlineStr">
+        <is>
+          <t>parcela</t>
+        </is>
+      </c>
+      <c r="C64" t="inlineStr">
+        <is>
+          <t>Hlavní město Praha</t>
+        </is>
+      </c>
+      <c r="D64" t="inlineStr">
+        <is>
+          <t>2428/21</t>
+        </is>
+      </c>
+      <c r="E64" t="inlineStr">
+        <is>
+          <t>Kunratice</t>
+        </is>
+      </c>
+      <c r="F64" t="inlineStr">
+        <is>
+          <t>č. 2428/21 Kunratice</t>
+        </is>
+      </c>
+      <c r="G64" t="n">
+        <v>1</v>
+      </c>
+      <c r="H64" t="inlineStr">
         <is>
           <t>číslo a KU za ním</t>
         </is>

</xml_diff>

<commit_message>
Uprava vykreslovani do mapy, p[ridan tooltip
</commit_message>
<xml_diff>
--- a/GIS2/vystup.xlsx
+++ b/GIS2/vystup.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H64"/>
+  <dimension ref="A1:H51"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -472,31 +472,31 @@
     </row>
     <row r="2">
       <c r="A2" t="n">
-        <v>58842</v>
+        <v>47800</v>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>parcela</t>
+          <t>jednotka</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Hlavní město Praha</t>
+          <t>Praha-východ</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>1044/2</t>
+          <t>st. 646</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>Libuš</t>
+          <t>Ládví</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>č. 1044/2 Libuš</t>
+          <t>jednotka č. 4680004, byt v budově č.p. 468, 467, 469, část obce Olešovice, na parcele st. 646 Ládví, podíl na společných částech domu a pozemku 7596/110533</t>
         </is>
       </c>
       <c r="G2" t="n">
@@ -504,37 +504,37 @@
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>číslo a KU za ním</t>
+          <t>jednotka na parcele s prefixem st. + KU</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="n">
-        <v>58841</v>
+        <v>47799</v>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>budova</t>
+          <t>parcela</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Hlavní město Praha</t>
+          <t>Praha-východ</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>1044/4</t>
+          <t>748/43</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>Libuš</t>
+          <t>Ládví</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>č. 1044/4 Libuš (součástí je stavba č.p. 957, čst obce Libuš)</t>
+          <t>č. 748/43 Ládví</t>
         </is>
       </c>
       <c r="G3" t="n">
@@ -542,37 +542,37 @@
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>č. + KU</t>
+          <t>číslo a KU za ním</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="n">
-        <v>58840</v>
+        <v>47798</v>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>parcela</t>
+          <t>budova</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Hlavní město Praha</t>
+          <t>Praha-východ</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>1087/2</t>
+          <t>st. 334</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>Libuš</t>
+          <t>Ládví</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>č. 1087/2 Libuš</t>
+          <t>stavební č. 334 Ládví (součástí je stavba č.p. 154, čst obce Ládví)</t>
         </is>
       </c>
       <c r="G4" t="n">
@@ -580,13 +580,13 @@
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>číslo a KU za ním</t>
+          <t>č. + KU</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="n">
-        <v>58839</v>
+        <v>47797</v>
       </c>
       <c r="B5" t="inlineStr">
         <is>
@@ -595,22 +595,22 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Hlavní město Praha</t>
+          <t>Praha-východ</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>1088</t>
+          <t>125/12</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>Libuš</t>
+          <t>Ládví</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>č. 1088 Libuš</t>
+          <t>č. 125/12 Ládví</t>
         </is>
       </c>
       <c r="G5" t="n">
@@ -624,7 +624,7 @@
     </row>
     <row r="6">
       <c r="A6" t="n">
-        <v>58838</v>
+        <v>47796</v>
       </c>
       <c r="B6" t="inlineStr">
         <is>
@@ -633,22 +633,22 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Hlavní město Praha</t>
+          <t>Praha-východ</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>1087/1</t>
+          <t>st. 1372</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>Libuš</t>
+          <t>Ládví</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>č. 1087/1 Libuš (součástí je stavba č.p. 435, čst obce Libuš)</t>
+          <t>stavební č. 1372 Ládví (součástí je stavba budova bez čp/če, jiná stavba)</t>
         </is>
       </c>
       <c r="G6" t="n">
@@ -662,31 +662,31 @@
     </row>
     <row r="7">
       <c r="A7" t="n">
-        <v>58837</v>
+        <v>47795</v>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>parcela</t>
+          <t>budova</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Hlavní město Praha</t>
+          <t>Praha-východ</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>546/1</t>
+          <t>st. 514</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>Libuš</t>
+          <t>Ládví</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>č. 546/1 Libuš</t>
+          <t>stavební č. 514 Ládví (součástí je stavba č.e. 1347, čst obce Ládví)</t>
         </is>
       </c>
       <c r="G7" t="n">
@@ -694,13 +694,13 @@
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>číslo a KU za ním</t>
+          <t>č. + KU</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="n">
-        <v>58836</v>
+        <v>47794</v>
       </c>
       <c r="B8" t="inlineStr">
         <is>
@@ -709,22 +709,22 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Hlavní město Praha</t>
+          <t>Praha-východ</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>546/3</t>
+          <t>255/8</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>Libuš</t>
+          <t>Ládví</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>č. 546/3 Libuš</t>
+          <t>č. 255/8 Ládví</t>
         </is>
       </c>
       <c r="G8" t="n">
@@ -738,31 +738,31 @@
     </row>
     <row r="9">
       <c r="A9" t="n">
-        <v>58835</v>
+        <v>47793</v>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>budova</t>
+          <t>parcela</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Hlavní město Praha</t>
+          <t>Praha-východ</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>546/2</t>
+          <t>722/12</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>Libuš</t>
+          <t>Ládví</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>č. 546/2 Libuš (součástí je stavba budova bez čp/če, jiná stavba)</t>
+          <t>č. 722/12 Ládví</t>
         </is>
       </c>
       <c r="G9" t="n">
@@ -770,37 +770,37 @@
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>č. + KU</t>
+          <t>číslo a KU za ním</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="n">
-        <v>58834</v>
+        <v>47792</v>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>budova</t>
+          <t>parcela</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Hlavní město Praha</t>
+          <t>Praha-východ</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>546/4</t>
+          <t>234/4</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>Libuš</t>
+          <t>Ládví</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>č. 546/4 Libuš (součástí je stavba budova bez čp/če, jiná stavba)</t>
+          <t>č. 234/4 Ládví</t>
         </is>
       </c>
       <c r="G10" t="n">
@@ -808,13 +808,13 @@
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>č. + KU</t>
+          <t>číslo a KU za ním</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="n">
-        <v>58833</v>
+        <v>47791</v>
       </c>
       <c r="B11" t="inlineStr">
         <is>
@@ -823,22 +823,22 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Hlavní město Praha</t>
+          <t>Praha-východ</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>835/84</t>
+          <t>646/32</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>Písnice</t>
+          <t>Ládví</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>č. 835/84 Písnice</t>
+          <t>č. 646/32 Ládví</t>
         </is>
       </c>
       <c r="G11" t="n">
@@ -852,31 +852,31 @@
     </row>
     <row r="12">
       <c r="A12" t="n">
-        <v>58832</v>
+        <v>47790</v>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>parcela</t>
+          <t>budova</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Hlavní město Praha</t>
+          <t>Praha-východ</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>761</t>
+          <t>st. 877</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>Písnice</t>
+          <t>Ládví</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>č. 761 Písnice</t>
+          <t>stavební č. 877 Ládví (součástí je stavba č.p. 1425, čst obce Olešovice)</t>
         </is>
       </c>
       <c r="G12" t="n">
@@ -884,37 +884,37 @@
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>číslo a KU za ním</t>
+          <t>č. + KU</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="n">
-        <v>58831</v>
+        <v>47789</v>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>budova</t>
+          <t>parcela</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Hlavní město Praha</t>
+          <t>Praha-východ</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>760</t>
+          <t>628/4</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>Písnice</t>
+          <t>Ládví</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>č. 760 Písnice (součástí je stavba č.p. 329, čst obce Písnice)</t>
+          <t>č. 628/4 Ládví</t>
         </is>
       </c>
       <c r="G13" t="n">
@@ -922,37 +922,37 @@
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>č. + KU</t>
+          <t>číslo a KU za ním</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="n">
-        <v>58830</v>
+        <v>47788</v>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>jednotka</t>
+          <t>parcela</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Hlavní město Praha</t>
+          <t>Praha-východ</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>910/2</t>
+          <t>628/33</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>Písnice</t>
+          <t>Ládví</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>jednotka č. 3660007, byt v budově č.p. 361, 362, 363, 364, 365, 366, část obce Písnice, na parcele 910/2 Písnice (*), 910/3 Písnice (*), 910/4 Písnice (*), 910/5 Písnice (*), 910/6 Písnice (*), 910/7 Písnice, podíl na společných částech domu a pozemku 106/10000</t>
+          <t>č. 628/33 Ládví</t>
         </is>
       </c>
       <c r="G14" t="n">
@@ -960,13 +960,13 @@
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>jednotka na parcele bez prefixu st. + KU</t>
+          <t>číslo a KU za ním</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="n">
-        <v>58830</v>
+        <v>47787</v>
       </c>
       <c r="B15" t="inlineStr">
         <is>
@@ -975,22 +975,22 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Hlavní město Praha</t>
+          <t>Praha-východ</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>910/3</t>
+          <t>st. 1313</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>Písnice</t>
+          <t>Ládví</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>jednotka č. 3660007, byt v budově č.p. 361, 362, 363, 364, 365, 366, část obce Písnice, na parcele 910/2 Písnice (*), 910/3 Písnice (*), 910/4 Písnice (*), 910/5 Písnice (*), 910/6 Písnice (*), 910/7 Písnice, podíl na společných částech domu a pozemku 106/10000</t>
+          <t>jednotka č. 24010022, byt v budově č.p. 2401, část obce Olešovice, na parcele st. 1313 Ládví (součástí je stavba č.p. 2401, čst obce Olešovice), podíl na společných částech domu a pozemku 458/4518</t>
         </is>
       </c>
       <c r="G15" t="n">
@@ -998,37 +998,37 @@
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>více parcel oddělených čárkou</t>
+          <t>jednotka na parcele s prefixem st. + KU</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="n">
-        <v>58830</v>
+        <v>47786</v>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>jednotka</t>
+          <t>parcela</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Hlavní město Praha</t>
+          <t>Praha-východ</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>910/4</t>
+          <t>634/4</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>Písnice</t>
+          <t>Ládví</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>jednotka č. 3660007, byt v budově č.p. 361, 362, 363, 364, 365, 366, část obce Písnice, na parcele 910/2 Písnice (*), 910/3 Písnice (*), 910/4 Písnice (*), 910/5 Písnice (*), 910/6 Písnice (*), 910/7 Písnice, podíl na společných částech domu a pozemku 106/10000</t>
+          <t>č. 634/4 Ládví</t>
         </is>
       </c>
       <c r="G16" t="n">
@@ -1036,37 +1036,37 @@
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>více parcel oddělených čárkou</t>
+          <t>číslo a KU za ním</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="n">
-        <v>58830</v>
+        <v>47785</v>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>jednotka</t>
+          <t>parcela</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Hlavní město Praha</t>
+          <t>Praha-východ</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>910/5</t>
+          <t>634/5</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>Písnice</t>
+          <t>Ládví</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>jednotka č. 3660007, byt v budově č.p. 361, 362, 363, 364, 365, 366, část obce Písnice, na parcele 910/2 Písnice (*), 910/3 Písnice (*), 910/4 Písnice (*), 910/5 Písnice (*), 910/6 Písnice (*), 910/7 Písnice, podíl na společných částech domu a pozemku 106/10000</t>
+          <t>č. 634/5 Ládví</t>
         </is>
       </c>
       <c r="G17" t="n">
@@ -1074,37 +1074,37 @@
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>více parcel oddělených čárkou</t>
+          <t>číslo a KU za ním</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="n">
-        <v>58830</v>
+        <v>47784</v>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>jednotka</t>
+          <t>parcela</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Hlavní město Praha</t>
+          <t>Praha-východ</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>910/6</t>
+          <t>328/91</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>Písnice</t>
+          <t>Ládví</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>jednotka č. 3660007, byt v budově č.p. 361, 362, 363, 364, 365, 366, část obce Písnice, na parcele 910/2 Písnice (*), 910/3 Písnice (*), 910/4 Písnice (*), 910/5 Písnice (*), 910/6 Písnice (*), 910/7 Písnice, podíl na společných částech domu a pozemku 106/10000</t>
+          <t>č. 328/91 Ládví</t>
         </is>
       </c>
       <c r="G18" t="n">
@@ -1112,37 +1112,37 @@
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>více parcel oddělených čárkou</t>
+          <t>číslo a KU za ním</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="n">
-        <v>58830</v>
+        <v>47783</v>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>jednotka</t>
+          <t>parcela</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>Hlavní město Praha</t>
+          <t>Praha-východ</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>910/7</t>
+          <t>328/143</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>Písnice</t>
+          <t>Ládví</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>jednotka č. 3660007, byt v budově č.p. 361, 362, 363, 364, 365, 366, část obce Písnice, na parcele 910/2 Písnice (*), 910/3 Písnice (*), 910/4 Písnice (*), 910/5 Písnice (*), 910/6 Písnice (*), 910/7 Písnice, podíl na společných částech domu a pozemku 106/10000</t>
+          <t>č. 328/143 Ládví</t>
         </is>
       </c>
       <c r="G19" t="n">
@@ -1150,13 +1150,13 @@
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>více parcel oddělených čárkou</t>
+          <t>číslo a KU za ním</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="n">
-        <v>58829</v>
+        <v>47782</v>
       </c>
       <c r="B20" t="inlineStr">
         <is>
@@ -1165,22 +1165,22 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>Havlíčkův Brod</t>
+          <t>Praha-východ</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>2197/2</t>
+          <t>414/49</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>Ledeč nad Sázavou</t>
+          <t>Ládví</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>č. 2197/2 Ledeč nad Sázavou</t>
+          <t>č. 414/49 Ládví</t>
         </is>
       </c>
       <c r="G20" t="n">
@@ -1194,31 +1194,31 @@
     </row>
     <row r="21">
       <c r="A21" t="n">
-        <v>58828</v>
+        <v>47781</v>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>budova</t>
+          <t>parcela</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>Havlíčkův Brod</t>
+          <t>Praha-východ</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>st. 500</t>
+          <t>414/48</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>Ledeč nad Sázavou</t>
+          <t>Ládví</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>stavební č. 500 Ledeč nad Sázavou (součástí je stavba č.p. 117, čst obce Horní Ledeč)</t>
+          <t>č. 414/48 Ládví</t>
         </is>
       </c>
       <c r="G21" t="n">
@@ -1226,37 +1226,37 @@
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>č. + KU</t>
+          <t>číslo a KU za ním</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="n">
-        <v>58827</v>
+        <v>47780</v>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>jednotka</t>
+          <t>budova</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>Havlíčkův Brod</t>
+          <t>Praha-východ</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>st. 825</t>
+          <t>st. 1294</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>Ledeč nad Sázavou</t>
+          <t>Ládví</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>jednotka č. 6450002, byt v budově č.p. 645, 646, část obce Ledeč nad Sázavou, na parcele st. 825 Ledeč nad Sázavou, podíl na společných částech domu a pozemku 237/12278</t>
+          <t>stavební č. 1294 Ládví (součástí je stavba budova bez čp/če, garáž)</t>
         </is>
       </c>
       <c r="G22" t="n">
@@ -1264,13 +1264,13 @@
       </c>
       <c r="H22" t="inlineStr">
         <is>
-          <t>jednotka na parcele s prefixem st. + KU</t>
+          <t>č. + KU</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="n">
-        <v>58826</v>
+        <v>47779</v>
       </c>
       <c r="B23" t="inlineStr">
         <is>
@@ -1279,22 +1279,22 @@
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>Havlíčkův Brod</t>
+          <t>Praha-východ</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>2090/24</t>
+          <t>95/15</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>Ledeč nad Sázavou</t>
+          <t>Ládví</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>č. 2090/24 Ledeč nad Sázavou</t>
+          <t>č. 95/15 Ládví</t>
         </is>
       </c>
       <c r="G23" t="n">
@@ -1308,31 +1308,31 @@
     </row>
     <row r="24">
       <c r="A24" t="n">
-        <v>58825</v>
+        <v>47778</v>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>jednotka</t>
+          <t>parcela</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>Havlíčkův Brod</t>
+          <t>Praha-východ</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>st. 614</t>
+          <t>96/5</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>Ledeč nad Sázavou</t>
+          <t>Ládví</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>jednotka č. 5540005, byt v budově č.p. 553, 554, část obce Ledeč nad Sázavou, na parcele st. 614 Ledeč nad Sázavou, podíl na společných částech domu a pozemku 629/8741</t>
+          <t>č. 96/5 Ládví</t>
         </is>
       </c>
       <c r="G24" t="n">
@@ -1340,37 +1340,37 @@
       </c>
       <c r="H24" t="inlineStr">
         <is>
-          <t>jednotka na parcele s prefixem st. + KU</t>
+          <t>číslo a KU za ním</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="n">
-        <v>58824</v>
+        <v>47777</v>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>jednotka</t>
+          <t>parcela</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>Havlíčkův Brod</t>
+          <t>Praha-východ</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>st. 722</t>
+          <t>97/10</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>Ledeč nad Sázavou</t>
+          <t>Ládví</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>jednotka č. 6700007, byt v budově č.p. 670, část obce Ledeč nad Sázavou, na parcele st. 722 Ledeč nad Sázavou, podíl na společných částech domu a pozemku 52/1000</t>
+          <t>č. 97/10 Ládví</t>
         </is>
       </c>
       <c r="G25" t="n">
@@ -1378,37 +1378,37 @@
       </c>
       <c r="H25" t="inlineStr">
         <is>
-          <t>jednotka na parcele s prefixem st. + KU</t>
+          <t>číslo a KU za ním</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="n">
-        <v>58823</v>
+        <v>47776</v>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>parcela</t>
+          <t>budova</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>Havlíčkův Brod</t>
+          <t>Praha-východ</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>823/5</t>
+          <t>st. 1315</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>Ledeč nad Sázavou</t>
+          <t>Ládví</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>č. 823/5 Ledeč nad Sázavou</t>
+          <t>stavební č. 1315 Ládví (součástí je stavba č.p. 2132, čst obce Ládví)</t>
         </is>
       </c>
       <c r="G26" t="n">
@@ -1416,13 +1416,13 @@
       </c>
       <c r="H26" t="inlineStr">
         <is>
-          <t>číslo a KU za ním</t>
+          <t>č. + KU</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="n">
-        <v>58822</v>
+        <v>47775</v>
       </c>
       <c r="B27" t="inlineStr">
         <is>
@@ -1431,22 +1431,22 @@
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>Havlíčkův Brod</t>
+          <t>Praha-východ</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>823/25</t>
+          <t>511/4</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>Ledeč nad Sázavou</t>
+          <t>Ládví</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>č. 823/25 Ledeč nad Sázavou</t>
+          <t>č. 511/4 Ládví</t>
         </is>
       </c>
       <c r="G27" t="n">
@@ -1460,7 +1460,7 @@
     </row>
     <row r="28">
       <c r="A28" t="n">
-        <v>58821</v>
+        <v>47774</v>
       </c>
       <c r="B28" t="inlineStr">
         <is>
@@ -1469,22 +1469,22 @@
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>Havlíčkův Brod</t>
+          <t>Praha-východ</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>823/32</t>
+          <t>103/17</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>Ledeč nad Sázavou</t>
+          <t>Ládví</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>č. 823/32 Ledeč nad Sázavou</t>
+          <t>č. 103/17 Ládví</t>
         </is>
       </c>
       <c r="G28" t="n">
@@ -1498,31 +1498,31 @@
     </row>
     <row r="29">
       <c r="A29" t="n">
-        <v>58820</v>
+        <v>47773</v>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>budova</t>
+          <t>parcela</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>Havlíčkův Brod</t>
+          <t>Praha-východ</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>st. 1640</t>
+          <t>27/10</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>Ledeč nad Sázavou</t>
+          <t>Ládví</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>stavební č. 1640 Ledeč nad Sázavou (součástí je stavba budova bez čp/če, garáž)</t>
+          <t>č. 27/10 Ládví</t>
         </is>
       </c>
       <c r="G29" t="n">
@@ -1530,37 +1530,37 @@
       </c>
       <c r="H29" t="inlineStr">
         <is>
-          <t>č. + KU</t>
+          <t>číslo a KU za ním</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="n">
-        <v>58819</v>
+        <v>47772</v>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>budova</t>
+          <t>parcela</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>Havlíčkův Brod</t>
+          <t>Praha-východ</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>st. 710/2</t>
+          <t>103/16</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>Ledeč nad Sázavou</t>
+          <t>Ládví</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>stavební č. 710/2 Ledeč nad Sázavou (součástí je stavba budova bez čp/če, jiná stavba)</t>
+          <t>č. 103/16 Ládví</t>
         </is>
       </c>
       <c r="G30" t="n">
@@ -1568,37 +1568,37 @@
       </c>
       <c r="H30" t="inlineStr">
         <is>
-          <t>č. + KU</t>
+          <t>číslo a KU za ním</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="n">
-        <v>58818</v>
+        <v>47771</v>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>budova</t>
+          <t>parcela</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>Havlíčkův Brod</t>
+          <t>Praha-východ</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>st. 710/1</t>
+          <t>103/12</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>Ledeč nad Sázavou</t>
+          <t>Ládví</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>stavební č. 710/1 Ledeč nad Sázavou (součástí je stavba č.p. 674, čst obce Ledeč nad Sázavou)</t>
+          <t>č. 103/12 Ládví</t>
         </is>
       </c>
       <c r="G31" t="n">
@@ -1606,13 +1606,13 @@
       </c>
       <c r="H31" t="inlineStr">
         <is>
-          <t>č. + KU</t>
+          <t>číslo a KU za ním</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="n">
-        <v>58817</v>
+        <v>47770</v>
       </c>
       <c r="B32" t="inlineStr">
         <is>
@@ -1621,22 +1621,22 @@
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>Havlíčkův Brod</t>
+          <t>Praha-východ</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>964</t>
+          <t>102/8</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>Ledeč nad Sázavou</t>
+          <t>Ládví</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>č. 964 Ledeč nad Sázavou</t>
+          <t>č. 102/8 Ládví</t>
         </is>
       </c>
       <c r="G32" t="n">
@@ -1650,31 +1650,31 @@
     </row>
     <row r="33">
       <c r="A33" t="n">
-        <v>58816</v>
+        <v>47769</v>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>jednotka</t>
+          <t>parcela</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>Havlíčkův Brod</t>
+          <t>Praha-východ</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>st. 601</t>
+          <t>103/10</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>Ledeč nad Sázavou</t>
+          <t>Ládví</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>jednotka č. 5560004, byt v budově č.p. 557, 555, 556, část obce Ledeč nad Sázavou, na parcele st. 601 Ledeč nad Sázavou, podíl na společných částech domu a pozemku 519/9693</t>
+          <t>č. 103/10 Ládví</t>
         </is>
       </c>
       <c r="G33" t="n">
@@ -1682,37 +1682,37 @@
       </c>
       <c r="H33" t="inlineStr">
         <is>
-          <t>jednotka na parcele s prefixem st. + KU</t>
+          <t>číslo a KU za ním</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="n">
-        <v>58815</v>
+        <v>47768</v>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>jednotka</t>
+          <t>parcela</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>Hlavní město Praha</t>
+          <t>Praha-východ</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>429/48</t>
+          <t>103/13</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>Libuš</t>
+          <t>Ládví</t>
         </is>
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>jednotka č. 9860006, garáž v budově č.p. 986, část obce Libuš, na parcele 429/48 Libuš, podíl na společných částech domu a pozemku 184814/679789</t>
+          <t>č. 103/13 Ládví</t>
         </is>
       </c>
       <c r="G34" t="n">
@@ -1720,13 +1720,13 @@
       </c>
       <c r="H34" t="inlineStr">
         <is>
-          <t>jednotka na parcele bez prefixu st. + KU</t>
+          <t>číslo a KU za ním</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="n">
-        <v>58814</v>
+        <v>47767</v>
       </c>
       <c r="B35" t="inlineStr">
         <is>
@@ -1735,22 +1735,22 @@
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>Hlavní město Praha</t>
+          <t>Praha-východ</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>429/48</t>
+          <t>st. 118</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>Libuš</t>
+          <t>Ládví</t>
         </is>
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>jednotka č. 9860410, byt v budově č.p. 986, část obce Libuš, na parcele 429/48 Libuš, podíl na společných částech domu a pozemku 5732/679789</t>
+          <t>jednotka č. 11480029, byt v budově č.p. 1148, část obce Ládví, na parcele st. 118 Ládví, podíl na společných částech domu a pozemku 732/32916</t>
         </is>
       </c>
       <c r="G35" t="n">
@@ -1758,13 +1758,13 @@
       </c>
       <c r="H35" t="inlineStr">
         <is>
-          <t>jednotka na parcele bez prefixu st. + KU</t>
+          <t>jednotka na parcele s prefixem st. + KU</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="n">
-        <v>58813</v>
+        <v>47766</v>
       </c>
       <c r="B36" t="inlineStr">
         <is>
@@ -1773,22 +1773,22 @@
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>Hlavní město Praha</t>
+          <t>Praha-východ</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>1123/116</t>
+          <t>364/36</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>Libuš</t>
+          <t>Ládví</t>
         </is>
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>č. 1123/116 Libuš</t>
+          <t>č. 364/36 Ládví</t>
         </is>
       </c>
       <c r="G36" t="n">
@@ -1802,7 +1802,7 @@
     </row>
     <row r="37">
       <c r="A37" t="n">
-        <v>58812</v>
+        <v>47765</v>
       </c>
       <c r="B37" t="inlineStr">
         <is>
@@ -1811,22 +1811,22 @@
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>Hlavní město Praha</t>
+          <t>Praha-východ</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>1123/76</t>
+          <t>798</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>Libuš</t>
+          <t>Ládví</t>
         </is>
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>č. 1123/76 Libuš</t>
+          <t>č. 798 Ládví</t>
         </is>
       </c>
       <c r="G37" t="n">
@@ -1840,7 +1840,7 @@
     </row>
     <row r="38">
       <c r="A38" t="n">
-        <v>58811</v>
+        <v>47764</v>
       </c>
       <c r="B38" t="inlineStr">
         <is>
@@ -1849,22 +1849,22 @@
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>Hlavní město Praha</t>
+          <t>Praha-východ</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>1123/73</t>
+          <t>618/9</t>
         </is>
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>Libuš</t>
+          <t>Ládví</t>
         </is>
       </c>
       <c r="F38" t="inlineStr">
         <is>
-          <t>č. 1123/73 Libuš</t>
+          <t>č. 618/9 Ládví</t>
         </is>
       </c>
       <c r="G38" t="n">
@@ -1878,31 +1878,31 @@
     </row>
     <row r="39">
       <c r="A39" t="n">
-        <v>58810</v>
+        <v>47763</v>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>parcela</t>
+          <t>budova</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>Hlavní město Praha</t>
+          <t>Praha-východ</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>1123/120</t>
+          <t>st. 931</t>
         </is>
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>Libuš</t>
+          <t>Ládví</t>
         </is>
       </c>
       <c r="F39" t="inlineStr">
         <is>
-          <t>č. 1123/120 Libuš</t>
+          <t>stavební č. 931 Ládví (součástí je stavba č.p. 1434, čst obce Olešovice)</t>
         </is>
       </c>
       <c r="G39" t="n">
@@ -1910,13 +1910,13 @@
       </c>
       <c r="H39" t="inlineStr">
         <is>
-          <t>číslo a KU za ním</t>
+          <t>č. + KU</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="n">
-        <v>58809</v>
+        <v>47762</v>
       </c>
       <c r="B40" t="inlineStr">
         <is>
@@ -1925,22 +1925,22 @@
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>Hlavní město Praha</t>
+          <t>Praha-východ</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>1123/118</t>
+          <t>578/3</t>
         </is>
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>Libuš</t>
+          <t>Ládví</t>
         </is>
       </c>
       <c r="F40" t="inlineStr">
         <is>
-          <t>č. 1123/118 Libuš</t>
+          <t>č. 578/3 Ládví</t>
         </is>
       </c>
       <c r="G40" t="n">
@@ -1954,7 +1954,7 @@
     </row>
     <row r="41">
       <c r="A41" t="n">
-        <v>58808</v>
+        <v>47761</v>
       </c>
       <c r="B41" t="inlineStr">
         <is>
@@ -1963,22 +1963,22 @@
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>Hlavní město Praha</t>
+          <t>Praha-východ</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>1123/119</t>
+          <t>578/2</t>
         </is>
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>Libuš</t>
+          <t>Ládví</t>
         </is>
       </c>
       <c r="F41" t="inlineStr">
         <is>
-          <t>č. 1123/119 Libuš</t>
+          <t>č. 578/2 Ládví</t>
         </is>
       </c>
       <c r="G41" t="n">
@@ -1992,7 +1992,7 @@
     </row>
     <row r="42">
       <c r="A42" t="n">
-        <v>58807</v>
+        <v>47760</v>
       </c>
       <c r="B42" t="inlineStr">
         <is>
@@ -2001,22 +2001,22 @@
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>Hlavní město Praha</t>
+          <t>Praha-východ</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>1123/117</t>
+          <t>578/1</t>
         </is>
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>Libuš</t>
+          <t>Ládví</t>
         </is>
       </c>
       <c r="F42" t="inlineStr">
         <is>
-          <t>č. 1123/117 Libuš</t>
+          <t>č. 578/1 Ládví</t>
         </is>
       </c>
       <c r="G42" t="n">
@@ -2030,7 +2030,7 @@
     </row>
     <row r="43">
       <c r="A43" t="n">
-        <v>58806</v>
+        <v>47759</v>
       </c>
       <c r="B43" t="inlineStr">
         <is>
@@ -2039,22 +2039,22 @@
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>Hlavní město Praha</t>
+          <t>Praha-východ</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>2382/8</t>
+          <t>340/1</t>
         </is>
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>Kunratice</t>
+          <t>Ládví</t>
         </is>
       </c>
       <c r="F43" t="inlineStr">
         <is>
-          <t>č. 2382/8 Kunratice</t>
+          <t>č. 340/1 Ládví</t>
         </is>
       </c>
       <c r="G43" t="n">
@@ -2068,7 +2068,7 @@
     </row>
     <row r="44">
       <c r="A44" t="n">
-        <v>58805</v>
+        <v>47758</v>
       </c>
       <c r="B44" t="inlineStr">
         <is>
@@ -2077,22 +2077,22 @@
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>Hlavní město Praha</t>
+          <t>Praha-východ</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>2342/27</t>
+          <t>432/9</t>
         </is>
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>Kunratice</t>
+          <t>Ládví</t>
         </is>
       </c>
       <c r="F44" t="inlineStr">
         <is>
-          <t>č. 2342/27 Kunratice</t>
+          <t>č. 432/9 Ládví</t>
         </is>
       </c>
       <c r="G44" t="n">
@@ -2106,7 +2106,7 @@
     </row>
     <row r="45">
       <c r="A45" t="n">
-        <v>58804</v>
+        <v>47757</v>
       </c>
       <c r="B45" t="inlineStr">
         <is>
@@ -2115,22 +2115,22 @@
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>Hlavní město Praha</t>
+          <t>Praha-východ</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>2342/30</t>
+          <t>432/8</t>
         </is>
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>Kunratice</t>
+          <t>Ládví</t>
         </is>
       </c>
       <c r="F45" t="inlineStr">
         <is>
-          <t>č. 2342/30 Kunratice</t>
+          <t>č. 432/8 Ládví</t>
         </is>
       </c>
       <c r="G45" t="n">
@@ -2144,7 +2144,7 @@
     </row>
     <row r="46">
       <c r="A46" t="n">
-        <v>58803</v>
+        <v>47756</v>
       </c>
       <c r="B46" t="inlineStr">
         <is>
@@ -2153,22 +2153,22 @@
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>Hlavní město Praha</t>
+          <t>Praha-východ</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>2342/28</t>
+          <t>430/2</t>
         </is>
       </c>
       <c r="E46" t="inlineStr">
         <is>
-          <t>Kunratice</t>
+          <t>Ládví</t>
         </is>
       </c>
       <c r="F46" t="inlineStr">
         <is>
-          <t>č. 2342/28 Kunratice</t>
+          <t>č. 430/2 Ládví</t>
         </is>
       </c>
       <c r="G46" t="n">
@@ -2182,7 +2182,7 @@
     </row>
     <row r="47">
       <c r="A47" t="n">
-        <v>58802</v>
+        <v>47755</v>
       </c>
       <c r="B47" t="inlineStr">
         <is>
@@ -2191,22 +2191,22 @@
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>Hlavní město Praha</t>
+          <t>Praha-východ</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>2342/29</t>
+          <t>459/9</t>
         </is>
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t>Kunratice</t>
+          <t>Ládví</t>
         </is>
       </c>
       <c r="F47" t="inlineStr">
         <is>
-          <t>č. 2342/29 Kunratice</t>
+          <t>č. 459/9 Ládví</t>
         </is>
       </c>
       <c r="G47" t="n">
@@ -2220,7 +2220,7 @@
     </row>
     <row r="48">
       <c r="A48" t="n">
-        <v>58801</v>
+        <v>47754</v>
       </c>
       <c r="B48" t="inlineStr">
         <is>
@@ -2229,22 +2229,22 @@
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>Hlavní město Praha</t>
+          <t>Praha-východ</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>2342/31</t>
+          <t>st. 1186</t>
         </is>
       </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t>Kunratice</t>
+          <t>Ládví</t>
         </is>
       </c>
       <c r="F48" t="inlineStr">
         <is>
-          <t>č. 2342/31 Kunratice</t>
+          <t>stavební č. 1186 Ládví (součástí je stavba budova bez čp/če, jiná stavba)</t>
         </is>
       </c>
       <c r="G48" t="n">
@@ -2258,31 +2258,31 @@
     </row>
     <row r="49">
       <c r="A49" t="n">
-        <v>58800</v>
+        <v>47753</v>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>jednotka</t>
+          <t>budova</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>Hlavní město Praha</t>
+          <t>Praha-východ</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>2342/27</t>
+          <t>st. 476</t>
         </is>
       </c>
       <c r="E49" t="inlineStr">
         <is>
-          <t>Kunratice</t>
+          <t>Ládví</t>
         </is>
       </c>
       <c r="F49" t="inlineStr">
         <is>
-          <t>jednotka č. 11500902, garáž v budově č.p. 1152, 1148, 1149, 1150, 1151, část obce Kunratice, na parcele 2342/27 Kunratice, 2342/28 Kunratice, 2342/29 Kunratice, 2342/30 Kunratice, 2342/31 Kunratice, podíl na společných částech domu a pozemku 17/7754</t>
+          <t>stavební č. 476 Ládví (součástí je stavba č.e. 1424, čst obce Ládví)</t>
         </is>
       </c>
       <c r="G49" t="n">
@@ -2290,37 +2290,37 @@
       </c>
       <c r="H49" t="inlineStr">
         <is>
-          <t>jednotka na parcele bez prefixu st. + KU</t>
+          <t>č. + KU</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="n">
-        <v>58800</v>
+        <v>47752</v>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>jednotka</t>
+          <t>parcela</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>Hlavní město Praha</t>
+          <t>Praha-východ</t>
         </is>
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>2342/28</t>
+          <t>519/1</t>
         </is>
       </c>
       <c r="E50" t="inlineStr">
         <is>
-          <t>Kunratice</t>
+          <t>Ládví</t>
         </is>
       </c>
       <c r="F50" t="inlineStr">
         <is>
-          <t>jednotka č. 11500902, garáž v budově č.p. 1152, 1148, 1149, 1150, 1151, část obce Kunratice, na parcele 2342/27 Kunratice, 2342/28 Kunratice, 2342/29 Kunratice, 2342/30 Kunratice, 2342/31 Kunratice, podíl na společných částech domu a pozemku 17/7754</t>
+          <t>č. 519/1 Ládví</t>
         </is>
       </c>
       <c r="G50" t="n">
@@ -2328,37 +2328,37 @@
       </c>
       <c r="H50" t="inlineStr">
         <is>
-          <t>více parcel oddělených čárkou</t>
+          <t>číslo a KU za ním</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="n">
-        <v>58800</v>
+        <v>47751</v>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>jednotka</t>
+          <t>budova</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>Hlavní město Praha</t>
+          <t>Praha-východ</t>
         </is>
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>2342/29</t>
+          <t>st. 128</t>
         </is>
       </c>
       <c r="E51" t="inlineStr">
         <is>
-          <t>Kunratice</t>
+          <t>Ládví</t>
         </is>
       </c>
       <c r="F51" t="inlineStr">
         <is>
-          <t>jednotka č. 11500902, garáž v budově č.p. 1152, 1148, 1149, 1150, 1151, část obce Kunratice, na parcele 2342/27 Kunratice, 2342/28 Kunratice, 2342/29 Kunratice, 2342/30 Kunratice, 2342/31 Kunratice, podíl na společných částech domu a pozemku 17/7754</t>
+          <t>stavební č. 128 Ládví (součástí je stavba č.e. 1485, čst obce Ládví)</t>
         </is>
       </c>
       <c r="G51" t="n">
@@ -2366,501 +2366,7 @@
       </c>
       <c r="H51" t="inlineStr">
         <is>
-          <t>více parcel oddělených čárkou</t>
-        </is>
-      </c>
-    </row>
-    <row r="52">
-      <c r="A52" t="n">
-        <v>58800</v>
-      </c>
-      <c r="B52" t="inlineStr">
-        <is>
-          <t>jednotka</t>
-        </is>
-      </c>
-      <c r="C52" t="inlineStr">
-        <is>
-          <t>Hlavní město Praha</t>
-        </is>
-      </c>
-      <c r="D52" t="inlineStr">
-        <is>
-          <t>2342/30</t>
-        </is>
-      </c>
-      <c r="E52" t="inlineStr">
-        <is>
-          <t>Kunratice</t>
-        </is>
-      </c>
-      <c r="F52" t="inlineStr">
-        <is>
-          <t>jednotka č. 11500902, garáž v budově č.p. 1152, 1148, 1149, 1150, 1151, část obce Kunratice, na parcele 2342/27 Kunratice, 2342/28 Kunratice, 2342/29 Kunratice, 2342/30 Kunratice, 2342/31 Kunratice, podíl na společných částech domu a pozemku 17/7754</t>
-        </is>
-      </c>
-      <c r="G52" t="n">
-        <v>1</v>
-      </c>
-      <c r="H52" t="inlineStr">
-        <is>
-          <t>více parcel oddělených čárkou</t>
-        </is>
-      </c>
-    </row>
-    <row r="53">
-      <c r="A53" t="n">
-        <v>58800</v>
-      </c>
-      <c r="B53" t="inlineStr">
-        <is>
-          <t>jednotka</t>
-        </is>
-      </c>
-      <c r="C53" t="inlineStr">
-        <is>
-          <t>Hlavní město Praha</t>
-        </is>
-      </c>
-      <c r="D53" t="inlineStr">
-        <is>
-          <t>2342/31</t>
-        </is>
-      </c>
-      <c r="E53" t="inlineStr">
-        <is>
-          <t>Kunratice</t>
-        </is>
-      </c>
-      <c r="F53" t="inlineStr">
-        <is>
-          <t>jednotka č. 11500902, garáž v budově č.p. 1152, 1148, 1149, 1150, 1151, část obce Kunratice, na parcele 2342/27 Kunratice, 2342/28 Kunratice, 2342/29 Kunratice, 2342/30 Kunratice, 2342/31 Kunratice, podíl na společných částech domu a pozemku 17/7754</t>
-        </is>
-      </c>
-      <c r="G53" t="n">
-        <v>1</v>
-      </c>
-      <c r="H53" t="inlineStr">
-        <is>
-          <t>více parcel oddělených čárkou</t>
-        </is>
-      </c>
-    </row>
-    <row r="54">
-      <c r="A54" t="n">
-        <v>58799</v>
-      </c>
-      <c r="B54" t="inlineStr">
-        <is>
-          <t>jednotka</t>
-        </is>
-      </c>
-      <c r="C54" t="inlineStr">
-        <is>
-          <t>Hlavní město Praha</t>
-        </is>
-      </c>
-      <c r="D54" t="inlineStr">
-        <is>
-          <t>2342/27</t>
-        </is>
-      </c>
-      <c r="E54" t="inlineStr">
-        <is>
-          <t>Kunratice</t>
-        </is>
-      </c>
-      <c r="F54" t="inlineStr">
-        <is>
-          <t>jednotka č. 11500061, byt v budově č.p. 1152, 1148, 1149, 1150, 1151, část obce Kunratice, na parcele 2342/27 Kunratice, 2342/28 Kunratice, 2342/29 Kunratice, 2342/30 Kunratice, 2342/31 Kunratice, podíl na společných částech domu a pozemku 82/7754</t>
-        </is>
-      </c>
-      <c r="G54" t="n">
-        <v>1</v>
-      </c>
-      <c r="H54" t="inlineStr">
-        <is>
-          <t>jednotka na parcele bez prefixu st. + KU</t>
-        </is>
-      </c>
-    </row>
-    <row r="55">
-      <c r="A55" t="n">
-        <v>58799</v>
-      </c>
-      <c r="B55" t="inlineStr">
-        <is>
-          <t>jednotka</t>
-        </is>
-      </c>
-      <c r="C55" t="inlineStr">
-        <is>
-          <t>Hlavní město Praha</t>
-        </is>
-      </c>
-      <c r="D55" t="inlineStr">
-        <is>
-          <t>2342/28</t>
-        </is>
-      </c>
-      <c r="E55" t="inlineStr">
-        <is>
-          <t>Kunratice</t>
-        </is>
-      </c>
-      <c r="F55" t="inlineStr">
-        <is>
-          <t>jednotka č. 11500061, byt v budově č.p. 1152, 1148, 1149, 1150, 1151, část obce Kunratice, na parcele 2342/27 Kunratice, 2342/28 Kunratice, 2342/29 Kunratice, 2342/30 Kunratice, 2342/31 Kunratice, podíl na společných částech domu a pozemku 82/7754</t>
-        </is>
-      </c>
-      <c r="G55" t="n">
-        <v>1</v>
-      </c>
-      <c r="H55" t="inlineStr">
-        <is>
-          <t>více parcel oddělených čárkou</t>
-        </is>
-      </c>
-    </row>
-    <row r="56">
-      <c r="A56" t="n">
-        <v>58799</v>
-      </c>
-      <c r="B56" t="inlineStr">
-        <is>
-          <t>jednotka</t>
-        </is>
-      </c>
-      <c r="C56" t="inlineStr">
-        <is>
-          <t>Hlavní město Praha</t>
-        </is>
-      </c>
-      <c r="D56" t="inlineStr">
-        <is>
-          <t>2342/29</t>
-        </is>
-      </c>
-      <c r="E56" t="inlineStr">
-        <is>
-          <t>Kunratice</t>
-        </is>
-      </c>
-      <c r="F56" t="inlineStr">
-        <is>
-          <t>jednotka č. 11500061, byt v budově č.p. 1152, 1148, 1149, 1150, 1151, část obce Kunratice, na parcele 2342/27 Kunratice, 2342/28 Kunratice, 2342/29 Kunratice, 2342/30 Kunratice, 2342/31 Kunratice, podíl na společných částech domu a pozemku 82/7754</t>
-        </is>
-      </c>
-      <c r="G56" t="n">
-        <v>1</v>
-      </c>
-      <c r="H56" t="inlineStr">
-        <is>
-          <t>více parcel oddělených čárkou</t>
-        </is>
-      </c>
-    </row>
-    <row r="57">
-      <c r="A57" t="n">
-        <v>58799</v>
-      </c>
-      <c r="B57" t="inlineStr">
-        <is>
-          <t>jednotka</t>
-        </is>
-      </c>
-      <c r="C57" t="inlineStr">
-        <is>
-          <t>Hlavní město Praha</t>
-        </is>
-      </c>
-      <c r="D57" t="inlineStr">
-        <is>
-          <t>2342/30</t>
-        </is>
-      </c>
-      <c r="E57" t="inlineStr">
-        <is>
-          <t>Kunratice</t>
-        </is>
-      </c>
-      <c r="F57" t="inlineStr">
-        <is>
-          <t>jednotka č. 11500061, byt v budově č.p. 1152, 1148, 1149, 1150, 1151, část obce Kunratice, na parcele 2342/27 Kunratice, 2342/28 Kunratice, 2342/29 Kunratice, 2342/30 Kunratice, 2342/31 Kunratice, podíl na společných částech domu a pozemku 82/7754</t>
-        </is>
-      </c>
-      <c r="G57" t="n">
-        <v>1</v>
-      </c>
-      <c r="H57" t="inlineStr">
-        <is>
-          <t>více parcel oddělených čárkou</t>
-        </is>
-      </c>
-    </row>
-    <row r="58">
-      <c r="A58" t="n">
-        <v>58799</v>
-      </c>
-      <c r="B58" t="inlineStr">
-        <is>
-          <t>jednotka</t>
-        </is>
-      </c>
-      <c r="C58" t="inlineStr">
-        <is>
-          <t>Hlavní město Praha</t>
-        </is>
-      </c>
-      <c r="D58" t="inlineStr">
-        <is>
-          <t>2342/31</t>
-        </is>
-      </c>
-      <c r="E58" t="inlineStr">
-        <is>
-          <t>Kunratice</t>
-        </is>
-      </c>
-      <c r="F58" t="inlineStr">
-        <is>
-          <t>jednotka č. 11500061, byt v budově č.p. 1152, 1148, 1149, 1150, 1151, část obce Kunratice, na parcele 2342/27 Kunratice, 2342/28 Kunratice, 2342/29 Kunratice, 2342/30 Kunratice, 2342/31 Kunratice, podíl na společných částech domu a pozemku 82/7754</t>
-        </is>
-      </c>
-      <c r="G58" t="n">
-        <v>1</v>
-      </c>
-      <c r="H58" t="inlineStr">
-        <is>
-          <t>více parcel oddělených čárkou</t>
-        </is>
-      </c>
-    </row>
-    <row r="59">
-      <c r="A59" t="n">
-        <v>58798</v>
-      </c>
-      <c r="B59" t="inlineStr">
-        <is>
-          <t>parcela</t>
-        </is>
-      </c>
-      <c r="C59" t="inlineStr">
-        <is>
-          <t>Hlavní město Praha</t>
-        </is>
-      </c>
-      <c r="D59" t="inlineStr">
-        <is>
-          <t>1433/13</t>
-        </is>
-      </c>
-      <c r="E59" t="inlineStr">
-        <is>
-          <t>Kunratice</t>
-        </is>
-      </c>
-      <c r="F59" t="inlineStr">
-        <is>
-          <t>č. 1433/13 Kunratice</t>
-        </is>
-      </c>
-      <c r="G59" t="n">
-        <v>1</v>
-      </c>
-      <c r="H59" t="inlineStr">
-        <is>
-          <t>číslo a KU za ním</t>
-        </is>
-      </c>
-    </row>
-    <row r="60">
-      <c r="A60" t="n">
-        <v>58797</v>
-      </c>
-      <c r="B60" t="inlineStr">
-        <is>
-          <t>parcela</t>
-        </is>
-      </c>
-      <c r="C60" t="inlineStr">
-        <is>
-          <t>Hlavní město Praha</t>
-        </is>
-      </c>
-      <c r="D60" t="inlineStr">
-        <is>
-          <t>1433/12</t>
-        </is>
-      </c>
-      <c r="E60" t="inlineStr">
-        <is>
-          <t>Kunratice</t>
-        </is>
-      </c>
-      <c r="F60" t="inlineStr">
-        <is>
-          <t>č. 1433/12 Kunratice</t>
-        </is>
-      </c>
-      <c r="G60" t="n">
-        <v>1</v>
-      </c>
-      <c r="H60" t="inlineStr">
-        <is>
-          <t>číslo a KU za ním</t>
-        </is>
-      </c>
-    </row>
-    <row r="61">
-      <c r="A61" t="n">
-        <v>58796</v>
-      </c>
-      <c r="B61" t="inlineStr">
-        <is>
-          <t>parcela</t>
-        </is>
-      </c>
-      <c r="C61" t="inlineStr">
-        <is>
-          <t>Hlavní město Praha</t>
-        </is>
-      </c>
-      <c r="D61" t="inlineStr">
-        <is>
-          <t>59/12</t>
-        </is>
-      </c>
-      <c r="E61" t="inlineStr">
-        <is>
-          <t>Kunratice</t>
-        </is>
-      </c>
-      <c r="F61" t="inlineStr">
-        <is>
-          <t>č. 59/12 Kunratice</t>
-        </is>
-      </c>
-      <c r="G61" t="n">
-        <v>1</v>
-      </c>
-      <c r="H61" t="inlineStr">
-        <is>
-          <t>číslo a KU za ním</t>
-        </is>
-      </c>
-    </row>
-    <row r="62">
-      <c r="A62" t="n">
-        <v>58795</v>
-      </c>
-      <c r="B62" t="inlineStr">
-        <is>
-          <t>budova</t>
-        </is>
-      </c>
-      <c r="C62" t="inlineStr">
-        <is>
-          <t>Hlavní město Praha</t>
-        </is>
-      </c>
-      <c r="D62" t="inlineStr">
-        <is>
-          <t>59/45</t>
-        </is>
-      </c>
-      <c r="E62" t="inlineStr">
-        <is>
-          <t>Kunratice</t>
-        </is>
-      </c>
-      <c r="F62" t="inlineStr">
-        <is>
-          <t>č. 59/45 Kunratice (součástí je stavba č.p. 1045, čst obce Kunratice)</t>
-        </is>
-      </c>
-      <c r="G62" t="n">
-        <v>1</v>
-      </c>
-      <c r="H62" t="inlineStr">
-        <is>
           <t>č. + KU</t>
-        </is>
-      </c>
-    </row>
-    <row r="63">
-      <c r="A63" t="n">
-        <v>58794</v>
-      </c>
-      <c r="B63" t="inlineStr">
-        <is>
-          <t>budova</t>
-        </is>
-      </c>
-      <c r="C63" t="inlineStr">
-        <is>
-          <t>Hlavní město Praha</t>
-        </is>
-      </c>
-      <c r="D63" t="inlineStr">
-        <is>
-          <t>267/9</t>
-        </is>
-      </c>
-      <c r="E63" t="inlineStr">
-        <is>
-          <t>Kunratice</t>
-        </is>
-      </c>
-      <c r="F63" t="inlineStr">
-        <is>
-          <t>budova bez čp/če, jiná stavba, na parcele 267/9 Kunratice</t>
-        </is>
-      </c>
-      <c r="G63" t="n">
-        <v>1</v>
-      </c>
-      <c r="H63" t="inlineStr">
-        <is>
-          <t>budova na parcele č.</t>
-        </is>
-      </c>
-    </row>
-    <row r="64">
-      <c r="A64" t="n">
-        <v>58793</v>
-      </c>
-      <c r="B64" t="inlineStr">
-        <is>
-          <t>parcela</t>
-        </is>
-      </c>
-      <c r="C64" t="inlineStr">
-        <is>
-          <t>Hlavní město Praha</t>
-        </is>
-      </c>
-      <c r="D64" t="inlineStr">
-        <is>
-          <t>2428/21</t>
-        </is>
-      </c>
-      <c r="E64" t="inlineStr">
-        <is>
-          <t>Kunratice</t>
-        </is>
-      </c>
-      <c r="F64" t="inlineStr">
-        <is>
-          <t>č. 2428/21 Kunratice</t>
-        </is>
-      </c>
-      <c r="G64" t="n">
-        <v>1</v>
-      </c>
-      <c r="H64" t="inlineStr">
-        <is>
-          <t>číslo a KU za ním</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update vystup.xlsx with new data and formatting changes
</commit_message>
<xml_diff>
--- a/GIS2/vystup.xlsx
+++ b/GIS2/vystup.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H51"/>
+  <dimension ref="A1:H71"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -472,7 +472,7 @@
     </row>
     <row r="2">
       <c r="A2" t="n">
-        <v>47800</v>
+        <v>55243</v>
       </c>
       <c r="B2" t="inlineStr">
         <is>
@@ -481,22 +481,22 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Praha-východ</t>
+          <t>Hlavní město Praha</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>st. 646</t>
+          <t>1921/32</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>Ládví</t>
+          <t>Braník</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>jednotka č. 4680004, byt v budově č.p. 468, 467, 469, část obce Olešovice, na parcele st. 646 Ládví, podíl na společných částech domu a pozemku 7596/110533</t>
+          <t>jednotka č. 508, garáž v budově budova bez čp/če, garáž, na parcele 1921/32 Braník, 1921/33 Braník, 1921/34 Braník, 1921/35 Braník, 1921/36 Braník, 1921/37 Braník, 1921/38 Braník, 1921/39 Braník, podíl na společných částech domu a pozemku 19/140</t>
         </is>
       </c>
       <c r="G2" t="n">
@@ -504,37 +504,37 @@
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>jednotka na parcele s prefixem st. + KU</t>
+          <t>jednotka na parcele bez prefixu st. + KU</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="n">
-        <v>47799</v>
+        <v>55243</v>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>parcela</t>
+          <t>jednotka</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Praha-východ</t>
+          <t>Hlavní město Praha</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>748/43</t>
+          <t>1921/33</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>Ládví</t>
+          <t>Braník</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>č. 748/43 Ládví</t>
+          <t>jednotka č. 508, garáž v budově budova bez čp/če, garáž, na parcele 1921/32 Braník, 1921/33 Braník, 1921/34 Braník, 1921/35 Braník, 1921/36 Braník, 1921/37 Braník, 1921/38 Braník, 1921/39 Braník, podíl na společných částech domu a pozemku 19/140</t>
         </is>
       </c>
       <c r="G3" t="n">
@@ -542,37 +542,37 @@
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>číslo a KU za ním</t>
+          <t>více parcel oddělených čárkou</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="n">
-        <v>47798</v>
+        <v>55243</v>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>budova</t>
+          <t>jednotka</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Praha-východ</t>
+          <t>Hlavní město Praha</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>st. 334</t>
+          <t>1921/34</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>Ládví</t>
+          <t>Braník</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>stavební č. 334 Ládví (součástí je stavba č.p. 154, čst obce Ládví)</t>
+          <t>jednotka č. 508, garáž v budově budova bez čp/če, garáž, na parcele 1921/32 Braník, 1921/33 Braník, 1921/34 Braník, 1921/35 Braník, 1921/36 Braník, 1921/37 Braník, 1921/38 Braník, 1921/39 Braník, podíl na společných částech domu a pozemku 19/140</t>
         </is>
       </c>
       <c r="G4" t="n">
@@ -580,37 +580,37 @@
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>č. + KU</t>
+          <t>více parcel oddělených čárkou</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="n">
-        <v>47797</v>
+        <v>55243</v>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>parcela</t>
+          <t>jednotka</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Praha-východ</t>
+          <t>Hlavní město Praha</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>125/12</t>
+          <t>1921/35</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>Ládví</t>
+          <t>Braník</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>č. 125/12 Ládví</t>
+          <t>jednotka č. 508, garáž v budově budova bez čp/če, garáž, na parcele 1921/32 Braník, 1921/33 Braník, 1921/34 Braník, 1921/35 Braník, 1921/36 Braník, 1921/37 Braník, 1921/38 Braník, 1921/39 Braník, podíl na společných částech domu a pozemku 19/140</t>
         </is>
       </c>
       <c r="G5" t="n">
@@ -618,37 +618,37 @@
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>číslo a KU za ním</t>
+          <t>více parcel oddělených čárkou</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="n">
-        <v>47796</v>
+        <v>55243</v>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>budova</t>
+          <t>jednotka</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Praha-východ</t>
+          <t>Hlavní město Praha</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>st. 1372</t>
+          <t>1921/36</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>Ládví</t>
+          <t>Braník</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>stavební č. 1372 Ládví (součástí je stavba budova bez čp/če, jiná stavba)</t>
+          <t>jednotka č. 508, garáž v budově budova bez čp/če, garáž, na parcele 1921/32 Braník, 1921/33 Braník, 1921/34 Braník, 1921/35 Braník, 1921/36 Braník, 1921/37 Braník, 1921/38 Braník, 1921/39 Braník, podíl na společných částech domu a pozemku 19/140</t>
         </is>
       </c>
       <c r="G6" t="n">
@@ -656,37 +656,37 @@
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>č. + KU</t>
+          <t>více parcel oddělených čárkou</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="n">
-        <v>47795</v>
+        <v>55243</v>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>budova</t>
+          <t>jednotka</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Praha-východ</t>
+          <t>Hlavní město Praha</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>st. 514</t>
+          <t>1921/37</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>Ládví</t>
+          <t>Braník</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>stavební č. 514 Ládví (součástí je stavba č.e. 1347, čst obce Ládví)</t>
+          <t>jednotka č. 508, garáž v budově budova bez čp/če, garáž, na parcele 1921/32 Braník, 1921/33 Braník, 1921/34 Braník, 1921/35 Braník, 1921/36 Braník, 1921/37 Braník, 1921/38 Braník, 1921/39 Braník, podíl na společných částech domu a pozemku 19/140</t>
         </is>
       </c>
       <c r="G7" t="n">
@@ -694,37 +694,37 @@
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>č. + KU</t>
+          <t>více parcel oddělených čárkou</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="n">
-        <v>47794</v>
+        <v>55243</v>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>parcela</t>
+          <t>jednotka</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Praha-východ</t>
+          <t>Hlavní město Praha</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>255/8</t>
+          <t>1921/38</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>Ládví</t>
+          <t>Braník</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>č. 255/8 Ládví</t>
+          <t>jednotka č. 508, garáž v budově budova bez čp/če, garáž, na parcele 1921/32 Braník, 1921/33 Braník, 1921/34 Braník, 1921/35 Braník, 1921/36 Braník, 1921/37 Braník, 1921/38 Braník, 1921/39 Braník, podíl na společných částech domu a pozemku 19/140</t>
         </is>
       </c>
       <c r="G8" t="n">
@@ -732,37 +732,37 @@
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>číslo a KU za ním</t>
+          <t>více parcel oddělených čárkou</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="n">
-        <v>47793</v>
+        <v>55243</v>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>parcela</t>
+          <t>jednotka</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Praha-východ</t>
+          <t>Hlavní město Praha</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>722/12</t>
+          <t>1921/39</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>Ládví</t>
+          <t>Braník</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>č. 722/12 Ládví</t>
+          <t>jednotka č. 508, garáž v budově budova bez čp/če, garáž, na parcele 1921/32 Braník, 1921/33 Braník, 1921/34 Braník, 1921/35 Braník, 1921/36 Braník, 1921/37 Braník, 1921/38 Braník, 1921/39 Braník, podíl na společných částech domu a pozemku 19/140</t>
         </is>
       </c>
       <c r="G9" t="n">
@@ -770,37 +770,37 @@
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>číslo a KU za ním</t>
+          <t>více parcel oddělených čárkou</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="n">
-        <v>47792</v>
+        <v>52108</v>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>parcela</t>
+          <t>jednotka</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Praha-východ</t>
+          <t>Hlavní město Praha</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>234/4</t>
+          <t>1857/142</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>Ládví</t>
+          <t>Kamýk</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>č. 234/4 Ládví</t>
+          <t>jednotka č. 4640062, garáž v budově č.p. 464, část obce Kamýk, na parcele 1857/142 Kamýk, podíl na společných částech domu a pozemku 291/62868</t>
         </is>
       </c>
       <c r="G10" t="n">
@@ -808,37 +808,37 @@
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>číslo a KU za ním</t>
+          <t>jednotka na parcele bez prefixu st. + KU</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="n">
-        <v>47791</v>
+        <v>51882</v>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>parcela</t>
+          <t>jednotka</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Praha-východ</t>
+          <t>Hlavní město Praha</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>646/32</t>
+          <t>1765/5</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>Ládví</t>
+          <t>Nusle</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>č. 646/32 Ládví</t>
+          <t>jednotka č. 17410902, garáž v budově č.p. 1741, část obce Nusle, na parcele 1765/5 Nusle (součástí je stavba č.p. 1741, čst obce Nusle), podíl na společných částech domu a pozemku 23569/70347</t>
         </is>
       </c>
       <c r="G11" t="n">
@@ -846,37 +846,37 @@
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>číslo a KU za ním</t>
+          <t>jednotka na parcele bez prefixu st. + KU</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="n">
-        <v>47790</v>
+        <v>51450</v>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>budova</t>
+          <t>jednotka</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Praha-východ</t>
+          <t>Hlavní město Praha</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>st. 877</t>
+          <t>1857/142</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>Ládví</t>
+          <t>Kamýk</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>stavební č. 877 Ládví (součástí je stavba č.p. 1425, čst obce Olešovice)</t>
+          <t>jednotka č. 4640105, garáž v budově č.p. 464, část obce Kamýk, na parcele 1857/142 Kamýk, podíl na společných částech domu a pozemku 276/62868</t>
         </is>
       </c>
       <c r="G12" t="n">
@@ -884,37 +884,37 @@
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>č. + KU</t>
+          <t>jednotka na parcele bez prefixu st. + KU</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="n">
-        <v>47789</v>
+        <v>49904</v>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>parcela</t>
+          <t>jednotka</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Praha-východ</t>
+          <t>Hlavní město Praha</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>628/4</t>
+          <t>2114/3</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>Ládví</t>
+          <t>Krč</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>č. 628/4 Ládví</t>
+          <t>jednotka č. 15680103, garáž v budově č.p. 1570, 1568, 1569, část obce Krč, na parcele 2114/3 Krč, 2114/4 Krč, 2114/5 Krč, podíl na společných částech domu a pozemku 2230/184350</t>
         </is>
       </c>
       <c r="G13" t="n">
@@ -922,37 +922,37 @@
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>číslo a KU za ním</t>
+          <t>jednotka na parcele bez prefixu st. + KU</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="n">
-        <v>47788</v>
+        <v>49904</v>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>parcela</t>
+          <t>jednotka</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Praha-východ</t>
+          <t>Hlavní město Praha</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>628/33</t>
+          <t>2114/4</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>Ládví</t>
+          <t>Krč</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>č. 628/33 Ládví</t>
+          <t>jednotka č. 15680103, garáž v budově č.p. 1570, 1568, 1569, část obce Krč, na parcele 2114/3 Krč, 2114/4 Krč, 2114/5 Krč, podíl na společných částech domu a pozemku 2230/184350</t>
         </is>
       </c>
       <c r="G14" t="n">
@@ -960,13 +960,13 @@
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>číslo a KU za ním</t>
+          <t>více parcel oddělených čárkou</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="n">
-        <v>47787</v>
+        <v>49904</v>
       </c>
       <c r="B15" t="inlineStr">
         <is>
@@ -975,22 +975,22 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Praha-východ</t>
+          <t>Hlavní město Praha</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>st. 1313</t>
+          <t>2114/5</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>Ládví</t>
+          <t>Krč</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>jednotka č. 24010022, byt v budově č.p. 2401, část obce Olešovice, na parcele st. 1313 Ládví (součástí je stavba č.p. 2401, čst obce Olešovice), podíl na společných částech domu a pozemku 458/4518</t>
+          <t>jednotka č. 15680103, garáž v budově č.p. 1570, 1568, 1569, část obce Krč, na parcele 2114/3 Krč, 2114/4 Krč, 2114/5 Krč, podíl na společných částech domu a pozemku 2230/184350</t>
         </is>
       </c>
       <c r="G15" t="n">
@@ -998,37 +998,37 @@
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>jednotka na parcele s prefixem st. + KU</t>
+          <t>více parcel oddělených čárkou</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="n">
-        <v>47786</v>
+        <v>39291</v>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>parcela</t>
+          <t>jednotka</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Praha-východ</t>
+          <t>Hlavní město Praha</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>634/4</t>
+          <t>2715/2</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>Ládví</t>
+          <t>Dejvice</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>č. 634/4 Ládví</t>
+          <t>jednotka č. 28220301, garáž v budově č.p. 2822, část obce Dejvice, na parcele 2715/2 Dejvice (součástí je stavba č.p. 2822, čst obce Dejvice), 2715/96 Dejvice, 2715/97 Dejvice, podíl na společných částech domu a pozemku 21306/116531</t>
         </is>
       </c>
       <c r="G16" t="n">
@@ -1036,37 +1036,37 @@
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>číslo a KU za ním</t>
+          <t>jednotka na parcele bez prefixu st. + KU</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="n">
-        <v>47785</v>
+        <v>39291</v>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>parcela</t>
+          <t>jednotka</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Praha-východ</t>
+          <t>Hlavní město Praha</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>634/5</t>
+          <t>2715/96</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>Ládví</t>
+          <t>Dejvice</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>č. 634/5 Ládví</t>
+          <t>jednotka č. 28220301, garáž v budově č.p. 2822, část obce Dejvice, na parcele 2715/2 Dejvice (součástí je stavba č.p. 2822, čst obce Dejvice), 2715/96 Dejvice, 2715/97 Dejvice, podíl na společných částech domu a pozemku 21306/116531</t>
         </is>
       </c>
       <c r="G17" t="n">
@@ -1074,37 +1074,37 @@
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>číslo a KU za ním</t>
+          <t>více parcel oddělených čárkou</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="n">
-        <v>47784</v>
+        <v>39291</v>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>parcela</t>
+          <t>jednotka</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Praha-východ</t>
+          <t>Hlavní město Praha</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>328/91</t>
+          <t>2715/97</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>Ládví</t>
+          <t>Dejvice</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>č. 328/91 Ládví</t>
+          <t>jednotka č. 28220301, garáž v budově č.p. 2822, část obce Dejvice, na parcele 2715/2 Dejvice (součástí je stavba č.p. 2822, čst obce Dejvice), 2715/96 Dejvice, 2715/97 Dejvice, podíl na společných částech domu a pozemku 21306/116531</t>
         </is>
       </c>
       <c r="G18" t="n">
@@ -1112,37 +1112,37 @@
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>číslo a KU za ním</t>
+          <t>více parcel oddělených čárkou</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="n">
-        <v>47783</v>
+        <v>37308</v>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>parcela</t>
+          <t>jednotka</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>Praha-východ</t>
+          <t>Hlavní město Praha</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>328/143</t>
+          <t>580/5</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>Ládví</t>
+          <t>Holešovice</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>č. 328/143 Ládví</t>
+          <t>jednotka č. 16320038, garáž v budově č.p. 1632, část obce Holešovice, na parcele 580/5 Holešovice, 581 Holešovice (součástí je stavba č.p. 1632, čst obce Holešovice), podíl na společných částech domu a pozemku 24385/139693</t>
         </is>
       </c>
       <c r="G19" t="n">
@@ -1150,37 +1150,37 @@
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>číslo a KU za ním</t>
+          <t>jednotka na parcele bez prefixu st. + KU</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="n">
-        <v>47782</v>
+        <v>37308</v>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>parcela</t>
+          <t>jednotka</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>Praha-východ</t>
+          <t>Hlavní město Praha</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>414/49</t>
+          <t>581</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>Ládví</t>
+          <t>Holešovice</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>č. 414/49 Ládví</t>
+          <t>jednotka č. 16320038, garáž v budově č.p. 1632, část obce Holešovice, na parcele 580/5 Holešovice, 581 Holešovice (součástí je stavba č.p. 1632, čst obce Holešovice), podíl na společných částech domu a pozemku 24385/139693</t>
         </is>
       </c>
       <c r="G20" t="n">
@@ -1188,37 +1188,37 @@
       </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t>číslo a KU za ním</t>
+          <t>více parcel oddělených čárkou</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="n">
-        <v>47781</v>
+        <v>36099</v>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>parcela</t>
+          <t>jednotka</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>Praha-východ</t>
+          <t>Hlavní město Praha</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>414/48</t>
+          <t>160/423</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>Ládví</t>
+          <t>Stodůlky</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>č. 414/48 Ládví</t>
+          <t>jednotka č. 28180010, garáž v budově č.p. 2818, část obce Stodůlky, na parcele 160/423 Stodůlky, podíl na společných částech domu a pozemku 24784/119926</t>
         </is>
       </c>
       <c r="G21" t="n">
@@ -1226,37 +1226,37 @@
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>číslo a KU za ním</t>
+          <t>jednotka na parcele bez prefixu st. + KU</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="n">
-        <v>47780</v>
+        <v>35956</v>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>budova</t>
+          <t>jednotka</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>Praha-východ</t>
+          <t>Hlavní město Praha</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>st. 1294</t>
+          <t>2780/217</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>Ládví</t>
+          <t>Stodůlky</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>stavební č. 1294 Ládví (součástí je stavba budova bez čp/če, garáž)</t>
+          <t>jednotka č. 25480013, garáž v budově č.p. 2548, část obce Stodůlky, na parcele 2780/217 Stodůlky, podíl na společných částech domu a pozemku 2779/628880</t>
         </is>
       </c>
       <c r="G22" t="n">
@@ -1264,37 +1264,37 @@
       </c>
       <c r="H22" t="inlineStr">
         <is>
-          <t>č. + KU</t>
+          <t>jednotka na parcele bez prefixu st. + KU</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="n">
-        <v>47779</v>
+        <v>35418</v>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>parcela</t>
+          <t>jednotka</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>Praha-východ</t>
+          <t>Hlavní město Praha</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>95/15</t>
+          <t>2780/217</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>Ládví</t>
+          <t>Stodůlky</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>č. 95/15 Ládví</t>
+          <t>jednotka č. 25480036, garáž v budově č.p. 2548, část obce Stodůlky, na parcele 2780/217 Stodůlky, podíl na společných částech domu a pozemku 2779/628880</t>
         </is>
       </c>
       <c r="G23" t="n">
@@ -1302,37 +1302,37 @@
       </c>
       <c r="H23" t="inlineStr">
         <is>
-          <t>číslo a KU za ním</t>
+          <t>jednotka na parcele bez prefixu st. + KU</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="n">
-        <v>47778</v>
+        <v>33434</v>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>parcela</t>
+          <t>jednotka</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>Praha-východ</t>
+          <t>Hlavní město Praha</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>96/5</t>
+          <t>580/5</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>Ládví</t>
+          <t>Holešovice</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>č. 96/5 Ládví</t>
+          <t>jednotka č. 16320038, garáž v budově č.p. 1632, část obce Holešovice, na parcele 580/5 Holešovice, 581 Holešovice (součástí je stavba č.p. 1632, čst obce Holešovice), podíl na společných částech domu a pozemku 24385/139693</t>
         </is>
       </c>
       <c r="G24" t="n">
@@ -1340,37 +1340,37 @@
       </c>
       <c r="H24" t="inlineStr">
         <is>
-          <t>číslo a KU za ním</t>
+          <t>jednotka na parcele bez prefixu st. + KU</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="n">
-        <v>47777</v>
+        <v>33434</v>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>parcela</t>
+          <t>jednotka</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>Praha-východ</t>
+          <t>Hlavní město Praha</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>97/10</t>
+          <t>581</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>Ládví</t>
+          <t>Holešovice</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>č. 97/10 Ládví</t>
+          <t>jednotka č. 16320038, garáž v budově č.p. 1632, část obce Holešovice, na parcele 580/5 Holešovice, 581 Holešovice (součástí je stavba č.p. 1632, čst obce Holešovice), podíl na společných částech domu a pozemku 24385/139693</t>
         </is>
       </c>
       <c r="G25" t="n">
@@ -1378,37 +1378,37 @@
       </c>
       <c r="H25" t="inlineStr">
         <is>
-          <t>číslo a KU za ním</t>
+          <t>více parcel oddělených čárkou</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="n">
-        <v>47776</v>
+        <v>33430</v>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>budova</t>
+          <t>jednotka</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>Praha-východ</t>
+          <t>Hlavní město Praha</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>st. 1315</t>
+          <t>580/5</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>Ládví</t>
+          <t>Holešovice</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>stavební č. 1315 Ládví (součástí je stavba č.p. 2132, čst obce Ládví)</t>
+          <t>jednotka č. 16320038, garáž v budově č.p. 1632, část obce Holešovice, na parcele 580/5 Holešovice, 581 Holešovice (součástí je stavba č.p. 1632, čst obce Holešovice), podíl na společných částech domu a pozemku 24385/139693</t>
         </is>
       </c>
       <c r="G26" t="n">
@@ -1416,37 +1416,37 @@
       </c>
       <c r="H26" t="inlineStr">
         <is>
-          <t>č. + KU</t>
+          <t>jednotka na parcele bez prefixu st. + KU</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="n">
-        <v>47775</v>
+        <v>33430</v>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>parcela</t>
+          <t>jednotka</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>Praha-východ</t>
+          <t>Hlavní město Praha</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>511/4</t>
+          <t>581</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>Ládví</t>
+          <t>Holešovice</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>č. 511/4 Ládví</t>
+          <t>jednotka č. 16320038, garáž v budově č.p. 1632, část obce Holešovice, na parcele 580/5 Holešovice, 581 Holešovice (součástí je stavba č.p. 1632, čst obce Holešovice), podíl na společných částech domu a pozemku 24385/139693</t>
         </is>
       </c>
       <c r="G27" t="n">
@@ -1454,37 +1454,37 @@
       </c>
       <c r="H27" t="inlineStr">
         <is>
-          <t>číslo a KU za ním</t>
+          <t>více parcel oddělených čárkou</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="n">
-        <v>47774</v>
+        <v>33351</v>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>parcela</t>
+          <t>jednotka</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>Praha-východ</t>
+          <t>Hlavní město Praha</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>103/17</t>
+          <t>580/5</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>Ládví</t>
+          <t>Holešovice</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>č. 103/17 Ládví</t>
+          <t>jednotka č. 16320038, garáž v budově č.p. 1632, část obce Holešovice, na parcele 580/5 Holešovice, 581 Holešovice (součástí je stavba č.p. 1632, čst obce Holešovice), podíl na společných částech domu a pozemku 24385/139693</t>
         </is>
       </c>
       <c r="G28" t="n">
@@ -1492,37 +1492,37 @@
       </c>
       <c r="H28" t="inlineStr">
         <is>
-          <t>číslo a KU za ním</t>
+          <t>jednotka na parcele bez prefixu st. + KU</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="n">
-        <v>47773</v>
+        <v>33351</v>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>parcela</t>
+          <t>jednotka</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>Praha-východ</t>
+          <t>Hlavní město Praha</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>27/10</t>
+          <t>581</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>Ládví</t>
+          <t>Holešovice</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>č. 27/10 Ládví</t>
+          <t>jednotka č. 16320038, garáž v budově č.p. 1632, část obce Holešovice, na parcele 580/5 Holešovice, 581 Holešovice (součástí je stavba č.p. 1632, čst obce Holešovice), podíl na společných částech domu a pozemku 24385/139693</t>
         </is>
       </c>
       <c r="G29" t="n">
@@ -1530,37 +1530,37 @@
       </c>
       <c r="H29" t="inlineStr">
         <is>
-          <t>číslo a KU za ním</t>
+          <t>více parcel oddělených čárkou</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="n">
-        <v>47772</v>
+        <v>33337</v>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>parcela</t>
+          <t>jednotka</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>Praha-východ</t>
+          <t>Hlavní město Praha</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>103/16</t>
+          <t>954</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>Ládví</t>
+          <t>Holešovice</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>č. 103/16 Ládví</t>
+          <t>jednotka č. 16330902, garáž v budově č.p. 1633, část obce Holešovice, na parcele 954 Holešovice (součástí je stavba č.p. 1633, čst obce Holešovice), podíl na společných částech domu a pozemku 28655/130700</t>
         </is>
       </c>
       <c r="G30" t="n">
@@ -1568,37 +1568,37 @@
       </c>
       <c r="H30" t="inlineStr">
         <is>
-          <t>číslo a KU za ním</t>
+          <t>jednotka na parcele bez prefixu st. + KU</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="n">
-        <v>47771</v>
+        <v>33268</v>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>parcela</t>
+          <t>jednotka</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>Praha-východ</t>
+          <t>Hlavní město Praha</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>103/12</t>
+          <t>580/5</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>Ládví</t>
+          <t>Holešovice</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>č. 103/12 Ládví</t>
+          <t>jednotka č. 16320038, garáž v budově č.p. 1632, část obce Holešovice, na parcele 580/5 Holešovice, 581 Holešovice (součástí je stavba č.p. 1632, čst obce Holešovice), podíl na společných částech domu a pozemku 24385/139693</t>
         </is>
       </c>
       <c r="G31" t="n">
@@ -1606,37 +1606,37 @@
       </c>
       <c r="H31" t="inlineStr">
         <is>
-          <t>číslo a KU za ním</t>
+          <t>jednotka na parcele bez prefixu st. + KU</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="n">
-        <v>47770</v>
+        <v>33268</v>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>parcela</t>
+          <t>jednotka</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>Praha-východ</t>
+          <t>Hlavní město Praha</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>102/8</t>
+          <t>581</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>Ládví</t>
+          <t>Holešovice</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>č. 102/8 Ládví</t>
+          <t>jednotka č. 16320038, garáž v budově č.p. 1632, část obce Holešovice, na parcele 580/5 Holešovice, 581 Holešovice (součástí je stavba č.p. 1632, čst obce Holešovice), podíl na společných částech domu a pozemku 24385/139693</t>
         </is>
       </c>
       <c r="G32" t="n">
@@ -1644,37 +1644,37 @@
       </c>
       <c r="H32" t="inlineStr">
         <is>
-          <t>číslo a KU za ním</t>
+          <t>více parcel oddělených čárkou</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="n">
-        <v>47769</v>
+        <v>33201</v>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>parcela</t>
+          <t>jednotka</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>Praha-východ</t>
+          <t>Hlavní město Praha</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>103/10</t>
+          <t>580/5</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>Ládví</t>
+          <t>Holešovice</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>č. 103/10 Ládví</t>
+          <t>jednotka č. 16320038, garáž v budově č.p. 1632, část obce Holešovice, na parcele 580/5 Holešovice, 581 Holešovice (součástí je stavba č.p. 1632, čst obce Holešovice), podíl na společných částech domu a pozemku 24385/139693</t>
         </is>
       </c>
       <c r="G33" t="n">
@@ -1682,37 +1682,37 @@
       </c>
       <c r="H33" t="inlineStr">
         <is>
-          <t>číslo a KU za ním</t>
+          <t>jednotka na parcele bez prefixu st. + KU</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="n">
-        <v>47768</v>
+        <v>33201</v>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>parcela</t>
+          <t>jednotka</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>Praha-východ</t>
+          <t>Hlavní město Praha</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>103/13</t>
+          <t>581</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>Ládví</t>
+          <t>Holešovice</t>
         </is>
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>č. 103/13 Ládví</t>
+          <t>jednotka č. 16320038, garáž v budově č.p. 1632, část obce Holešovice, na parcele 580/5 Holešovice, 581 Holešovice (součástí je stavba č.p. 1632, čst obce Holešovice), podíl na společných částech domu a pozemku 24385/139693</t>
         </is>
       </c>
       <c r="G34" t="n">
@@ -1720,13 +1720,13 @@
       </c>
       <c r="H34" t="inlineStr">
         <is>
-          <t>číslo a KU za ním</t>
+          <t>více parcel oddělených čárkou</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="n">
-        <v>47767</v>
+        <v>32934</v>
       </c>
       <c r="B35" t="inlineStr">
         <is>
@@ -1735,22 +1735,22 @@
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>Praha-východ</t>
+          <t>Hlavní město Praha</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>st. 118</t>
+          <t>734/1</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>Ládví</t>
+          <t>Holešovice</t>
         </is>
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>jednotka č. 11480029, byt v budově č.p. 1148, část obce Ládví, na parcele st. 118 Ládví, podíl na společných částech domu a pozemku 732/32916</t>
+          <t>jednotka č. 8690341, garáž v budově č.p. 869, část obce Holešovice, na parcele 734/1 Holešovice, podíl na společných částech domu a pozemku 2450/197252</t>
         </is>
       </c>
       <c r="G35" t="n">
@@ -1758,37 +1758,37 @@
       </c>
       <c r="H35" t="inlineStr">
         <is>
-          <t>jednotka na parcele s prefixem st. + KU</t>
+          <t>jednotka na parcele bez prefixu st. + KU</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="n">
-        <v>47766</v>
+        <v>31596</v>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>parcela</t>
+          <t>jednotka</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>Praha-východ</t>
+          <t>Hlavní město Praha</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>364/36</t>
+          <t>1061/92</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>Ládví</t>
+          <t>Liboc</t>
         </is>
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>č. 364/36 Ládví</t>
+          <t>jednotka č. 6260342, garáž v budově č.p. 626, část obce Liboc, na parcele 1061/92 Liboc, 1061/153 Liboc, 1061/156 Liboc, podíl na společných částech domu a pozemku 201/31365</t>
         </is>
       </c>
       <c r="G36" t="n">
@@ -1796,37 +1796,37 @@
       </c>
       <c r="H36" t="inlineStr">
         <is>
-          <t>číslo a KU za ním</t>
+          <t>jednotka na parcele bez prefixu st. + KU</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="n">
-        <v>47765</v>
+        <v>31596</v>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>parcela</t>
+          <t>jednotka</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>Praha-východ</t>
+          <t>Hlavní město Praha</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>798</t>
+          <t>1061/153</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>Ládví</t>
+          <t>Liboc</t>
         </is>
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>č. 798 Ládví</t>
+          <t>jednotka č. 6260342, garáž v budově č.p. 626, část obce Liboc, na parcele 1061/92 Liboc, 1061/153 Liboc, 1061/156 Liboc, podíl na společných částech domu a pozemku 201/31365</t>
         </is>
       </c>
       <c r="G37" t="n">
@@ -1834,37 +1834,37 @@
       </c>
       <c r="H37" t="inlineStr">
         <is>
-          <t>číslo a KU za ním</t>
+          <t>více parcel oddělených čárkou</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="n">
-        <v>47764</v>
+        <v>31596</v>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>parcela</t>
+          <t>jednotka</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>Praha-východ</t>
+          <t>Hlavní město Praha</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>618/9</t>
+          <t>1061/156</t>
         </is>
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>Ládví</t>
+          <t>Liboc</t>
         </is>
       </c>
       <c r="F38" t="inlineStr">
         <is>
-          <t>č. 618/9 Ládví</t>
+          <t>jednotka č. 6260342, garáž v budově č.p. 626, část obce Liboc, na parcele 1061/92 Liboc, 1061/153 Liboc, 1061/156 Liboc, podíl na společných částech domu a pozemku 201/31365</t>
         </is>
       </c>
       <c r="G38" t="n">
@@ -1872,37 +1872,37 @@
       </c>
       <c r="H38" t="inlineStr">
         <is>
-          <t>číslo a KU za ním</t>
+          <t>více parcel oddělených čárkou</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="n">
-        <v>47763</v>
+        <v>31344</v>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>budova</t>
+          <t>jednotka</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>Praha-východ</t>
+          <t>Hlavní město Praha</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>st. 931</t>
+          <t>1818/396</t>
         </is>
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>Ládví</t>
+          <t>Hostivař</t>
         </is>
       </c>
       <c r="F39" t="inlineStr">
         <is>
-          <t>stavební č. 931 Ládví (součástí je stavba č.p. 1434, čst obce Olešovice)</t>
+          <t>jednotka č. 15860205, garáž v budově č.p. 1586, část obce Hostivař, na parcele 1818/396 Hostivař (součástí je stavba č.p. 1586, čst obce Hostivař), podíl na společných částech domu a pozemku 27680/89507</t>
         </is>
       </c>
       <c r="G39" t="n">
@@ -1910,37 +1910,37 @@
       </c>
       <c r="H39" t="inlineStr">
         <is>
-          <t>č. + KU</t>
+          <t>jednotka na parcele bez prefixu st. + KU</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="n">
-        <v>47762</v>
+        <v>30501</v>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>parcela</t>
+          <t>jednotka</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>Praha-východ</t>
+          <t>Hlavní město Praha</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>578/3</t>
+          <t>1818/375</t>
         </is>
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>Ládví</t>
+          <t>Hostivař</t>
         </is>
       </c>
       <c r="F40" t="inlineStr">
         <is>
-          <t>č. 578/3 Ládví</t>
+          <t>jednotka č. 15800317, garáž v budově č.p. 1580, část obce Hostivař, na parcele 1818/375 Hostivař, 1818/376 Hostivař, 1818/377 Hostivař (součástí je stavba č.p. 1580, čst obce Hostivař), podíl na společných částech domu a pozemku 28543/155716</t>
         </is>
       </c>
       <c r="G40" t="n">
@@ -1948,37 +1948,37 @@
       </c>
       <c r="H40" t="inlineStr">
         <is>
-          <t>číslo a KU za ním</t>
+          <t>jednotka na parcele bez prefixu st. + KU</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="n">
-        <v>47761</v>
+        <v>30501</v>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>parcela</t>
+          <t>jednotka</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>Praha-východ</t>
+          <t>Hlavní město Praha</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>578/2</t>
+          <t>1818/376</t>
         </is>
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>Ládví</t>
+          <t>Hostivař</t>
         </is>
       </c>
       <c r="F41" t="inlineStr">
         <is>
-          <t>č. 578/2 Ládví</t>
+          <t>jednotka č. 15800317, garáž v budově č.p. 1580, část obce Hostivař, na parcele 1818/375 Hostivař, 1818/376 Hostivař, 1818/377 Hostivař (součástí je stavba č.p. 1580, čst obce Hostivař), podíl na společných částech domu a pozemku 28543/155716</t>
         </is>
       </c>
       <c r="G41" t="n">
@@ -1986,37 +1986,37 @@
       </c>
       <c r="H41" t="inlineStr">
         <is>
-          <t>číslo a KU za ním</t>
+          <t>více parcel oddělených čárkou</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="n">
-        <v>47760</v>
+        <v>30501</v>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>parcela</t>
+          <t>jednotka</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>Praha-východ</t>
+          <t>Hlavní město Praha</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>578/1</t>
+          <t>1818/377</t>
         </is>
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>Ládví</t>
+          <t>Hostivař</t>
         </is>
       </c>
       <c r="F42" t="inlineStr">
         <is>
-          <t>č. 578/1 Ládví</t>
+          <t>jednotka č. 15800317, garáž v budově č.p. 1580, část obce Hostivař, na parcele 1818/375 Hostivař, 1818/376 Hostivař, 1818/377 Hostivař (součástí je stavba č.p. 1580, čst obce Hostivař), podíl na společných částech domu a pozemku 28543/155716</t>
         </is>
       </c>
       <c r="G42" t="n">
@@ -2024,37 +2024,37 @@
       </c>
       <c r="H42" t="inlineStr">
         <is>
-          <t>číslo a KU za ním</t>
+          <t>více parcel oddělených čárkou</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="n">
-        <v>47759</v>
+        <v>25660</v>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>parcela</t>
+          <t>jednotka</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>Praha-východ</t>
+          <t>Hlavní město Praha</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>340/1</t>
+          <t>110/1</t>
         </is>
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>Ládví</t>
+          <t>Štěrboholy</t>
         </is>
       </c>
       <c r="F43" t="inlineStr">
         <is>
-          <t>č. 340/1 Ládví</t>
+          <t>jednotka č. 5900100, garáž v budově č.p. 590, část obce Štěrboholy, na parcele 110/1 Štěrboholy (součástí je stavba č.p. 590, čst obce Štěrboholy), podíl na společných částech domu a pozemku 27468/80987</t>
         </is>
       </c>
       <c r="G43" t="n">
@@ -2062,37 +2062,37 @@
       </c>
       <c r="H43" t="inlineStr">
         <is>
-          <t>číslo a KU za ním</t>
+          <t>jednotka na parcele bez prefixu st. + KU</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="n">
-        <v>47758</v>
+        <v>21331</v>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>parcela</t>
+          <t>jednotka</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>Praha-východ</t>
+          <t>Hlavní město Praha</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>432/9</t>
+          <t>527</t>
         </is>
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>Ládví</t>
+          <t>Smíchov</t>
         </is>
       </c>
       <c r="F44" t="inlineStr">
         <is>
-          <t>č. 432/9 Ládví</t>
+          <t>jednotka č. 4940102, garáž v budově č.p. 494, část obce Smíchov, na parcele 527 Smíchov (součástí je stavba č.p. 494, čst obce Smíchov), podíl na společných částech domu a pozemku 283/31473</t>
         </is>
       </c>
       <c r="G44" t="n">
@@ -2100,37 +2100,37 @@
       </c>
       <c r="H44" t="inlineStr">
         <is>
-          <t>číslo a KU za ním</t>
+          <t>jednotka na parcele bez prefixu st. + KU</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="n">
-        <v>47757</v>
+        <v>19260</v>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>parcela</t>
+          <t>jednotka</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>Praha-východ</t>
+          <t>Hlavní město Praha</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>432/8</t>
+          <t>46/6</t>
         </is>
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>Ládví</t>
+          <t>Cholupice</t>
         </is>
       </c>
       <c r="F45" t="inlineStr">
         <is>
-          <t>č. 432/8 Ládví</t>
+          <t>jednotka č. 1340101, garáž v budově č.p. 134, část obce Cholupice, na parcele 46/6 Cholupice, podíl na společných částech domu a pozemku 26236/37916</t>
         </is>
       </c>
       <c r="G45" t="n">
@@ -2138,37 +2138,37 @@
       </c>
       <c r="H45" t="inlineStr">
         <is>
-          <t>číslo a KU za ním</t>
+          <t>jednotka na parcele bez prefixu st. + KU</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="n">
-        <v>47756</v>
+        <v>19136</v>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>parcela</t>
+          <t>jednotka</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>Praha-východ</t>
+          <t>Hlavní město Praha</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>430/2</t>
+          <t>2715/2</t>
         </is>
       </c>
       <c r="E46" t="inlineStr">
         <is>
-          <t>Ládví</t>
+          <t>Dejvice</t>
         </is>
       </c>
       <c r="F46" t="inlineStr">
         <is>
-          <t>č. 430/2 Ládví</t>
+          <t>jednotka č. 28220301, garáž v budově č.p. 2822, část obce Dejvice, na parcele 2715/2 Dejvice (součástí je stavba č.p. 2822, čst obce Dejvice), 2715/96 Dejvice, 2715/97 Dejvice, podíl na společných částech domu a pozemku 21306/116531</t>
         </is>
       </c>
       <c r="G46" t="n">
@@ -2176,37 +2176,37 @@
       </c>
       <c r="H46" t="inlineStr">
         <is>
-          <t>číslo a KU za ním</t>
+          <t>jednotka na parcele bez prefixu st. + KU</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="n">
-        <v>47755</v>
+        <v>19136</v>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>parcela</t>
+          <t>jednotka</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>Praha-východ</t>
+          <t>Hlavní město Praha</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>459/9</t>
+          <t>2715/96</t>
         </is>
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t>Ládví</t>
+          <t>Dejvice</t>
         </is>
       </c>
       <c r="F47" t="inlineStr">
         <is>
-          <t>č. 459/9 Ládví</t>
+          <t>jednotka č. 28220301, garáž v budově č.p. 2822, část obce Dejvice, na parcele 2715/2 Dejvice (součástí je stavba č.p. 2822, čst obce Dejvice), 2715/96 Dejvice, 2715/97 Dejvice, podíl na společných částech domu a pozemku 21306/116531</t>
         </is>
       </c>
       <c r="G47" t="n">
@@ -2214,37 +2214,37 @@
       </c>
       <c r="H47" t="inlineStr">
         <is>
-          <t>číslo a KU za ním</t>
+          <t>více parcel oddělených čárkou</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="n">
-        <v>47754</v>
+        <v>19136</v>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>budova</t>
+          <t>jednotka</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>Praha-východ</t>
+          <t>Hlavní město Praha</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>st. 1186</t>
+          <t>2715/97</t>
         </is>
       </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t>Ládví</t>
+          <t>Dejvice</t>
         </is>
       </c>
       <c r="F48" t="inlineStr">
         <is>
-          <t>stavební č. 1186 Ládví (součástí je stavba budova bez čp/če, jiná stavba)</t>
+          <t>jednotka č. 28220301, garáž v budově č.p. 2822, část obce Dejvice, na parcele 2715/2 Dejvice (součástí je stavba č.p. 2822, čst obce Dejvice), 2715/96 Dejvice, 2715/97 Dejvice, podíl na společných částech domu a pozemku 21306/116531</t>
         </is>
       </c>
       <c r="G48" t="n">
@@ -2252,37 +2252,37 @@
       </c>
       <c r="H48" t="inlineStr">
         <is>
-          <t>č. + KU</t>
+          <t>více parcel oddělených čárkou</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="n">
-        <v>47753</v>
+        <v>17392</v>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>budova</t>
+          <t>jednotka</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>Praha-východ</t>
+          <t>Hlavní město Praha</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>st. 476</t>
+          <t>4817/5</t>
         </is>
       </c>
       <c r="E49" t="inlineStr">
         <is>
-          <t>Ládví</t>
+          <t>Modřany</t>
         </is>
       </c>
       <c r="F49" t="inlineStr">
         <is>
-          <t>stavební č. 476 Ládví (součástí je stavba č.e. 1424, čst obce Ládví)</t>
+          <t>jednotka č. 23900002, garáž v budově č.p. 2390, část obce Modřany, na parcele 4817/5 Modřany, 4825/9 Modřany (součástí je stavba č.p. 2390, čst obce Modřany), podíl na společných částech domu a pozemku 21507/227640</t>
         </is>
       </c>
       <c r="G49" t="n">
@@ -2290,37 +2290,37 @@
       </c>
       <c r="H49" t="inlineStr">
         <is>
-          <t>č. + KU</t>
+          <t>jednotka na parcele bez prefixu st. + KU</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="n">
-        <v>47752</v>
+        <v>17392</v>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>parcela</t>
+          <t>jednotka</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>Praha-východ</t>
+          <t>Hlavní město Praha</t>
         </is>
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>519/1</t>
+          <t>4825/9</t>
         </is>
       </c>
       <c r="E50" t="inlineStr">
         <is>
-          <t>Ládví</t>
+          <t>Modřany</t>
         </is>
       </c>
       <c r="F50" t="inlineStr">
         <is>
-          <t>č. 519/1 Ládví</t>
+          <t>jednotka č. 23900002, garáž v budově č.p. 2390, část obce Modřany, na parcele 4817/5 Modřany, 4825/9 Modřany (součástí je stavba č.p. 2390, čst obce Modřany), podíl na společných částech domu a pozemku 21507/227640</t>
         </is>
       </c>
       <c r="G50" t="n">
@@ -2328,37 +2328,37 @@
       </c>
       <c r="H50" t="inlineStr">
         <is>
-          <t>číslo a KU za ním</t>
+          <t>více parcel oddělených čárkou</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="n">
-        <v>47751</v>
+        <v>16986</v>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>budova</t>
+          <t>jednotka</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>Praha-východ</t>
+          <t>Hlavní město Praha</t>
         </is>
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>st. 128</t>
+          <t>2780/217</t>
         </is>
       </c>
       <c r="E51" t="inlineStr">
         <is>
-          <t>Ládví</t>
+          <t>Stodůlky</t>
         </is>
       </c>
       <c r="F51" t="inlineStr">
         <is>
-          <t>stavební č. 128 Ládví (součástí je stavba č.e. 1485, čst obce Ládví)</t>
+          <t>jednotka č. 25480162, garáž v budově č.p. 2548, část obce Stodůlky, na parcele 2780/217 Stodůlky, podíl na společných částech domu a pozemku 2779/628880</t>
         </is>
       </c>
       <c r="G51" t="n">
@@ -2366,7 +2366,767 @@
       </c>
       <c r="H51" t="inlineStr">
         <is>
-          <t>č. + KU</t>
+          <t>jednotka na parcele bez prefixu st. + KU</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="n">
+        <v>16435</v>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>jednotka</t>
+        </is>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>Hlavní město Praha</t>
+        </is>
+      </c>
+      <c r="D52" t="inlineStr">
+        <is>
+          <t>3448</t>
+        </is>
+      </c>
+      <c r="E52" t="inlineStr">
+        <is>
+          <t>Smíchov</t>
+        </is>
+      </c>
+      <c r="F52" t="inlineStr">
+        <is>
+          <t>jednotka č. 33810102, garáž v budově č.p. 3381, část obce Smíchov, na parcele 3448 Smíchov (součástí je stavba č.p. 3381, čst obce Smíchov), podíl na společných částech domu a pozemku 2946/19124</t>
+        </is>
+      </c>
+      <c r="G52" t="n">
+        <v>1</v>
+      </c>
+      <c r="H52" t="inlineStr">
+        <is>
+          <t>jednotka na parcele bez prefixu st. + KU</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="n">
+        <v>16373</v>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>jednotka</t>
+        </is>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>Hlavní město Praha</t>
+        </is>
+      </c>
+      <c r="D53" t="inlineStr">
+        <is>
+          <t>3448</t>
+        </is>
+      </c>
+      <c r="E53" t="inlineStr">
+        <is>
+          <t>Smíchov</t>
+        </is>
+      </c>
+      <c r="F53" t="inlineStr">
+        <is>
+          <t>jednotka č. 33810102, garáž v budově č.p. 3381, část obce Smíchov, na parcele 3448 Smíchov (součástí je stavba č.p. 3381, čst obce Smíchov), podíl na společných částech domu a pozemku 2946/19124</t>
+        </is>
+      </c>
+      <c r="G53" t="n">
+        <v>1</v>
+      </c>
+      <c r="H53" t="inlineStr">
+        <is>
+          <t>jednotka na parcele bez prefixu st. + KU</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="n">
+        <v>16331</v>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>jednotka</t>
+        </is>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>Hlavní město Praha</t>
+        </is>
+      </c>
+      <c r="D54" t="inlineStr">
+        <is>
+          <t>3109/20</t>
+        </is>
+      </c>
+      <c r="E54" t="inlineStr">
+        <is>
+          <t>Smíchov</t>
+        </is>
+      </c>
+      <c r="F54" t="inlineStr">
+        <is>
+          <t>jednotka č. 33540101, garáž v budově č.p. 3354, část obce Smíchov, na parcele 3109/20 Smíchov (součástí je stavba č.p. 3354, čst obce Smíchov), podíl na společných částech domu a pozemku 21600/76084</t>
+        </is>
+      </c>
+      <c r="G54" t="n">
+        <v>1</v>
+      </c>
+      <c r="H54" t="inlineStr">
+        <is>
+          <t>jednotka na parcele bez prefixu st. + KU</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="n">
+        <v>14903</v>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>jednotka</t>
+        </is>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>Hlavní město Praha</t>
+        </is>
+      </c>
+      <c r="D55" t="inlineStr">
+        <is>
+          <t>4817/5</t>
+        </is>
+      </c>
+      <c r="E55" t="inlineStr">
+        <is>
+          <t>Modřany</t>
+        </is>
+      </c>
+      <c r="F55" t="inlineStr">
+        <is>
+          <t>jednotka č. 23900002, garáž v budově č.p. 2390, část obce Modřany, na parcele 4817/5 Modřany, 4825/9 Modřany (součástí je stavba č.p. 2390, čst obce Modřany), podíl na společných částech domu a pozemku 21507/227640</t>
+        </is>
+      </c>
+      <c r="G55" t="n">
+        <v>1</v>
+      </c>
+      <c r="H55" t="inlineStr">
+        <is>
+          <t>jednotka na parcele bez prefixu st. + KU</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="n">
+        <v>14903</v>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>jednotka</t>
+        </is>
+      </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>Hlavní město Praha</t>
+        </is>
+      </c>
+      <c r="D56" t="inlineStr">
+        <is>
+          <t>4825/9</t>
+        </is>
+      </c>
+      <c r="E56" t="inlineStr">
+        <is>
+          <t>Modřany</t>
+        </is>
+      </c>
+      <c r="F56" t="inlineStr">
+        <is>
+          <t>jednotka č. 23900002, garáž v budově č.p. 2390, část obce Modřany, na parcele 4817/5 Modřany, 4825/9 Modřany (součástí je stavba č.p. 2390, čst obce Modřany), podíl na společných částech domu a pozemku 21507/227640</t>
+        </is>
+      </c>
+      <c r="G56" t="n">
+        <v>1</v>
+      </c>
+      <c r="H56" t="inlineStr">
+        <is>
+          <t>více parcel oddělených čárkou</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="n">
+        <v>13623</v>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>jednotka</t>
+        </is>
+      </c>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>Hlavní město Praha</t>
+        </is>
+      </c>
+      <c r="D57" t="inlineStr">
+        <is>
+          <t>3109/20</t>
+        </is>
+      </c>
+      <c r="E57" t="inlineStr">
+        <is>
+          <t>Smíchov</t>
+        </is>
+      </c>
+      <c r="F57" t="inlineStr">
+        <is>
+          <t>jednotka č. 33540101, garáž v budově č.p. 3354, část obce Smíchov, na parcele 3109/20 Smíchov (součástí je stavba č.p. 3354, čst obce Smíchov), podíl na společných částech domu a pozemku 21600/76084</t>
+        </is>
+      </c>
+      <c r="G57" t="n">
+        <v>1</v>
+      </c>
+      <c r="H57" t="inlineStr">
+        <is>
+          <t>jednotka na parcele bez prefixu st. + KU</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="n">
+        <v>12849</v>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>jednotka</t>
+        </is>
+      </c>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>Hlavní město Praha</t>
+        </is>
+      </c>
+      <c r="D58" t="inlineStr">
+        <is>
+          <t>2780/217</t>
+        </is>
+      </c>
+      <c r="E58" t="inlineStr">
+        <is>
+          <t>Stodůlky</t>
+        </is>
+      </c>
+      <c r="F58" t="inlineStr">
+        <is>
+          <t>jednotka č. 25480082, garáž v budově č.p. 2548, část obce Stodůlky, na parcele 2780/217 Stodůlky, podíl na společných částech domu a pozemku 2779/628880</t>
+        </is>
+      </c>
+      <c r="G58" t="n">
+        <v>1</v>
+      </c>
+      <c r="H58" t="inlineStr">
+        <is>
+          <t>jednotka na parcele bez prefixu st. + KU</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="n">
+        <v>12839</v>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>jednotka</t>
+        </is>
+      </c>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>Hlavní město Praha</t>
+        </is>
+      </c>
+      <c r="D59" t="inlineStr">
+        <is>
+          <t>2780/217</t>
+        </is>
+      </c>
+      <c r="E59" t="inlineStr">
+        <is>
+          <t>Stodůlky</t>
+        </is>
+      </c>
+      <c r="F59" t="inlineStr">
+        <is>
+          <t>jednotka č. 25480066, garáž v budově č.p. 2548, část obce Stodůlky, na parcele 2780/217 Stodůlky, podíl na společných částech domu a pozemku 2779/628880</t>
+        </is>
+      </c>
+      <c r="G59" t="n">
+        <v>1</v>
+      </c>
+      <c r="H59" t="inlineStr">
+        <is>
+          <t>jednotka na parcele bez prefixu st. + KU</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="n">
+        <v>12708</v>
+      </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>jednotka</t>
+        </is>
+      </c>
+      <c r="C60" t="inlineStr">
+        <is>
+          <t>Hlavní město Praha</t>
+        </is>
+      </c>
+      <c r="D60" t="inlineStr">
+        <is>
+          <t>1061/91</t>
+        </is>
+      </c>
+      <c r="E60" t="inlineStr">
+        <is>
+          <t>Liboc</t>
+        </is>
+      </c>
+      <c r="F60" t="inlineStr">
+        <is>
+          <t>jednotka č. 6270201, garáž v budově č.p. 627, část obce Liboc, na parcele 1061/91 Liboc, podíl na společných částech domu a pozemku 2073/328428</t>
+        </is>
+      </c>
+      <c r="G60" t="n">
+        <v>1</v>
+      </c>
+      <c r="H60" t="inlineStr">
+        <is>
+          <t>jednotka na parcele bez prefixu st. + KU</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="n">
+        <v>11783</v>
+      </c>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>jednotka</t>
+        </is>
+      </c>
+      <c r="C61" t="inlineStr">
+        <is>
+          <t>Hlavní město Praha</t>
+        </is>
+      </c>
+      <c r="D61" t="inlineStr">
+        <is>
+          <t>3109/20</t>
+        </is>
+      </c>
+      <c r="E61" t="inlineStr">
+        <is>
+          <t>Smíchov</t>
+        </is>
+      </c>
+      <c r="F61" t="inlineStr">
+        <is>
+          <t>jednotka č. 33540101, garáž v budově č.p. 3354, část obce Smíchov, na parcele 3109/20 Smíchov (součástí je stavba č.p. 3354, čst obce Smíchov), podíl na společných částech domu a pozemku 21600/76084</t>
+        </is>
+      </c>
+      <c r="G61" t="n">
+        <v>1</v>
+      </c>
+      <c r="H61" t="inlineStr">
+        <is>
+          <t>jednotka na parcele bez prefixu st. + KU</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="n">
+        <v>11710</v>
+      </c>
+      <c r="B62" t="inlineStr">
+        <is>
+          <t>jednotka</t>
+        </is>
+      </c>
+      <c r="C62" t="inlineStr">
+        <is>
+          <t>Hlavní město Praha</t>
+        </is>
+      </c>
+      <c r="D62" t="inlineStr">
+        <is>
+          <t>3109/20</t>
+        </is>
+      </c>
+      <c r="E62" t="inlineStr">
+        <is>
+          <t>Smíchov</t>
+        </is>
+      </c>
+      <c r="F62" t="inlineStr">
+        <is>
+          <t>jednotka č. 33540101, garáž v budově č.p. 3354, část obce Smíchov, na parcele 3109/20 Smíchov (součástí je stavba č.p. 3354, čst obce Smíchov), podíl na společných částech domu a pozemku 21600/76084</t>
+        </is>
+      </c>
+      <c r="G62" t="n">
+        <v>1</v>
+      </c>
+      <c r="H62" t="inlineStr">
+        <is>
+          <t>jednotka na parcele bez prefixu st. + KU</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="n">
+        <v>10936</v>
+      </c>
+      <c r="B63" t="inlineStr">
+        <is>
+          <t>jednotka</t>
+        </is>
+      </c>
+      <c r="C63" t="inlineStr">
+        <is>
+          <t>Hlavní město Praha</t>
+        </is>
+      </c>
+      <c r="D63" t="inlineStr">
+        <is>
+          <t>3443</t>
+        </is>
+      </c>
+      <c r="E63" t="inlineStr">
+        <is>
+          <t>Smíchov</t>
+        </is>
+      </c>
+      <c r="F63" t="inlineStr">
+        <is>
+          <t>jednotka č. 33310101, garáž v budově č.p. 3331, část obce Smíchov, na parcele 3443 Smíchov (součástí je stavba č.p. 3331, čst obce Smíchov), podíl na společných částech domu a pozemku 29648/145749</t>
+        </is>
+      </c>
+      <c r="G63" t="n">
+        <v>1</v>
+      </c>
+      <c r="H63" t="inlineStr">
+        <is>
+          <t>jednotka na parcele bez prefixu st. + KU</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="n">
+        <v>10672</v>
+      </c>
+      <c r="B64" t="inlineStr">
+        <is>
+          <t>jednotka</t>
+        </is>
+      </c>
+      <c r="C64" t="inlineStr">
+        <is>
+          <t>Hlavní město Praha</t>
+        </is>
+      </c>
+      <c r="D64" t="inlineStr">
+        <is>
+          <t>2183/139</t>
+        </is>
+      </c>
+      <c r="E64" t="inlineStr">
+        <is>
+          <t>Žižkov</t>
+        </is>
+      </c>
+      <c r="F64" t="inlineStr">
+        <is>
+          <t>jednotka č. 28220001, garáž v budově č.p. 2822, část obce Žižkov, na parcele 2183/139 Žižkov, podíl na společných částech domu a pozemku 2339/14798</t>
+        </is>
+      </c>
+      <c r="G64" t="n">
+        <v>1</v>
+      </c>
+      <c r="H64" t="inlineStr">
+        <is>
+          <t>jednotka na parcele bez prefixu st. + KU</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="n">
+        <v>8863</v>
+      </c>
+      <c r="B65" t="inlineStr">
+        <is>
+          <t>jednotka</t>
+        </is>
+      </c>
+      <c r="C65" t="inlineStr">
+        <is>
+          <t>Hlavní město Praha</t>
+        </is>
+      </c>
+      <c r="D65" t="inlineStr">
+        <is>
+          <t>2342/472</t>
+        </is>
+      </c>
+      <c r="E65" t="inlineStr">
+        <is>
+          <t>Stodůlky</t>
+        </is>
+      </c>
+      <c r="F65" t="inlineStr">
+        <is>
+          <t>jednotka č. 25660240, garáž v budově č.p. 2566, část obce Stodůlky, na parcele 2342/472 Stodůlky, 2342/473 Stodůlky, podíl na společných částech domu a pozemku 201/28865</t>
+        </is>
+      </c>
+      <c r="G65" t="n">
+        <v>1</v>
+      </c>
+      <c r="H65" t="inlineStr">
+        <is>
+          <t>jednotka na parcele bez prefixu st. + KU</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="n">
+        <v>8863</v>
+      </c>
+      <c r="B66" t="inlineStr">
+        <is>
+          <t>jednotka</t>
+        </is>
+      </c>
+      <c r="C66" t="inlineStr">
+        <is>
+          <t>Hlavní město Praha</t>
+        </is>
+      </c>
+      <c r="D66" t="inlineStr">
+        <is>
+          <t>2342/473</t>
+        </is>
+      </c>
+      <c r="E66" t="inlineStr">
+        <is>
+          <t>Stodůlky</t>
+        </is>
+      </c>
+      <c r="F66" t="inlineStr">
+        <is>
+          <t>jednotka č. 25660240, garáž v budově č.p. 2566, část obce Stodůlky, na parcele 2342/472 Stodůlky, 2342/473 Stodůlky, podíl na společných částech domu a pozemku 201/28865</t>
+        </is>
+      </c>
+      <c r="G66" t="n">
+        <v>1</v>
+      </c>
+      <c r="H66" t="inlineStr">
+        <is>
+          <t>více parcel oddělených čárkou</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="n">
+        <v>7949</v>
+      </c>
+      <c r="B67" t="inlineStr">
+        <is>
+          <t>jednotka</t>
+        </is>
+      </c>
+      <c r="C67" t="inlineStr">
+        <is>
+          <t>Hlavní město Praha</t>
+        </is>
+      </c>
+      <c r="D67" t="inlineStr">
+        <is>
+          <t>3109/20</t>
+        </is>
+      </c>
+      <c r="E67" t="inlineStr">
+        <is>
+          <t>Smíchov</t>
+        </is>
+      </c>
+      <c r="F67" t="inlineStr">
+        <is>
+          <t>jednotka č. 33540101, garáž v budově č.p. 3354, část obce Smíchov, na parcele 3109/20 Smíchov (součástí je stavba č.p. 3354, čst obce Smíchov), podíl na společných částech domu a pozemku 21600/76084</t>
+        </is>
+      </c>
+      <c r="G67" t="n">
+        <v>1</v>
+      </c>
+      <c r="H67" t="inlineStr">
+        <is>
+          <t>jednotka na parcele bez prefixu st. + KU</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="n">
+        <v>7380</v>
+      </c>
+      <c r="B68" t="inlineStr">
+        <is>
+          <t>jednotka</t>
+        </is>
+      </c>
+      <c r="C68" t="inlineStr">
+        <is>
+          <t>Hlavní město Praha</t>
+        </is>
+      </c>
+      <c r="D68" t="inlineStr">
+        <is>
+          <t>527</t>
+        </is>
+      </c>
+      <c r="E68" t="inlineStr">
+        <is>
+          <t>Smíchov</t>
+        </is>
+      </c>
+      <c r="F68" t="inlineStr">
+        <is>
+          <t>jednotka č. 4940103, garáž v budově č.p. 494, část obce Smíchov, na parcele 527 Smíchov (součástí je stavba č.p. 494, čst obce Smíchov), podíl na společných částech domu a pozemku 283/31473</t>
+        </is>
+      </c>
+      <c r="G68" t="n">
+        <v>1</v>
+      </c>
+      <c r="H68" t="inlineStr">
+        <is>
+          <t>jednotka na parcele bez prefixu st. + KU</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="n">
+        <v>7352</v>
+      </c>
+      <c r="B69" t="inlineStr">
+        <is>
+          <t>jednotka</t>
+        </is>
+      </c>
+      <c r="C69" t="inlineStr">
+        <is>
+          <t>Hlavní město Praha</t>
+        </is>
+      </c>
+      <c r="D69" t="inlineStr">
+        <is>
+          <t>3109/20</t>
+        </is>
+      </c>
+      <c r="E69" t="inlineStr">
+        <is>
+          <t>Smíchov</t>
+        </is>
+      </c>
+      <c r="F69" t="inlineStr">
+        <is>
+          <t>jednotka č. 33540101, garáž v budově č.p. 3354, část obce Smíchov, na parcele 3109/20 Smíchov (součástí je stavba č.p. 3354, čst obce Smíchov), podíl na společných částech domu a pozemku 21600/76084</t>
+        </is>
+      </c>
+      <c r="G69" t="n">
+        <v>1</v>
+      </c>
+      <c r="H69" t="inlineStr">
+        <is>
+          <t>jednotka na parcele bez prefixu st. + KU</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="n">
+        <v>2557</v>
+      </c>
+      <c r="B70" t="inlineStr">
+        <is>
+          <t>jednotka</t>
+        </is>
+      </c>
+      <c r="C70" t="inlineStr">
+        <is>
+          <t>Hlavní město Praha</t>
+        </is>
+      </c>
+      <c r="D70" t="inlineStr">
+        <is>
+          <t>2183/139</t>
+        </is>
+      </c>
+      <c r="E70" t="inlineStr">
+        <is>
+          <t>Žižkov</t>
+        </is>
+      </c>
+      <c r="F70" t="inlineStr">
+        <is>
+          <t>jednotka č. 28220002, garáž v budově č.p. 2822, část obce Žižkov, na parcele 2183/139 Žižkov, podíl na společných částech domu a pozemku 2212/14798</t>
+        </is>
+      </c>
+      <c r="G70" t="n">
+        <v>1</v>
+      </c>
+      <c r="H70" t="inlineStr">
+        <is>
+          <t>jednotka na parcele bez prefixu st. + KU</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="n">
+        <v>2028</v>
+      </c>
+      <c r="B71" t="inlineStr">
+        <is>
+          <t>jednotka</t>
+        </is>
+      </c>
+      <c r="C71" t="inlineStr">
+        <is>
+          <t>Hlavní město Praha</t>
+        </is>
+      </c>
+      <c r="D71" t="inlineStr">
+        <is>
+          <t>162/279</t>
+        </is>
+      </c>
+      <c r="E71" t="inlineStr">
+        <is>
+          <t>Stodůlky</t>
+        </is>
+      </c>
+      <c r="F71" t="inlineStr">
+        <is>
+          <t>jednotka č. 27290907, garáž v budově č.p. 2729, část obce Stodůlky, na parcele 162/279 Stodůlky, podíl na společných částech domu a pozemku 24657/144950</t>
+        </is>
+      </c>
+      <c r="G71" t="n">
+        <v>1</v>
+      </c>
+      <c r="H71" t="inlineStr">
+        <is>
+          <t>jednotka na parcele bez prefixu st. + KU</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add new map HTML files for V-86046, V-86597, and V-9328 with Leaflet integration
- Created map_top_V-86046_2019-101.html with interactive map features and multiple tile layers.
- Created map_top_V-86597_2014-101.html with similar structure and functionality.
- Created map_top_V-9328_2024-101.html, ensuring consistent design and features across all maps.
- Integrated OpenStreetMap, Ortofotomapa ČÚZK, and other tile layers for enhanced mapping experience.
- Added GeoJSON data handling for dynamic feature rendering on the maps.
</commit_message>
<xml_diff>
--- a/GIS2/vystup.xlsx
+++ b/GIS2/vystup.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H82"/>
+  <dimension ref="A1:H101"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -472,11 +472,11 @@
     </row>
     <row r="2">
       <c r="A2" t="n">
-        <v>37283</v>
+        <v>27854</v>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>jednotka</t>
+          <t>parcela</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -486,17 +486,17 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>2131/26</t>
+          <t>2838/22</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>Stodůlky</t>
+          <t>Strašnice</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>jednotka č. 20570023, byt v budově č.p. 2057, 2054, 2055, 2056, část obce Stodůlky, na parcele 2131/26 Stodůlky, 2131/27 Stodůlky, 2131/28 Stodůlky, 2131/29 Stodůlky, podíl na společných částech domu a pozemku 7294/839119</t>
+          <t>č. 2838/22 Strašnice</t>
         </is>
       </c>
       <c r="G2" t="n">
@@ -504,17 +504,17 @@
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>jednotka na parcele bez prefixu st. + KU</t>
+          <t>číslo a KU za ním</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="n">
-        <v>37283</v>
+        <v>68251</v>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>jednotka</t>
+          <t>parcela</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -524,17 +524,17 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>2131/27</t>
+          <t>1200/2</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>Stodůlky</t>
+          <t>Hostivař</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>jednotka č. 20570023, byt v budově č.p. 2057, 2054, 2055, 2056, část obce Stodůlky, na parcele 2131/26 Stodůlky, 2131/27 Stodůlky, 2131/28 Stodůlky, 2131/29 Stodůlky, podíl na společných částech domu a pozemku 7294/839119</t>
+          <t>č. 1200/2 Hostivař</t>
         </is>
       </c>
       <c r="G3" t="n">
@@ -542,17 +542,17 @@
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>více parcel oddělených čárkou</t>
+          <t>číslo a KU za ním</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="n">
-        <v>37283</v>
+        <v>27875</v>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>jednotka</t>
+          <t>parcela</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -562,17 +562,17 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>2131/28</t>
+          <t>2838/118</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>Stodůlky</t>
+          <t>Strašnice</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>jednotka č. 20570023, byt v budově č.p. 2057, 2054, 2055, 2056, část obce Stodůlky, na parcele 2131/26 Stodůlky, 2131/27 Stodůlky, 2131/28 Stodůlky, 2131/29 Stodůlky, podíl na společných částech domu a pozemku 7294/839119</t>
+          <t>č. 2838/118 Strašnice</t>
         </is>
       </c>
       <c r="G4" t="n">
@@ -580,17 +580,17 @@
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>více parcel oddělených čárkou</t>
+          <t>číslo a KU za ním</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="n">
-        <v>37283</v>
+        <v>26224</v>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>jednotka</t>
+          <t>parcela</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -600,17 +600,17 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>2131/29</t>
+          <t>378/114</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>Stodůlky</t>
+          <t>Štěrboholy</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>jednotka č. 20570023, byt v budově č.p. 2057, 2054, 2055, 2056, část obce Stodůlky, na parcele 2131/26 Stodůlky, 2131/27 Stodůlky, 2131/28 Stodůlky, 2131/29 Stodůlky, podíl na společných částech domu a pozemku 7294/839119</t>
+          <t>č. 378/114 Štěrboholy</t>
         </is>
       </c>
       <c r="G5" t="n">
@@ -618,17 +618,17 @@
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>více parcel oddělených čárkou</t>
+          <t>číslo a KU za ním</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="n">
-        <v>37282</v>
+        <v>68265</v>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>jednotka</t>
+          <t>parcela</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -638,17 +638,17 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>160/773</t>
+          <t>903/35</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>Stodůlky</t>
+          <t>Malešice</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>jednotka č. 29470010, jiný nebytový prostor v budově č.p. 2947, část obce Stodůlky, na parcele 160/773 Stodůlky (součástí je stavba č.p. 2947, čst obce Stodůlky), podíl na společných částech domu a pozemku 14243/92994</t>
+          <t>č. 903/35 Malešice</t>
         </is>
       </c>
       <c r="G6" t="n">
@@ -656,17 +656,17 @@
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>jednotka na parcele bez prefixu st. + KU</t>
+          <t>číslo a KU za ním</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="n">
-        <v>37281</v>
+        <v>25179</v>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>jednotka</t>
+          <t>parcela</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
@@ -676,17 +676,17 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>160/773</t>
+          <t>378/75</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>Stodůlky</t>
+          <t>Štěrboholy</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>jednotka č. 29470906, byt v budově č.p. 2947, část obce Stodůlky, na parcele 160/773 Stodůlky (součástí je stavba č.p. 2947, čst obce Stodůlky), podíl na společných částech domu a pozemku 591/92994</t>
+          <t>č. 378/75 Štěrboholy</t>
         </is>
       </c>
       <c r="G7" t="n">
@@ -694,13 +694,13 @@
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>jednotka na parcele bez prefixu st. + KU</t>
+          <t>číslo a KU za ním</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="n">
-        <v>37280</v>
+        <v>30732</v>
       </c>
       <c r="B8" t="inlineStr">
         <is>
@@ -714,17 +714,17 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>2969</t>
+          <t>370/151</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>Stodůlky</t>
+          <t>Hostivař</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>č. 2969 Stodůlky</t>
+          <t>č. 370/151 Hostivař</t>
         </is>
       </c>
       <c r="G8" t="n">
@@ -738,7 +738,7 @@
     </row>
     <row r="9">
       <c r="A9" t="n">
-        <v>37279</v>
+        <v>30750</v>
       </c>
       <c r="B9" t="inlineStr">
         <is>
@@ -752,17 +752,17 @@
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>2967</t>
+          <t>370/145</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>Stodůlky</t>
+          <t>Hostivař</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>č. 2967 Stodůlky</t>
+          <t>č. 370/145 Hostivař</t>
         </is>
       </c>
       <c r="G9" t="n">
@@ -776,7 +776,7 @@
     </row>
     <row r="10">
       <c r="A10" t="n">
-        <v>37278</v>
+        <v>68357</v>
       </c>
       <c r="B10" t="inlineStr">
         <is>
@@ -790,17 +790,17 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>2973</t>
+          <t>415/57</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>Stodůlky</t>
+          <t>Štěrboholy</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>č. 2973 Stodůlky</t>
+          <t>č. 415/57 Štěrboholy</t>
         </is>
       </c>
       <c r="G10" t="n">
@@ -814,7 +814,7 @@
     </row>
     <row r="11">
       <c r="A11" t="n">
-        <v>37277</v>
+        <v>27851</v>
       </c>
       <c r="B11" t="inlineStr">
         <is>
@@ -828,17 +828,17 @@
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>2965</t>
+          <t>2794/20</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>Stodůlky</t>
+          <t>Strašnice</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>č. 2965 Stodůlky</t>
+          <t>č. 2794/20 Strašnice</t>
         </is>
       </c>
       <c r="G11" t="n">
@@ -852,7 +852,7 @@
     </row>
     <row r="12">
       <c r="A12" t="n">
-        <v>37276</v>
+        <v>24869</v>
       </c>
       <c r="B12" t="inlineStr">
         <is>
@@ -866,17 +866,17 @@
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>2976</t>
+          <t>903/35</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>Stodůlky</t>
+          <t>Malešice</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>č. 2976 Stodůlky</t>
+          <t>č. 903/35 Malešice</t>
         </is>
       </c>
       <c r="G12" t="n">
@@ -890,7 +890,7 @@
     </row>
     <row r="13">
       <c r="A13" t="n">
-        <v>37275</v>
+        <v>68439</v>
       </c>
       <c r="B13" t="inlineStr">
         <is>
@@ -904,17 +904,17 @@
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>2977</t>
+          <t>3432/47</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>Stodůlky</t>
+          <t>Strašnice</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>č. 2977 Stodůlky</t>
+          <t>č. 3432/47 Strašnice</t>
         </is>
       </c>
       <c r="G13" t="n">
@@ -928,7 +928,7 @@
     </row>
     <row r="14">
       <c r="A14" t="n">
-        <v>37274</v>
+        <v>68376</v>
       </c>
       <c r="B14" t="inlineStr">
         <is>
@@ -942,17 +942,17 @@
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>2970</t>
+          <t>2798/21</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>Stodůlky</t>
+          <t>Strašnice</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>č. 2970 Stodůlky</t>
+          <t>č. 2798/21 Strašnice</t>
         </is>
       </c>
       <c r="G14" t="n">
@@ -966,7 +966,7 @@
     </row>
     <row r="15">
       <c r="A15" t="n">
-        <v>37273</v>
+        <v>27827</v>
       </c>
       <c r="B15" t="inlineStr">
         <is>
@@ -980,17 +980,17 @@
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>2974</t>
+          <t>3118/98</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>Stodůlky</t>
+          <t>Strašnice</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>č. 2974 Stodůlky</t>
+          <t>č. 3118/98 Strašnice</t>
         </is>
       </c>
       <c r="G15" t="n">
@@ -1004,11 +1004,11 @@
     </row>
     <row r="16">
       <c r="A16" t="n">
-        <v>37272</v>
+        <v>26215</v>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>budova</t>
+          <t>parcela</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
@@ -1018,17 +1018,17 @@
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>2964</t>
+          <t>348/155</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>Stodůlky</t>
+          <t>Štěrboholy</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>č. 2964 Stodůlky</t>
+          <t>č. 348/155 Štěrboholy</t>
         </is>
       </c>
       <c r="G16" t="n">
@@ -1036,17 +1036,17 @@
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>č. + KU</t>
+          <t>číslo a KU za ním</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="n">
-        <v>37271</v>
+        <v>30749</v>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>budova</t>
+          <t>parcela</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
@@ -1056,17 +1056,17 @@
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>2971</t>
+          <t>1818/253</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>Stodůlky</t>
+          <t>Hostivař</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>č. 2971 Stodůlky</t>
+          <t>č. 1818/253 Hostivař</t>
         </is>
       </c>
       <c r="G17" t="n">
@@ -1074,17 +1074,17 @@
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>č. + KU</t>
+          <t>číslo a KU za ním</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="n">
-        <v>37270</v>
+        <v>68472</v>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>jednotka</t>
+          <t>parcela</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
@@ -1094,17 +1094,17 @@
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>2964</t>
+          <t>2798/36</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>Stodůlky</t>
+          <t>Strašnice</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>jednotka č. 21480208, garáž v budově č.p. 2144, 2145, 2146, 2147, 2148, 2149, 2150, 2151, 2152, 2153, 2154, část obce Stodůlky, na parcele 2964 Stodůlky, 2965 Stodůlky, 2967 Stodůlky, 2968 Stodůlky, 2969 Stodůlky, 2970 Stodůlky, 2973 Stodůlky, 2974 Stodůlky, 2975 Stodůlky, 2976 Stodůlky, 2977 Stodůlky, podíl na společných částech domu a pozemku 366/476600</t>
+          <t>č. 2798/36 Strašnice</t>
         </is>
       </c>
       <c r="G18" t="n">
@@ -1112,17 +1112,17 @@
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>jednotka na parcele bez prefixu st. + KU</t>
+          <t>číslo a KU za ním</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="n">
-        <v>37270</v>
+        <v>26204</v>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>jednotka</t>
+          <t>parcela</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
@@ -1132,17 +1132,17 @@
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>2965</t>
+          <t>242/15</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>Stodůlky</t>
+          <t>Štěrboholy</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>jednotka č. 21480208, garáž v budově č.p. 2144, 2145, 2146, 2147, 2148, 2149, 2150, 2151, 2152, 2153, 2154, část obce Stodůlky, na parcele 2964 Stodůlky, 2965 Stodůlky, 2967 Stodůlky, 2968 Stodůlky, 2969 Stodůlky, 2970 Stodůlky, 2973 Stodůlky, 2974 Stodůlky, 2975 Stodůlky, 2976 Stodůlky, 2977 Stodůlky, podíl na společných částech domu a pozemku 366/476600</t>
+          <t>č. 242/15 Štěrboholy</t>
         </is>
       </c>
       <c r="G19" t="n">
@@ -1150,17 +1150,17 @@
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>více parcel oddělených čárkou</t>
+          <t>číslo a KU za ním</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="n">
-        <v>37270</v>
+        <v>68347</v>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>jednotka</t>
+          <t>parcela</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
@@ -1170,17 +1170,17 @@
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>2967</t>
+          <t>584/318</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>Stodůlky</t>
+          <t>Dolní Měcholupy</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>jednotka č. 21480208, garáž v budově č.p. 2144, 2145, 2146, 2147, 2148, 2149, 2150, 2151, 2152, 2153, 2154, část obce Stodůlky, na parcele 2964 Stodůlky, 2965 Stodůlky, 2967 Stodůlky, 2968 Stodůlky, 2969 Stodůlky, 2970 Stodůlky, 2973 Stodůlky, 2974 Stodůlky, 2975 Stodůlky, 2976 Stodůlky, 2977 Stodůlky, podíl na společných částech domu a pozemku 366/476600</t>
+          <t>č. 584/318 Dolní Měcholupy</t>
         </is>
       </c>
       <c r="G20" t="n">
@@ -1188,17 +1188,17 @@
       </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t>více parcel oddělených čárkou</t>
+          <t>číslo a KU za ním</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="n">
-        <v>37270</v>
+        <v>27862</v>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>jednotka</t>
+          <t>parcela</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
@@ -1208,17 +1208,17 @@
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>2968</t>
+          <t>3118/98</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>Stodůlky</t>
+          <t>Strašnice</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>jednotka č. 21480208, garáž v budově č.p. 2144, 2145, 2146, 2147, 2148, 2149, 2150, 2151, 2152, 2153, 2154, část obce Stodůlky, na parcele 2964 Stodůlky, 2965 Stodůlky, 2967 Stodůlky, 2968 Stodůlky, 2969 Stodůlky, 2970 Stodůlky, 2973 Stodůlky, 2974 Stodůlky, 2975 Stodůlky, 2976 Stodůlky, 2977 Stodůlky, podíl na společných částech domu a pozemku 366/476600</t>
+          <t>č. 3118/98 Strašnice</t>
         </is>
       </c>
       <c r="G21" t="n">
@@ -1226,17 +1226,17 @@
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>více parcel oddělených čárkou</t>
+          <t>číslo a KU za ním</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="n">
-        <v>37270</v>
+        <v>68349</v>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>jednotka</t>
+          <t>parcela</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
@@ -1246,17 +1246,17 @@
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>2969</t>
+          <t>370/217</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>Stodůlky</t>
+          <t>Štěrboholy</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>jednotka č. 21480208, garáž v budově č.p. 2144, 2145, 2146, 2147, 2148, 2149, 2150, 2151, 2152, 2153, 2154, část obce Stodůlky, na parcele 2964 Stodůlky, 2965 Stodůlky, 2967 Stodůlky, 2968 Stodůlky, 2969 Stodůlky, 2970 Stodůlky, 2973 Stodůlky, 2974 Stodůlky, 2975 Stodůlky, 2976 Stodůlky, 2977 Stodůlky, podíl na společných částech domu a pozemku 366/476600</t>
+          <t>č. 370/217 Štěrboholy</t>
         </is>
       </c>
       <c r="G22" t="n">
@@ -1264,17 +1264,17 @@
       </c>
       <c r="H22" t="inlineStr">
         <is>
-          <t>více parcel oddělených čárkou</t>
+          <t>číslo a KU za ním</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="n">
-        <v>37270</v>
+        <v>68261</v>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>jednotka</t>
+          <t>parcela</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
@@ -1284,17 +1284,17 @@
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>2970</t>
+          <t>1766/32</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>Stodůlky</t>
+          <t>Hostivař</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>jednotka č. 21480208, garáž v budově č.p. 2144, 2145, 2146, 2147, 2148, 2149, 2150, 2151, 2152, 2153, 2154, část obce Stodůlky, na parcele 2964 Stodůlky, 2965 Stodůlky, 2967 Stodůlky, 2968 Stodůlky, 2969 Stodůlky, 2970 Stodůlky, 2973 Stodůlky, 2974 Stodůlky, 2975 Stodůlky, 2976 Stodůlky, 2977 Stodůlky, podíl na společných částech domu a pozemku 366/476600</t>
+          <t>č. 1766/32 Hostivař</t>
         </is>
       </c>
       <c r="G23" t="n">
@@ -1302,17 +1302,17 @@
       </c>
       <c r="H23" t="inlineStr">
         <is>
-          <t>více parcel oddělených čárkou</t>
+          <t>číslo a KU za ním</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="n">
-        <v>37270</v>
+        <v>24844</v>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>jednotka</t>
+          <t>parcela</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
@@ -1322,17 +1322,17 @@
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>2973</t>
+          <t>903/35</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>Stodůlky</t>
+          <t>Malešice</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>jednotka č. 21480208, garáž v budově č.p. 2144, 2145, 2146, 2147, 2148, 2149, 2150, 2151, 2152, 2153, 2154, část obce Stodůlky, na parcele 2964 Stodůlky, 2965 Stodůlky, 2967 Stodůlky, 2968 Stodůlky, 2969 Stodůlky, 2970 Stodůlky, 2973 Stodůlky, 2974 Stodůlky, 2975 Stodůlky, 2976 Stodůlky, 2977 Stodůlky, podíl na společných částech domu a pozemku 366/476600</t>
+          <t>č. 903/35 Malešice</t>
         </is>
       </c>
       <c r="G24" t="n">
@@ -1340,17 +1340,17 @@
       </c>
       <c r="H24" t="inlineStr">
         <is>
-          <t>více parcel oddělených čárkou</t>
+          <t>číslo a KU za ním</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="n">
-        <v>37270</v>
+        <v>24848</v>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>jednotka</t>
+          <t>parcela</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
@@ -1360,17 +1360,17 @@
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>2974</t>
+          <t>806/216</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>Stodůlky</t>
+          <t>Malešice</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>jednotka č. 21480208, garáž v budově č.p. 2144, 2145, 2146, 2147, 2148, 2149, 2150, 2151, 2152, 2153, 2154, část obce Stodůlky, na parcele 2964 Stodůlky, 2965 Stodůlky, 2967 Stodůlky, 2968 Stodůlky, 2969 Stodůlky, 2970 Stodůlky, 2973 Stodůlky, 2974 Stodůlky, 2975 Stodůlky, 2976 Stodůlky, 2977 Stodůlky, podíl na společných částech domu a pozemku 366/476600</t>
+          <t>č. 806/216 Malešice</t>
         </is>
       </c>
       <c r="G25" t="n">
@@ -1378,17 +1378,17 @@
       </c>
       <c r="H25" t="inlineStr">
         <is>
-          <t>více parcel oddělených čárkou</t>
+          <t>číslo a KU za ním</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="n">
-        <v>37270</v>
+        <v>26194</v>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>jednotka</t>
+          <t>parcela</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
@@ -1398,17 +1398,17 @@
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>2975</t>
+          <t>113/1</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>Stodůlky</t>
+          <t>Štěrboholy</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>jednotka č. 21480208, garáž v budově č.p. 2144, 2145, 2146, 2147, 2148, 2149, 2150, 2151, 2152, 2153, 2154, část obce Stodůlky, na parcele 2964 Stodůlky, 2965 Stodůlky, 2967 Stodůlky, 2968 Stodůlky, 2969 Stodůlky, 2970 Stodůlky, 2973 Stodůlky, 2974 Stodůlky, 2975 Stodůlky, 2976 Stodůlky, 2977 Stodůlky, podíl na společných částech domu a pozemku 366/476600</t>
+          <t>č. 113/1 Štěrboholy</t>
         </is>
       </c>
       <c r="G26" t="n">
@@ -1416,17 +1416,17 @@
       </c>
       <c r="H26" t="inlineStr">
         <is>
-          <t>více parcel oddělených čárkou</t>
+          <t>číslo a KU za ním</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="n">
-        <v>37270</v>
+        <v>30812</v>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>jednotka</t>
+          <t>parcela</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
@@ -1436,17 +1436,17 @@
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>2976</t>
+          <t>1818/25</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>Stodůlky</t>
+          <t>Hostivař</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>jednotka č. 21480208, garáž v budově č.p. 2144, 2145, 2146, 2147, 2148, 2149, 2150, 2151, 2152, 2153, 2154, část obce Stodůlky, na parcele 2964 Stodůlky, 2965 Stodůlky, 2967 Stodůlky, 2968 Stodůlky, 2969 Stodůlky, 2970 Stodůlky, 2973 Stodůlky, 2974 Stodůlky, 2975 Stodůlky, 2976 Stodůlky, 2977 Stodůlky, podíl na společných částech domu a pozemku 366/476600</t>
+          <t>č. 1818/25 Hostivař</t>
         </is>
       </c>
       <c r="G27" t="n">
@@ -1454,17 +1454,17 @@
       </c>
       <c r="H27" t="inlineStr">
         <is>
-          <t>více parcel oddělených čárkou</t>
+          <t>číslo a KU za ním</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="n">
-        <v>37270</v>
+        <v>68446</v>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>jednotka</t>
+          <t>parcela</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
@@ -1474,17 +1474,17 @@
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>2977</t>
+          <t>2344</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>Stodůlky</t>
+          <t>Strašnice</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>jednotka č. 21480208, garáž v budově č.p. 2144, 2145, 2146, 2147, 2148, 2149, 2150, 2151, 2152, 2153, 2154, část obce Stodůlky, na parcele 2964 Stodůlky, 2965 Stodůlky, 2967 Stodůlky, 2968 Stodůlky, 2969 Stodůlky, 2970 Stodůlky, 2973 Stodůlky, 2974 Stodůlky, 2975 Stodůlky, 2976 Stodůlky, 2977 Stodůlky, podíl na společných částech domu a pozemku 366/476600</t>
+          <t>č. 2344 Strašnice</t>
         </is>
       </c>
       <c r="G28" t="n">
@@ -1492,17 +1492,17 @@
       </c>
       <c r="H28" t="inlineStr">
         <is>
-          <t>více parcel oddělených čárkou</t>
+          <t>číslo a KU za ním</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="n">
-        <v>37269</v>
+        <v>68243</v>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>jednotka</t>
+          <t>parcela</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
@@ -1512,17 +1512,17 @@
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>2131/262</t>
+          <t>2078/464</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>Stodůlky</t>
+          <t>Záběhlice</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>jednotka č. 19550002, byt v budově č.p. 1955, 1950, 1951, 1952, 1953, 1954, část obce Stodůlky, na parcele 2131/262 Stodůlky (součástí je stavba č.p. 1955, 1950, 1951, 1952, 1953, 1954, čst obce Stodůlky), podíl na společných částech domu a pozemku 4466/1192569</t>
+          <t>č. 2078/464 Záběhlice</t>
         </is>
       </c>
       <c r="G29" t="n">
@@ -1530,17 +1530,17 @@
       </c>
       <c r="H29" t="inlineStr">
         <is>
-          <t>jednotka na parcele bez prefixu st. + KU</t>
+          <t>číslo a KU za ním</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="n">
-        <v>37268</v>
+        <v>28031</v>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>jednotka</t>
+          <t>parcela</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
@@ -1550,17 +1550,17 @@
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>2337/81</t>
+          <t>317/1</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>Stodůlky</t>
+          <t>Strašnice</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>jednotka č. 14650013, byt v budově č.p. 1465, část obce Stodůlky, na parcele 2337/81 Stodůlky, podíl na společných částech domu a pozemku 589/12411</t>
+          <t>č. 317/1 Strašnice</t>
         </is>
       </c>
       <c r="G30" t="n">
@@ -1568,17 +1568,17 @@
       </c>
       <c r="H30" t="inlineStr">
         <is>
-          <t>jednotka na parcele bez prefixu st. + KU</t>
+          <t>číslo a KU za ním</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="n">
-        <v>37267</v>
+        <v>31096</v>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>jednotka</t>
+          <t>parcela</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
@@ -1588,17 +1588,17 @@
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>2131/86</t>
+          <t>989/1</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>Stodůlky</t>
+          <t>Hostivař</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>jednotka č. 20440001, byt v budově č.p. 2044, část obce Stodůlky, na parcele 2131/86 Stodůlky, podíl na společných částech domu a pozemku 6748/206878</t>
+          <t>č. 989/1 Hostivař</t>
         </is>
       </c>
       <c r="G31" t="n">
@@ -1606,13 +1606,13 @@
       </c>
       <c r="H31" t="inlineStr">
         <is>
-          <t>jednotka na parcele bez prefixu st. + KU</t>
+          <t>číslo a KU za ním</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="n">
-        <v>37266</v>
+        <v>26222</v>
       </c>
       <c r="B32" t="inlineStr">
         <is>
@@ -1626,17 +1626,17 @@
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>2780/356</t>
+          <t>255/111</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>Stodůlky</t>
+          <t>Štěrboholy</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>č. 2780/356 Stodůlky</t>
+          <t>č. 255/111 Štěrboholy</t>
         </is>
       </c>
       <c r="G32" t="n">
@@ -1650,11 +1650,11 @@
     </row>
     <row r="33">
       <c r="A33" t="n">
-        <v>37265</v>
+        <v>26217</v>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>jednotka</t>
+          <t>parcela</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
@@ -1664,17 +1664,17 @@
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>2780/305</t>
+          <t>348/214</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>Stodůlky</t>
+          <t>Štěrboholy</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>jednotka č. 25760320, garáž v budově č.p. 2576, část obce Stodůlky, na parcele 2780/305 Stodůlky, 2780/355 Stodůlky, 2780/356 Stodůlky, podíl na společných částech domu a pozemku 61/9402</t>
+          <t>č. 348/214 Štěrboholy</t>
         </is>
       </c>
       <c r="G33" t="n">
@@ -1682,17 +1682,17 @@
       </c>
       <c r="H33" t="inlineStr">
         <is>
-          <t>jednotka na parcele bez prefixu st. + KU</t>
+          <t>číslo a KU za ním</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="n">
-        <v>37265</v>
+        <v>28074</v>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>jednotka</t>
+          <t>parcela</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
@@ -1702,17 +1702,17 @@
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>2780/355</t>
+          <t>317/8</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>Stodůlky</t>
+          <t>Strašnice</t>
         </is>
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>jednotka č. 25760320, garáž v budově č.p. 2576, část obce Stodůlky, na parcele 2780/305 Stodůlky, 2780/355 Stodůlky, 2780/356 Stodůlky, podíl na společných částech domu a pozemku 61/9402</t>
+          <t>č. 317/8 Strašnice</t>
         </is>
       </c>
       <c r="G34" t="n">
@@ -1720,17 +1720,17 @@
       </c>
       <c r="H34" t="inlineStr">
         <is>
-          <t>více parcel oddělených čárkou</t>
+          <t>číslo a KU za ním</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="n">
-        <v>37265</v>
+        <v>31116</v>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>jednotka</t>
+          <t>parcela</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
@@ -1740,17 +1740,17 @@
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>2780/356</t>
+          <t>1818/21</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>Stodůlky</t>
+          <t>Hostivař</t>
         </is>
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>jednotka č. 25760320, garáž v budově č.p. 2576, část obce Stodůlky, na parcele 2780/305 Stodůlky, 2780/355 Stodůlky, 2780/356 Stodůlky, podíl na společných částech domu a pozemku 61/9402</t>
+          <t>č. 1818/21 Hostivař</t>
         </is>
       </c>
       <c r="G35" t="n">
@@ -1758,17 +1758,17 @@
       </c>
       <c r="H35" t="inlineStr">
         <is>
-          <t>více parcel oddělených čárkou</t>
+          <t>číslo a KU za ním</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="n">
-        <v>37264</v>
+        <v>26219</v>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>jednotka</t>
+          <t>parcela</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
@@ -1778,17 +1778,17 @@
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>2131/26</t>
+          <t>326/1</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>Stodůlky</t>
+          <t>Štěrboholy</t>
         </is>
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>jednotka č. 20540022, byt v budově č.p. 2057, 2054, 2055, 2056, část obce Stodůlky, na parcele 2131/26 Stodůlky, 2131/27 Stodůlky, 2131/28 Stodůlky, 2131/29 Stodůlky, podíl na společných částech domu a pozemku 9011/839119</t>
+          <t>č. 326/1 Štěrboholy</t>
         </is>
       </c>
       <c r="G36" t="n">
@@ -1796,17 +1796,17 @@
       </c>
       <c r="H36" t="inlineStr">
         <is>
-          <t>jednotka na parcele bez prefixu st. + KU</t>
+          <t>číslo a KU za ním</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="n">
-        <v>37264</v>
+        <v>28035</v>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>jednotka</t>
+          <t>parcela</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
@@ -1816,17 +1816,17 @@
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>2131/27</t>
+          <t>2637/7</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>Stodůlky</t>
+          <t>Strašnice</t>
         </is>
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>jednotka č. 20540022, byt v budově č.p. 2057, 2054, 2055, 2056, část obce Stodůlky, na parcele 2131/26 Stodůlky, 2131/27 Stodůlky, 2131/28 Stodůlky, 2131/29 Stodůlky, podíl na společných částech domu a pozemku 9011/839119</t>
+          <t>č. 2637/7 Strašnice</t>
         </is>
       </c>
       <c r="G37" t="n">
@@ -1834,17 +1834,17 @@
       </c>
       <c r="H37" t="inlineStr">
         <is>
-          <t>více parcel oddělených čárkou</t>
+          <t>číslo a KU za ním</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="n">
-        <v>37264</v>
+        <v>28043</v>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>jednotka</t>
+          <t>parcela</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
@@ -1854,17 +1854,17 @@
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>2131/28</t>
+          <t>3925/16</t>
         </is>
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>Stodůlky</t>
+          <t>Strašnice</t>
         </is>
       </c>
       <c r="F38" t="inlineStr">
         <is>
-          <t>jednotka č. 20540022, byt v budově č.p. 2057, 2054, 2055, 2056, část obce Stodůlky, na parcele 2131/26 Stodůlky, 2131/27 Stodůlky, 2131/28 Stodůlky, 2131/29 Stodůlky, podíl na společných částech domu a pozemku 9011/839119</t>
+          <t>č. 3925/16 Strašnice</t>
         </is>
       </c>
       <c r="G38" t="n">
@@ -1872,17 +1872,17 @@
       </c>
       <c r="H38" t="inlineStr">
         <is>
-          <t>více parcel oddělených čárkou</t>
+          <t>číslo a KU za ním</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="n">
-        <v>37264</v>
+        <v>68506</v>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>jednotka</t>
+          <t>parcela</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
@@ -1892,17 +1892,17 @@
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>2131/29</t>
+          <t>1222</t>
         </is>
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>Stodůlky</t>
+          <t>Hostivař</t>
         </is>
       </c>
       <c r="F39" t="inlineStr">
         <is>
-          <t>jednotka č. 20540022, byt v budově č.p. 2057, 2054, 2055, 2056, část obce Stodůlky, na parcele 2131/26 Stodůlky, 2131/27 Stodůlky, 2131/28 Stodůlky, 2131/29 Stodůlky, podíl na společných částech domu a pozemku 9011/839119</t>
+          <t>č. 1222 Hostivař</t>
         </is>
       </c>
       <c r="G39" t="n">
@@ -1910,17 +1910,17 @@
       </c>
       <c r="H39" t="inlineStr">
         <is>
-          <t>více parcel oddělených čárkou</t>
+          <t>číslo a KU za ním</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="n">
-        <v>37263</v>
+        <v>27972</v>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>budova</t>
+          <t>parcela</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
@@ -1930,17 +1930,17 @@
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>2780/165</t>
+          <t>2838/64</t>
         </is>
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>Stodůlky</t>
+          <t>Strašnice</t>
         </is>
       </c>
       <c r="F40" t="inlineStr">
         <is>
-          <t>č. 2780/165 Stodůlky</t>
+          <t>č. 2838/64 Strašnice</t>
         </is>
       </c>
       <c r="G40" t="n">
@@ -1948,17 +1948,17 @@
       </c>
       <c r="H40" t="inlineStr">
         <is>
-          <t>č. + KU</t>
+          <t>číslo a KU za ním</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="n">
-        <v>37262</v>
+        <v>27966</v>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>jednotka</t>
+          <t>parcela</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
@@ -1968,17 +1968,17 @@
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>2780/165</t>
+          <t>2244/110</t>
         </is>
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>Stodůlky</t>
+          <t>Strašnice</t>
         </is>
       </c>
       <c r="F41" t="inlineStr">
         <is>
-          <t>jednotka č. 25220003, byt v budově č.p. 2522, část obce Stodůlky, na parcele 2780/165 Stodůlky, podíl na společných částech domu a pozemku 13592/683778</t>
+          <t>č. 2244/110 Strašnice</t>
         </is>
       </c>
       <c r="G41" t="n">
@@ -1986,17 +1986,17 @@
       </c>
       <c r="H41" t="inlineStr">
         <is>
-          <t>jednotka na parcele bez prefixu st. + KU</t>
+          <t>číslo a KU za ním</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="n">
-        <v>37261</v>
+        <v>25249</v>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>jednotka</t>
+          <t>parcela</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
@@ -2006,17 +2006,17 @@
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>2121/2</t>
+          <t>242/17</t>
         </is>
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>Stodůlky</t>
+          <t>Štěrboholy</t>
         </is>
       </c>
       <c r="F42" t="inlineStr">
         <is>
-          <t>jednotka č. 26040001, garáž v budově č.p. 2604, část obce Stodůlky, na parcele 2121/2 Stodůlky, podíl na společných částech domu a pozemku 43980/251890</t>
+          <t>č. 242/17 Štěrboholy</t>
         </is>
       </c>
       <c r="G42" t="n">
@@ -2024,17 +2024,17 @@
       </c>
       <c r="H42" t="inlineStr">
         <is>
-          <t>jednotka na parcele bez prefixu st. + KU</t>
+          <t>číslo a KU za ním</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="n">
-        <v>37260</v>
+        <v>68493</v>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>jednotka</t>
+          <t>parcela</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
@@ -2044,17 +2044,17 @@
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>2121/2</t>
+          <t>1766/32</t>
         </is>
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>Stodůlky</t>
+          <t>Hostivař</t>
         </is>
       </c>
       <c r="F43" t="inlineStr">
         <is>
-          <t>jednotka č. 26040033, byt v budově č.p. 2604, část obce Stodůlky, na parcele 2121/2 Stodůlky, podíl na společných částech domu a pozemku 12611/251890</t>
+          <t>č. 1766/32 Hostivař</t>
         </is>
       </c>
       <c r="G43" t="n">
@@ -2062,17 +2062,17 @@
       </c>
       <c r="H43" t="inlineStr">
         <is>
-          <t>jednotka na parcele bez prefixu st. + KU</t>
+          <t>číslo a KU za ním</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="n">
-        <v>37259</v>
+        <v>24841</v>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>jednotka</t>
+          <t>parcela</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
@@ -2082,17 +2082,17 @@
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>151/24</t>
+          <t>902/8</t>
         </is>
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>Stodůlky</t>
+          <t>Malešice</t>
         </is>
       </c>
       <c r="F44" t="inlineStr">
         <is>
-          <t>jednotka č. 15500003, byt v budově č.p. 1551, 1547, 1548, 1549, 1550, část obce Stodůlky, na parcele 151/24 Stodůlky, 151/25 Stodůlky, 151/26 Stodůlky, 151/27 Stodůlky, 151/28 Stodůlky, podíl na společných částech domu a pozemku 6967/750632</t>
+          <t>č. 902/8 Malešice</t>
         </is>
       </c>
       <c r="G44" t="n">
@@ -2100,17 +2100,17 @@
       </c>
       <c r="H44" t="inlineStr">
         <is>
-          <t>jednotka na parcele bez prefixu st. + KU</t>
+          <t>číslo a KU za ním</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="n">
-        <v>37259</v>
+        <v>68520</v>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>jednotka</t>
+          <t>parcela</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
@@ -2120,17 +2120,17 @@
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>151/25</t>
+          <t>223/4</t>
         </is>
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>Stodůlky</t>
+          <t>Malešice</t>
         </is>
       </c>
       <c r="F45" t="inlineStr">
         <is>
-          <t>jednotka č. 15500003, byt v budově č.p. 1551, 1547, 1548, 1549, 1550, část obce Stodůlky, na parcele 151/24 Stodůlky, 151/25 Stodůlky, 151/26 Stodůlky, 151/27 Stodůlky, 151/28 Stodůlky, podíl na společných částech domu a pozemku 6967/750632</t>
+          <t>č. 223/4 Malešice</t>
         </is>
       </c>
       <c r="G45" t="n">
@@ -2138,17 +2138,17 @@
       </c>
       <c r="H45" t="inlineStr">
         <is>
-          <t>více parcel oddělených čárkou</t>
+          <t>číslo a KU za ním</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="n">
-        <v>37259</v>
+        <v>68984</v>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>jednotka</t>
+          <t>parcela</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
@@ -2158,17 +2158,17 @@
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>151/26</t>
+          <t>119</t>
         </is>
       </c>
       <c r="E46" t="inlineStr">
         <is>
-          <t>Stodůlky</t>
+          <t>Štěrboholy</t>
         </is>
       </c>
       <c r="F46" t="inlineStr">
         <is>
-          <t>jednotka č. 15500003, byt v budově č.p. 1551, 1547, 1548, 1549, 1550, část obce Stodůlky, na parcele 151/24 Stodůlky, 151/25 Stodůlky, 151/26 Stodůlky, 151/27 Stodůlky, 151/28 Stodůlky, podíl na společných částech domu a pozemku 6967/750632</t>
+          <t>č. 119 Štěrboholy</t>
         </is>
       </c>
       <c r="G46" t="n">
@@ -2176,17 +2176,17 @@
       </c>
       <c r="H46" t="inlineStr">
         <is>
-          <t>více parcel oddělených čárkou</t>
+          <t>číslo a KU za ním</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="n">
-        <v>37259</v>
+        <v>68537</v>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>jednotka</t>
+          <t>parcela</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
@@ -2196,17 +2196,17 @@
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>151/27</t>
+          <t>119</t>
         </is>
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t>Stodůlky</t>
+          <t>Štěrboholy</t>
         </is>
       </c>
       <c r="F47" t="inlineStr">
         <is>
-          <t>jednotka č. 15500003, byt v budově č.p. 1551, 1547, 1548, 1549, 1550, část obce Stodůlky, na parcele 151/24 Stodůlky, 151/25 Stodůlky, 151/26 Stodůlky, 151/27 Stodůlky, 151/28 Stodůlky, podíl na společných částech domu a pozemku 6967/750632</t>
+          <t>č. 119 Štěrboholy</t>
         </is>
       </c>
       <c r="G47" t="n">
@@ -2214,17 +2214,17 @@
       </c>
       <c r="H47" t="inlineStr">
         <is>
-          <t>více parcel oddělených čárkou</t>
+          <t>číslo a KU za ním</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="n">
-        <v>37259</v>
+        <v>68992</v>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>jednotka</t>
+          <t>parcela</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
@@ -2234,17 +2234,17 @@
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>151/28</t>
+          <t>119</t>
         </is>
       </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t>Stodůlky</t>
+          <t>Štěrboholy</t>
         </is>
       </c>
       <c r="F48" t="inlineStr">
         <is>
-          <t>jednotka č. 15500003, byt v budově č.p. 1551, 1547, 1548, 1549, 1550, část obce Stodůlky, na parcele 151/24 Stodůlky, 151/25 Stodůlky, 151/26 Stodůlky, 151/27 Stodůlky, 151/28 Stodůlky, podíl na společných částech domu a pozemku 6967/750632</t>
+          <t>č. 119 Štěrboholy</t>
         </is>
       </c>
       <c r="G48" t="n">
@@ -2252,17 +2252,17 @@
       </c>
       <c r="H48" t="inlineStr">
         <is>
-          <t>více parcel oddělených čárkou</t>
+          <t>číslo a KU za ním</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="n">
-        <v>37258</v>
+        <v>68525</v>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>jednotka</t>
+          <t>parcela</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
@@ -2272,17 +2272,17 @@
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>2131/180</t>
+          <t>903/35</t>
         </is>
       </c>
       <c r="E49" t="inlineStr">
         <is>
-          <t>Stodůlky</t>
+          <t>Malešice</t>
         </is>
       </c>
       <c r="F49" t="inlineStr">
         <is>
-          <t>jednotka č. 27220100, byt v budově č.p. 2722, část obce Stodůlky, na parcele 2131/180 Stodůlky, podíl na společných částech domu a pozemku 6087/1627256</t>
+          <t>č. 903/35 Malešice</t>
         </is>
       </c>
       <c r="G49" t="n">
@@ -2290,17 +2290,17 @@
       </c>
       <c r="H49" t="inlineStr">
         <is>
-          <t>jednotka na parcele bez prefixu st. + KU</t>
+          <t>číslo a KU za ním</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="n">
-        <v>37257</v>
+        <v>68500</v>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>jednotka</t>
+          <t>parcela</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
@@ -2310,17 +2310,17 @@
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>2849/1</t>
+          <t>1818/253</t>
         </is>
       </c>
       <c r="E50" t="inlineStr">
         <is>
-          <t>Stodůlky</t>
+          <t>Hostivař</t>
         </is>
       </c>
       <c r="F50" t="inlineStr">
         <is>
-          <t>jednotka č. 25640013, byt v budově č.p. 2565, 2560, 2561, 2562, 2563, 2564, část obce Stodůlky, na parcele 2849/1 Stodůlky, 2849/2 Stodůlky, 2849/4 Stodůlky, 2850/1 Stodůlky, 2850/3 Stodůlky, 2851/1 Stodůlky, 2851/2 Stodůlky, 2852/1 Stodůlky, 2852/2 Stodůlky, 2852/3 Stodůlky, podíl na společných částech domu a pozemku 4040/1217029</t>
+          <t>č. 1818/253 Hostivař</t>
         </is>
       </c>
       <c r="G50" t="n">
@@ -2328,17 +2328,17 @@
       </c>
       <c r="H50" t="inlineStr">
         <is>
-          <t>jednotka na parcele bez prefixu st. + KU</t>
+          <t>číslo a KU za ním</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="n">
-        <v>37257</v>
+        <v>26227</v>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>jednotka</t>
+          <t>parcela</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
@@ -2348,17 +2348,17 @@
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>2849/2</t>
+          <t>349/25</t>
         </is>
       </c>
       <c r="E51" t="inlineStr">
         <is>
-          <t>Stodůlky</t>
+          <t>Štěrboholy</t>
         </is>
       </c>
       <c r="F51" t="inlineStr">
         <is>
-          <t>jednotka č. 25640013, byt v budově č.p. 2565, 2560, 2561, 2562, 2563, 2564, část obce Stodůlky, na parcele 2849/1 Stodůlky, 2849/2 Stodůlky, 2849/4 Stodůlky, 2850/1 Stodůlky, 2850/3 Stodůlky, 2851/1 Stodůlky, 2851/2 Stodůlky, 2852/1 Stodůlky, 2852/2 Stodůlky, 2852/3 Stodůlky, podíl na společných částech domu a pozemku 4040/1217029</t>
+          <t>č. 349/25 Štěrboholy</t>
         </is>
       </c>
       <c r="G51" t="n">
@@ -2366,17 +2366,17 @@
       </c>
       <c r="H51" t="inlineStr">
         <is>
-          <t>více parcel oddělených čárkou</t>
+          <t>číslo a KU za ním</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="n">
-        <v>37257</v>
+        <v>28057</v>
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>jednotka</t>
+          <t>parcela</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
@@ -2386,17 +2386,17 @@
       </c>
       <c r="D52" t="inlineStr">
         <is>
-          <t>2849/4</t>
+          <t>3925/16</t>
         </is>
       </c>
       <c r="E52" t="inlineStr">
         <is>
-          <t>Stodůlky</t>
+          <t>Strašnice</t>
         </is>
       </c>
       <c r="F52" t="inlineStr">
         <is>
-          <t>jednotka č. 25640013, byt v budově č.p. 2565, 2560, 2561, 2562, 2563, 2564, část obce Stodůlky, na parcele 2849/1 Stodůlky, 2849/2 Stodůlky, 2849/4 Stodůlky, 2850/1 Stodůlky, 2850/3 Stodůlky, 2851/1 Stodůlky, 2851/2 Stodůlky, 2852/1 Stodůlky, 2852/2 Stodůlky, 2852/3 Stodůlky, podíl na společných částech domu a pozemku 4040/1217029</t>
+          <t>č. 3925/16 Strašnice</t>
         </is>
       </c>
       <c r="G52" t="n">
@@ -2404,17 +2404,17 @@
       </c>
       <c r="H52" t="inlineStr">
         <is>
-          <t>více parcel oddělených čárkou</t>
+          <t>číslo a KU za ním</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="n">
-        <v>37257</v>
+        <v>28007</v>
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>jednotka</t>
+          <t>parcela</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
@@ -2424,17 +2424,17 @@
       </c>
       <c r="D53" t="inlineStr">
         <is>
-          <t>2850/1</t>
+          <t>3233/3</t>
         </is>
       </c>
       <c r="E53" t="inlineStr">
         <is>
-          <t>Stodůlky</t>
+          <t>Strašnice</t>
         </is>
       </c>
       <c r="F53" t="inlineStr">
         <is>
-          <t>jednotka č. 25640013, byt v budově č.p. 2565, 2560, 2561, 2562, 2563, 2564, část obce Stodůlky, na parcele 2849/1 Stodůlky, 2849/2 Stodůlky, 2849/4 Stodůlky, 2850/1 Stodůlky, 2850/3 Stodůlky, 2851/1 Stodůlky, 2851/2 Stodůlky, 2852/1 Stodůlky, 2852/2 Stodůlky, 2852/3 Stodůlky, podíl na společných částech domu a pozemku 4040/1217029</t>
+          <t>č. 3233/3 Strašnice</t>
         </is>
       </c>
       <c r="G53" t="n">
@@ -2442,17 +2442,17 @@
       </c>
       <c r="H53" t="inlineStr">
         <is>
-          <t>více parcel oddělených čárkou</t>
+          <t>číslo a KU za ním</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="n">
-        <v>37257</v>
+        <v>68583</v>
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>jednotka</t>
+          <t>parcela</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
@@ -2462,17 +2462,17 @@
       </c>
       <c r="D54" t="inlineStr">
         <is>
-          <t>2850/3</t>
+          <t>2438/1</t>
         </is>
       </c>
       <c r="E54" t="inlineStr">
         <is>
-          <t>Stodůlky</t>
+          <t>Strašnice</t>
         </is>
       </c>
       <c r="F54" t="inlineStr">
         <is>
-          <t>jednotka č. 25640013, byt v budově č.p. 2565, 2560, 2561, 2562, 2563, 2564, část obce Stodůlky, na parcele 2849/1 Stodůlky, 2849/2 Stodůlky, 2849/4 Stodůlky, 2850/1 Stodůlky, 2850/3 Stodůlky, 2851/1 Stodůlky, 2851/2 Stodůlky, 2852/1 Stodůlky, 2852/2 Stodůlky, 2852/3 Stodůlky, podíl na společných částech domu a pozemku 4040/1217029</t>
+          <t>č. 2438/1 Strašnice</t>
         </is>
       </c>
       <c r="G54" t="n">
@@ -2480,17 +2480,17 @@
       </c>
       <c r="H54" t="inlineStr">
         <is>
-          <t>více parcel oddělených čárkou</t>
+          <t>číslo a KU za ním</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="n">
-        <v>37257</v>
+        <v>30888</v>
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>jednotka</t>
+          <t>parcela</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
@@ -2500,17 +2500,17 @@
       </c>
       <c r="D55" t="inlineStr">
         <is>
-          <t>2851/1</t>
+          <t>1740/12</t>
         </is>
       </c>
       <c r="E55" t="inlineStr">
         <is>
-          <t>Stodůlky</t>
+          <t>Hostivař</t>
         </is>
       </c>
       <c r="F55" t="inlineStr">
         <is>
-          <t>jednotka č. 25640013, byt v budově č.p. 2565, 2560, 2561, 2562, 2563, 2564, část obce Stodůlky, na parcele 2849/1 Stodůlky, 2849/2 Stodůlky, 2849/4 Stodůlky, 2850/1 Stodůlky, 2850/3 Stodůlky, 2851/1 Stodůlky, 2851/2 Stodůlky, 2852/1 Stodůlky, 2852/2 Stodůlky, 2852/3 Stodůlky, podíl na společných částech domu a pozemku 4040/1217029</t>
+          <t>č. 1740/12 Hostivař</t>
         </is>
       </c>
       <c r="G55" t="n">
@@ -2518,17 +2518,17 @@
       </c>
       <c r="H55" t="inlineStr">
         <is>
-          <t>více parcel oddělených čárkou</t>
+          <t>číslo a KU za ním</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="n">
-        <v>37257</v>
+        <v>68528</v>
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>jednotka</t>
+          <t>parcela</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
@@ -2538,17 +2538,17 @@
       </c>
       <c r="D56" t="inlineStr">
         <is>
-          <t>2851/2</t>
+          <t>2244/2</t>
         </is>
       </c>
       <c r="E56" t="inlineStr">
         <is>
-          <t>Stodůlky</t>
+          <t>Strašnice</t>
         </is>
       </c>
       <c r="F56" t="inlineStr">
         <is>
-          <t>jednotka č. 25640013, byt v budově č.p. 2565, 2560, 2561, 2562, 2563, 2564, část obce Stodůlky, na parcele 2849/1 Stodůlky, 2849/2 Stodůlky, 2849/4 Stodůlky, 2850/1 Stodůlky, 2850/3 Stodůlky, 2851/1 Stodůlky, 2851/2 Stodůlky, 2852/1 Stodůlky, 2852/2 Stodůlky, 2852/3 Stodůlky, podíl na společných částech domu a pozemku 4040/1217029</t>
+          <t>č. 2244/2 Strašnice</t>
         </is>
       </c>
       <c r="G56" t="n">
@@ -2556,17 +2556,17 @@
       </c>
       <c r="H56" t="inlineStr">
         <is>
-          <t>více parcel oddělených čárkou</t>
+          <t>číslo a KU za ním</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="n">
-        <v>37257</v>
+        <v>68625</v>
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>jednotka</t>
+          <t>parcela</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
@@ -2576,17 +2576,17 @@
       </c>
       <c r="D57" t="inlineStr">
         <is>
-          <t>2852/1</t>
+          <t>1831/1</t>
         </is>
       </c>
       <c r="E57" t="inlineStr">
         <is>
-          <t>Stodůlky</t>
+          <t>Strašnice</t>
         </is>
       </c>
       <c r="F57" t="inlineStr">
         <is>
-          <t>jednotka č. 25640013, byt v budově č.p. 2565, 2560, 2561, 2562, 2563, 2564, část obce Stodůlky, na parcele 2849/1 Stodůlky, 2849/2 Stodůlky, 2849/4 Stodůlky, 2850/1 Stodůlky, 2850/3 Stodůlky, 2851/1 Stodůlky, 2851/2 Stodůlky, 2852/1 Stodůlky, 2852/2 Stodůlky, 2852/3 Stodůlky, podíl na společných částech domu a pozemku 4040/1217029</t>
+          <t>č. 1831/1 Strašnice</t>
         </is>
       </c>
       <c r="G57" t="n">
@@ -2594,17 +2594,17 @@
       </c>
       <c r="H57" t="inlineStr">
         <is>
-          <t>více parcel oddělených čárkou</t>
+          <t>číslo a KU za ním</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="n">
-        <v>37257</v>
+        <v>68610</v>
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>jednotka</t>
+          <t>parcela</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
@@ -2614,17 +2614,17 @@
       </c>
       <c r="D58" t="inlineStr">
         <is>
-          <t>2852/2</t>
+          <t>2798/172</t>
         </is>
       </c>
       <c r="E58" t="inlineStr">
         <is>
-          <t>Stodůlky</t>
+          <t>Strašnice</t>
         </is>
       </c>
       <c r="F58" t="inlineStr">
         <is>
-          <t>jednotka č. 25640013, byt v budově č.p. 2565, 2560, 2561, 2562, 2563, 2564, část obce Stodůlky, na parcele 2849/1 Stodůlky, 2849/2 Stodůlky, 2849/4 Stodůlky, 2850/1 Stodůlky, 2850/3 Stodůlky, 2851/1 Stodůlky, 2851/2 Stodůlky, 2852/1 Stodůlky, 2852/2 Stodůlky, 2852/3 Stodůlky, podíl na společných částech domu a pozemku 4040/1217029</t>
+          <t>č. 2798/172 Strašnice</t>
         </is>
       </c>
       <c r="G58" t="n">
@@ -2632,17 +2632,17 @@
       </c>
       <c r="H58" t="inlineStr">
         <is>
-          <t>více parcel oddělených čárkou</t>
+          <t>číslo a KU za ním</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="n">
-        <v>37257</v>
+        <v>27979</v>
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>jednotka</t>
+          <t>parcela</t>
         </is>
       </c>
       <c r="C59" t="inlineStr">
@@ -2652,17 +2652,17 @@
       </c>
       <c r="D59" t="inlineStr">
         <is>
-          <t>2852/3</t>
+          <t>2244/24</t>
         </is>
       </c>
       <c r="E59" t="inlineStr">
         <is>
-          <t>Stodůlky</t>
+          <t>Strašnice</t>
         </is>
       </c>
       <c r="F59" t="inlineStr">
         <is>
-          <t>jednotka č. 25640013, byt v budově č.p. 2565, 2560, 2561, 2562, 2563, 2564, část obce Stodůlky, na parcele 2849/1 Stodůlky, 2849/2 Stodůlky, 2849/4 Stodůlky, 2850/1 Stodůlky, 2850/3 Stodůlky, 2851/1 Stodůlky, 2851/2 Stodůlky, 2852/1 Stodůlky, 2852/2 Stodůlky, 2852/3 Stodůlky, podíl na společných částech domu a pozemku 4040/1217029</t>
+          <t>č. 2244/24 Strašnice</t>
         </is>
       </c>
       <c r="G59" t="n">
@@ -2670,13 +2670,13 @@
       </c>
       <c r="H59" t="inlineStr">
         <is>
-          <t>více parcel oddělených čárkou</t>
+          <t>číslo a KU za ním</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="n">
-        <v>37256</v>
+        <v>26184</v>
       </c>
       <c r="B60" t="inlineStr">
         <is>
@@ -2690,17 +2690,17 @@
       </c>
       <c r="D60" t="inlineStr">
         <is>
-          <t>1947/5</t>
+          <t>196/39</t>
         </is>
       </c>
       <c r="E60" t="inlineStr">
         <is>
-          <t>Stodůlky</t>
+          <t>Štěrboholy</t>
         </is>
       </c>
       <c r="F60" t="inlineStr">
         <is>
-          <t>č. 1947/5 Stodůlky</t>
+          <t>č. 196/39 Štěrboholy</t>
         </is>
       </c>
       <c r="G60" t="n">
@@ -2714,7 +2714,7 @@
     </row>
     <row r="61">
       <c r="A61" t="n">
-        <v>37255</v>
+        <v>68517</v>
       </c>
       <c r="B61" t="inlineStr">
         <is>
@@ -2728,17 +2728,17 @@
       </c>
       <c r="D61" t="inlineStr">
         <is>
-          <t>1947/1</t>
+          <t>806/205</t>
         </is>
       </c>
       <c r="E61" t="inlineStr">
         <is>
-          <t>Stodůlky</t>
+          <t>Malešice</t>
         </is>
       </c>
       <c r="F61" t="inlineStr">
         <is>
-          <t>č. 1947/1 Stodůlky</t>
+          <t>č. 806/205 Malešice</t>
         </is>
       </c>
       <c r="G61" t="n">
@@ -2752,7 +2752,7 @@
     </row>
     <row r="62">
       <c r="A62" t="n">
-        <v>37254</v>
+        <v>28033</v>
       </c>
       <c r="B62" t="inlineStr">
         <is>
@@ -2766,17 +2766,17 @@
       </c>
       <c r="D62" t="inlineStr">
         <is>
-          <t>1947/4</t>
+          <t>2796/116</t>
         </is>
       </c>
       <c r="E62" t="inlineStr">
         <is>
-          <t>Stodůlky</t>
+          <t>Strašnice</t>
         </is>
       </c>
       <c r="F62" t="inlineStr">
         <is>
-          <t>č. 1947/4 Stodůlky</t>
+          <t>č. 2796/116 Strašnice</t>
         </is>
       </c>
       <c r="G62" t="n">
@@ -2790,7 +2790,7 @@
     </row>
     <row r="63">
       <c r="A63" t="n">
-        <v>37253</v>
+        <v>30916</v>
       </c>
       <c r="B63" t="inlineStr">
         <is>
@@ -2804,17 +2804,17 @@
       </c>
       <c r="D63" t="inlineStr">
         <is>
-          <t>2010/225</t>
+          <t>1818/28</t>
         </is>
       </c>
       <c r="E63" t="inlineStr">
         <is>
-          <t>Stodůlky</t>
+          <t>Hostivař</t>
         </is>
       </c>
       <c r="F63" t="inlineStr">
         <is>
-          <t>č. 2010/225 Stodůlky</t>
+          <t>č. 1818/28 Hostivař</t>
         </is>
       </c>
       <c r="G63" t="n">
@@ -2828,7 +2828,7 @@
     </row>
     <row r="64">
       <c r="A64" t="n">
-        <v>37252</v>
+        <v>24881</v>
       </c>
       <c r="B64" t="inlineStr">
         <is>
@@ -2842,17 +2842,17 @@
       </c>
       <c r="D64" t="inlineStr">
         <is>
-          <t>2010/224</t>
+          <t>64/10</t>
         </is>
       </c>
       <c r="E64" t="inlineStr">
         <is>
-          <t>Stodůlky</t>
+          <t>Malešice</t>
         </is>
       </c>
       <c r="F64" t="inlineStr">
         <is>
-          <t>č. 2010/224 Stodůlky</t>
+          <t>č. 64/10 Malešice</t>
         </is>
       </c>
       <c r="G64" t="n">
@@ -2866,11 +2866,11 @@
     </row>
     <row r="65">
       <c r="A65" t="n">
-        <v>37251</v>
+        <v>28017</v>
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>budova</t>
+          <t>parcela</t>
         </is>
       </c>
       <c r="C65" t="inlineStr">
@@ -2880,17 +2880,17 @@
       </c>
       <c r="D65" t="inlineStr">
         <is>
-          <t>1947/8</t>
+          <t>4031/112</t>
         </is>
       </c>
       <c r="E65" t="inlineStr">
         <is>
-          <t>Stodůlky</t>
+          <t>Strašnice</t>
         </is>
       </c>
       <c r="F65" t="inlineStr">
         <is>
-          <t>č. 1947/8 Stodůlky (součástí je stavba č.p. 772, čst obce Stodůlky)</t>
+          <t>č. 4031/112 Strašnice</t>
         </is>
       </c>
       <c r="G65" t="n">
@@ -2898,17 +2898,17 @@
       </c>
       <c r="H65" t="inlineStr">
         <is>
-          <t>č. + KU</t>
+          <t>číslo a KU za ním</t>
         </is>
       </c>
     </row>
     <row r="66">
       <c r="A66" t="n">
-        <v>37250</v>
+        <v>68586</v>
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>jednotka</t>
+          <t>parcela</t>
         </is>
       </c>
       <c r="C66" t="inlineStr">
@@ -2918,17 +2918,17 @@
       </c>
       <c r="D66" t="inlineStr">
         <is>
-          <t>2131/46</t>
+          <t>248</t>
         </is>
       </c>
       <c r="E66" t="inlineStr">
         <is>
-          <t>Stodůlky</t>
+          <t>Strašnice</t>
         </is>
       </c>
       <c r="F66" t="inlineStr">
         <is>
-          <t>jednotka č. 19390003, byt v budově č.p. 1939, část obce Stodůlky, na parcele 2131/46 Stodůlky, podíl na společných částech domu a pozemku 558/53725</t>
+          <t>č. 248 Strašnice</t>
         </is>
       </c>
       <c r="G66" t="n">
@@ -2936,13 +2936,13 @@
       </c>
       <c r="H66" t="inlineStr">
         <is>
-          <t>jednotka na parcele bez prefixu st. + KU</t>
+          <t>číslo a KU za ním</t>
         </is>
       </c>
     </row>
     <row r="67">
       <c r="A67" t="n">
-        <v>37249</v>
+        <v>30606</v>
       </c>
       <c r="B67" t="inlineStr">
         <is>
@@ -2956,17 +2956,17 @@
       </c>
       <c r="D67" t="inlineStr">
         <is>
-          <t>2315/1</t>
+          <t>1766/13</t>
         </is>
       </c>
       <c r="E67" t="inlineStr">
         <is>
-          <t>Stodůlky</t>
+          <t>Hostivař</t>
         </is>
       </c>
       <c r="F67" t="inlineStr">
         <is>
-          <t>č. 2315/1 Stodůlky</t>
+          <t>č. 1766/13 Hostivař</t>
         </is>
       </c>
       <c r="G67" t="n">
@@ -2980,11 +2980,11 @@
     </row>
     <row r="68">
       <c r="A68" t="n">
-        <v>37248</v>
+        <v>24875</v>
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>jednotka</t>
+          <t>parcela</t>
         </is>
       </c>
       <c r="C68" t="inlineStr">
@@ -2994,17 +2994,17 @@
       </c>
       <c r="D68" t="inlineStr">
         <is>
-          <t>2315/78</t>
+          <t>1025/1</t>
         </is>
       </c>
       <c r="E68" t="inlineStr">
         <is>
-          <t>Stodůlky</t>
+          <t>Malešice</t>
         </is>
       </c>
       <c r="F68" t="inlineStr">
         <is>
-          <t>jednotka č. 26150035, jiný nebytový prostor v budově č.p. 2615, část obce Stodůlky, na parcele 2315/78 Stodůlky, podíl na společných částech domu a pozemku 18/39105</t>
+          <t>č. 1025/1 Malešice</t>
         </is>
       </c>
       <c r="G68" t="n">
@@ -3012,17 +3012,17 @@
       </c>
       <c r="H68" t="inlineStr">
         <is>
-          <t>jednotka na parcele bez prefixu st. + KU</t>
+          <t>číslo a KU za ním</t>
         </is>
       </c>
     </row>
     <row r="69">
       <c r="A69" t="n">
-        <v>37247</v>
+        <v>30921</v>
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>jednotka</t>
+          <t>parcela</t>
         </is>
       </c>
       <c r="C69" t="inlineStr">
@@ -3032,17 +3032,17 @@
       </c>
       <c r="D69" t="inlineStr">
         <is>
-          <t>2315/78</t>
+          <t>1818/28</t>
         </is>
       </c>
       <c r="E69" t="inlineStr">
         <is>
-          <t>Stodůlky</t>
+          <t>Hostivař</t>
         </is>
       </c>
       <c r="F69" t="inlineStr">
         <is>
-          <t>jednotka č. 26150205, byt v budově č.p. 2615, část obce Stodůlky, na parcele 2315/78 Stodůlky, podíl na společných částech domu a pozemku 404/39105</t>
+          <t>č. 1818/28 Hostivař</t>
         </is>
       </c>
       <c r="G69" t="n">
@@ -3050,13 +3050,13 @@
       </c>
       <c r="H69" t="inlineStr">
         <is>
-          <t>jednotka na parcele bez prefixu st. + KU</t>
+          <t>číslo a KU za ním</t>
         </is>
       </c>
     </row>
     <row r="70">
       <c r="A70" t="n">
-        <v>37246</v>
+        <v>30926</v>
       </c>
       <c r="B70" t="inlineStr">
         <is>
@@ -3070,17 +3070,17 @@
       </c>
       <c r="D70" t="inlineStr">
         <is>
-          <t>162/839</t>
+          <t>1761/233</t>
         </is>
       </c>
       <c r="E70" t="inlineStr">
         <is>
-          <t>Stodůlky</t>
+          <t>Hostivař</t>
         </is>
       </c>
       <c r="F70" t="inlineStr">
         <is>
-          <t>č. 162/839 Stodůlky</t>
+          <t>č. 1761/233 Hostivař</t>
         </is>
       </c>
       <c r="G70" t="n">
@@ -3094,7 +3094,7 @@
     </row>
     <row r="71">
       <c r="A71" t="n">
-        <v>37245</v>
+        <v>28092</v>
       </c>
       <c r="B71" t="inlineStr">
         <is>
@@ -3108,17 +3108,17 @@
       </c>
       <c r="D71" t="inlineStr">
         <is>
-          <t>162/848</t>
+          <t>4390/105</t>
         </is>
       </c>
       <c r="E71" t="inlineStr">
         <is>
-          <t>Stodůlky</t>
+          <t>Strašnice</t>
         </is>
       </c>
       <c r="F71" t="inlineStr">
         <is>
-          <t>č. 162/848 Stodůlky</t>
+          <t>č. 4390/105 Strašnice</t>
         </is>
       </c>
       <c r="G71" t="n">
@@ -3132,7 +3132,7 @@
     </row>
     <row r="72">
       <c r="A72" t="n">
-        <v>37244</v>
+        <v>24729</v>
       </c>
       <c r="B72" t="inlineStr">
         <is>
@@ -3146,17 +3146,17 @@
       </c>
       <c r="D72" t="inlineStr">
         <is>
-          <t>162/850</t>
+          <t>2244/2</t>
         </is>
       </c>
       <c r="E72" t="inlineStr">
         <is>
-          <t>Stodůlky</t>
+          <t>Strašnice</t>
         </is>
       </c>
       <c r="F72" t="inlineStr">
         <is>
-          <t>č. 162/850 Stodůlky</t>
+          <t>č. 2244/2 Strašnice</t>
         </is>
       </c>
       <c r="G72" t="n">
@@ -3170,7 +3170,7 @@
     </row>
     <row r="73">
       <c r="A73" t="n">
-        <v>37243</v>
+        <v>24888</v>
       </c>
       <c r="B73" t="inlineStr">
         <is>
@@ -3184,17 +3184,17 @@
       </c>
       <c r="D73" t="inlineStr">
         <is>
-          <t>162/845</t>
+          <t>1025/1</t>
         </is>
       </c>
       <c r="E73" t="inlineStr">
         <is>
-          <t>Stodůlky</t>
+          <t>Malešice</t>
         </is>
       </c>
       <c r="F73" t="inlineStr">
         <is>
-          <t>č. 162/845 Stodůlky</t>
+          <t>č. 1025/1 Malešice</t>
         </is>
       </c>
       <c r="G73" t="n">
@@ -3208,7 +3208,7 @@
     </row>
     <row r="74">
       <c r="A74" t="n">
-        <v>37242</v>
+        <v>25287</v>
       </c>
       <c r="B74" t="inlineStr">
         <is>
@@ -3222,17 +3222,17 @@
       </c>
       <c r="D74" t="inlineStr">
         <is>
-          <t>162/840</t>
+          <t>1025/1</t>
         </is>
       </c>
       <c r="E74" t="inlineStr">
         <is>
-          <t>Stodůlky</t>
+          <t>Malešice</t>
         </is>
       </c>
       <c r="F74" t="inlineStr">
         <is>
-          <t>č. 162/840 Stodůlky</t>
+          <t>č. 1025/1 Malešice</t>
         </is>
       </c>
       <c r="G74" t="n">
@@ -3246,7 +3246,7 @@
     </row>
     <row r="75">
       <c r="A75" t="n">
-        <v>37241</v>
+        <v>26229</v>
       </c>
       <c r="B75" t="inlineStr">
         <is>
@@ -3260,17 +3260,17 @@
       </c>
       <c r="D75" t="inlineStr">
         <is>
-          <t>162/842</t>
+          <t>349/107</t>
         </is>
       </c>
       <c r="E75" t="inlineStr">
         <is>
-          <t>Stodůlky</t>
+          <t>Štěrboholy</t>
         </is>
       </c>
       <c r="F75" t="inlineStr">
         <is>
-          <t>č. 162/842 Stodůlky</t>
+          <t>č. 349/107 Štěrboholy</t>
         </is>
       </c>
       <c r="G75" t="n">
@@ -3284,7 +3284,7 @@
     </row>
     <row r="76">
       <c r="A76" t="n">
-        <v>37240</v>
+        <v>28077</v>
       </c>
       <c r="B76" t="inlineStr">
         <is>
@@ -3298,17 +3298,17 @@
       </c>
       <c r="D76" t="inlineStr">
         <is>
-          <t>162/786</t>
+          <t>3925/16</t>
         </is>
       </c>
       <c r="E76" t="inlineStr">
         <is>
-          <t>Stodůlky</t>
+          <t>Strašnice</t>
         </is>
       </c>
       <c r="F76" t="inlineStr">
         <is>
-          <t>č. 162/786 Stodůlky</t>
+          <t>č. 3925/16 Strašnice</t>
         </is>
       </c>
       <c r="G76" t="n">
@@ -3322,7 +3322,7 @@
     </row>
     <row r="77">
       <c r="A77" t="n">
-        <v>37239</v>
+        <v>28089</v>
       </c>
       <c r="B77" t="inlineStr">
         <is>
@@ -3336,17 +3336,17 @@
       </c>
       <c r="D77" t="inlineStr">
         <is>
-          <t>162/849</t>
+          <t>4269/2</t>
         </is>
       </c>
       <c r="E77" t="inlineStr">
         <is>
-          <t>Stodůlky</t>
+          <t>Strašnice</t>
         </is>
       </c>
       <c r="F77" t="inlineStr">
         <is>
-          <t>č. 162/849 Stodůlky</t>
+          <t>č. 4269/2 Strašnice</t>
         </is>
       </c>
       <c r="G77" t="n">
@@ -3360,7 +3360,7 @@
     </row>
     <row r="78">
       <c r="A78" t="n">
-        <v>37238</v>
+        <v>68480</v>
       </c>
       <c r="B78" t="inlineStr">
         <is>
@@ -3374,17 +3374,17 @@
       </c>
       <c r="D78" t="inlineStr">
         <is>
-          <t>162/844</t>
+          <t>2742/119</t>
         </is>
       </c>
       <c r="E78" t="inlineStr">
         <is>
-          <t>Stodůlky</t>
+          <t>Hostivař</t>
         </is>
       </c>
       <c r="F78" t="inlineStr">
         <is>
-          <t>č. 162/844 Stodůlky</t>
+          <t>č. 2742/119 Hostivař</t>
         </is>
       </c>
       <c r="G78" t="n">
@@ -3398,7 +3398,7 @@
     </row>
     <row r="79">
       <c r="A79" t="n">
-        <v>37237</v>
+        <v>68572</v>
       </c>
       <c r="B79" t="inlineStr">
         <is>
@@ -3412,17 +3412,17 @@
       </c>
       <c r="D79" t="inlineStr">
         <is>
-          <t>162/783</t>
+          <t>3220/12</t>
         </is>
       </c>
       <c r="E79" t="inlineStr">
         <is>
-          <t>Stodůlky</t>
+          <t>Strašnice</t>
         </is>
       </c>
       <c r="F79" t="inlineStr">
         <is>
-          <t>č. 162/783 Stodůlky</t>
+          <t>č. 3220/12 Strašnice</t>
         </is>
       </c>
       <c r="G79" t="n">
@@ -3436,7 +3436,7 @@
     </row>
     <row r="80">
       <c r="A80" t="n">
-        <v>37236</v>
+        <v>28005</v>
       </c>
       <c r="B80" t="inlineStr">
         <is>
@@ -3450,17 +3450,17 @@
       </c>
       <c r="D80" t="inlineStr">
         <is>
-          <t>162/230</t>
+          <t>4458/2</t>
         </is>
       </c>
       <c r="E80" t="inlineStr">
         <is>
-          <t>Stodůlky</t>
+          <t>Strašnice</t>
         </is>
       </c>
       <c r="F80" t="inlineStr">
         <is>
-          <t>č. 162/230 Stodůlky</t>
+          <t>č. 4458/2 Strašnice</t>
         </is>
       </c>
       <c r="G80" t="n">
@@ -3474,7 +3474,7 @@
     </row>
     <row r="81">
       <c r="A81" t="n">
-        <v>37235</v>
+        <v>68617</v>
       </c>
       <c r="B81" t="inlineStr">
         <is>
@@ -3488,17 +3488,17 @@
       </c>
       <c r="D81" t="inlineStr">
         <is>
-          <t>162/846</t>
+          <t>1292/84</t>
         </is>
       </c>
       <c r="E81" t="inlineStr">
         <is>
-          <t>Stodůlky</t>
+          <t>Strašnice</t>
         </is>
       </c>
       <c r="F81" t="inlineStr">
         <is>
-          <t>č. 162/846 Stodůlky</t>
+          <t>č. 1292/84 Strašnice</t>
         </is>
       </c>
       <c r="G81" t="n">
@@ -3512,7 +3512,7 @@
     </row>
     <row r="82">
       <c r="A82" t="n">
-        <v>37234</v>
+        <v>30913</v>
       </c>
       <c r="B82" t="inlineStr">
         <is>
@@ -3526,23 +3526,745 @@
       </c>
       <c r="D82" t="inlineStr">
         <is>
-          <t>162/841</t>
+          <t>654/7</t>
         </is>
       </c>
       <c r="E82" t="inlineStr">
         <is>
-          <t>Stodůlky</t>
+          <t>Hostivař</t>
         </is>
       </c>
       <c r="F82" t="inlineStr">
         <is>
-          <t>č. 162/841 Stodůlky</t>
+          <t>č. 654/7 Hostivař (součástí je stavba budova bez čp/če, garáž)</t>
         </is>
       </c>
       <c r="G82" t="n">
         <v>1</v>
       </c>
       <c r="H82" t="inlineStr">
+        <is>
+          <t>číslo a KU za ním</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" t="n">
+        <v>68640</v>
+      </c>
+      <c r="B83" t="inlineStr">
+        <is>
+          <t>parcela</t>
+        </is>
+      </c>
+      <c r="C83" t="inlineStr">
+        <is>
+          <t>Hlavní město Praha</t>
+        </is>
+      </c>
+      <c r="D83" t="inlineStr">
+        <is>
+          <t>1292/103</t>
+        </is>
+      </c>
+      <c r="E83" t="inlineStr">
+        <is>
+          <t>Strašnice</t>
+        </is>
+      </c>
+      <c r="F83" t="inlineStr">
+        <is>
+          <t>č. 1292/103 Strašnice</t>
+        </is>
+      </c>
+      <c r="G83" t="n">
+        <v>1</v>
+      </c>
+      <c r="H83" t="inlineStr">
+        <is>
+          <t>číslo a KU za ním</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" t="n">
+        <v>28260</v>
+      </c>
+      <c r="B84" t="inlineStr">
+        <is>
+          <t>parcela</t>
+        </is>
+      </c>
+      <c r="C84" t="inlineStr">
+        <is>
+          <t>Hlavní město Praha</t>
+        </is>
+      </c>
+      <c r="D84" t="inlineStr">
+        <is>
+          <t>2840/3</t>
+        </is>
+      </c>
+      <c r="E84" t="inlineStr">
+        <is>
+          <t>Strašnice</t>
+        </is>
+      </c>
+      <c r="F84" t="inlineStr">
+        <is>
+          <t>č. 2840/3 Strašnice</t>
+        </is>
+      </c>
+      <c r="G84" t="n">
+        <v>1</v>
+      </c>
+      <c r="H84" t="inlineStr">
+        <is>
+          <t>číslo a KU za ním</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" t="n">
+        <v>68591</v>
+      </c>
+      <c r="B85" t="inlineStr">
+        <is>
+          <t>parcela</t>
+        </is>
+      </c>
+      <c r="C85" t="inlineStr">
+        <is>
+          <t>Hlavní město Praha</t>
+        </is>
+      </c>
+      <c r="D85" t="inlineStr">
+        <is>
+          <t>2585/35</t>
+        </is>
+      </c>
+      <c r="E85" t="inlineStr">
+        <is>
+          <t>Strašnice</t>
+        </is>
+      </c>
+      <c r="F85" t="inlineStr">
+        <is>
+          <t>č. 2585/35 Strašnice</t>
+        </is>
+      </c>
+      <c r="G85" t="n">
+        <v>1</v>
+      </c>
+      <c r="H85" t="inlineStr">
+        <is>
+          <t>číslo a KU za ním</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" t="n">
+        <v>68293</v>
+      </c>
+      <c r="B86" t="inlineStr">
+        <is>
+          <t>parcela</t>
+        </is>
+      </c>
+      <c r="C86" t="inlineStr">
+        <is>
+          <t>Hlavní město Praha</t>
+        </is>
+      </c>
+      <c r="D86" t="inlineStr">
+        <is>
+          <t>1002/2</t>
+        </is>
+      </c>
+      <c r="E86" t="inlineStr">
+        <is>
+          <t>Nové Sedlo u Lokte</t>
+        </is>
+      </c>
+      <c r="F86" t="inlineStr">
+        <is>
+          <t>č. 1002/2 Nové Sedlo u Lokte</t>
+        </is>
+      </c>
+      <c r="G86" t="n">
+        <v>1</v>
+      </c>
+      <c r="H86" t="inlineStr">
+        <is>
+          <t>číslo a KU za ním</t>
+        </is>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" t="n">
+        <v>68590</v>
+      </c>
+      <c r="B87" t="inlineStr">
+        <is>
+          <t>parcela</t>
+        </is>
+      </c>
+      <c r="C87" t="inlineStr">
+        <is>
+          <t>Hlavní město Praha</t>
+        </is>
+      </c>
+      <c r="D87" t="inlineStr">
+        <is>
+          <t>1292/84</t>
+        </is>
+      </c>
+      <c r="E87" t="inlineStr">
+        <is>
+          <t>Strašnice</t>
+        </is>
+      </c>
+      <c r="F87" t="inlineStr">
+        <is>
+          <t>č. 1292/84 Strašnice</t>
+        </is>
+      </c>
+      <c r="G87" t="n">
+        <v>1</v>
+      </c>
+      <c r="H87" t="inlineStr">
+        <is>
+          <t>číslo a KU za ním</t>
+        </is>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" t="n">
+        <v>68605</v>
+      </c>
+      <c r="B88" t="inlineStr">
+        <is>
+          <t>parcela</t>
+        </is>
+      </c>
+      <c r="C88" t="inlineStr">
+        <is>
+          <t>Hlavní město Praha</t>
+        </is>
+      </c>
+      <c r="D88" t="inlineStr">
+        <is>
+          <t>2885</t>
+        </is>
+      </c>
+      <c r="E88" t="inlineStr">
+        <is>
+          <t>Strašnice</t>
+        </is>
+      </c>
+      <c r="F88" t="inlineStr">
+        <is>
+          <t>č. 2885 Strašnice</t>
+        </is>
+      </c>
+      <c r="G88" t="n">
+        <v>1</v>
+      </c>
+      <c r="H88" t="inlineStr">
+        <is>
+          <t>číslo a KU za ním</t>
+        </is>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" t="n">
+        <v>28286</v>
+      </c>
+      <c r="B89" t="inlineStr">
+        <is>
+          <t>parcela</t>
+        </is>
+      </c>
+      <c r="C89" t="inlineStr">
+        <is>
+          <t>Hlavní město Praha</t>
+        </is>
+      </c>
+      <c r="D89" t="inlineStr">
+        <is>
+          <t>4089/1</t>
+        </is>
+      </c>
+      <c r="E89" t="inlineStr">
+        <is>
+          <t>Strašnice</t>
+        </is>
+      </c>
+      <c r="F89" t="inlineStr">
+        <is>
+          <t>č. 4089/1 Strašnice</t>
+        </is>
+      </c>
+      <c r="G89" t="n">
+        <v>1</v>
+      </c>
+      <c r="H89" t="inlineStr">
+        <is>
+          <t>číslo a KU za ním</t>
+        </is>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" t="n">
+        <v>68153</v>
+      </c>
+      <c r="B90" t="inlineStr">
+        <is>
+          <t>parcela</t>
+        </is>
+      </c>
+      <c r="C90" t="inlineStr">
+        <is>
+          <t>Hlavní město Praha</t>
+        </is>
+      </c>
+      <c r="D90" t="inlineStr">
+        <is>
+          <t>4031/112</t>
+        </is>
+      </c>
+      <c r="E90" t="inlineStr">
+        <is>
+          <t>Strašnice</t>
+        </is>
+      </c>
+      <c r="F90" t="inlineStr">
+        <is>
+          <t>č. 4031/112 Strašnice</t>
+        </is>
+      </c>
+      <c r="G90" t="n">
+        <v>1</v>
+      </c>
+      <c r="H90" t="inlineStr">
+        <is>
+          <t>číslo a KU za ním</t>
+        </is>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" t="n">
+        <v>24901</v>
+      </c>
+      <c r="B91" t="inlineStr">
+        <is>
+          <t>parcela</t>
+        </is>
+      </c>
+      <c r="C91" t="inlineStr">
+        <is>
+          <t>Hlavní město Praha</t>
+        </is>
+      </c>
+      <c r="D91" t="inlineStr">
+        <is>
+          <t>1025/1</t>
+        </is>
+      </c>
+      <c r="E91" t="inlineStr">
+        <is>
+          <t>Malešice</t>
+        </is>
+      </c>
+      <c r="F91" t="inlineStr">
+        <is>
+          <t>č. 1025/1 Malešice</t>
+        </is>
+      </c>
+      <c r="G91" t="n">
+        <v>1</v>
+      </c>
+      <c r="H91" t="inlineStr">
+        <is>
+          <t>číslo a KU za ním</t>
+        </is>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" t="n">
+        <v>25275</v>
+      </c>
+      <c r="B92" t="inlineStr">
+        <is>
+          <t>parcela</t>
+        </is>
+      </c>
+      <c r="C92" t="inlineStr">
+        <is>
+          <t>Hlavní město Praha</t>
+        </is>
+      </c>
+      <c r="D92" t="inlineStr">
+        <is>
+          <t>1025/1</t>
+        </is>
+      </c>
+      <c r="E92" t="inlineStr">
+        <is>
+          <t>Malešice</t>
+        </is>
+      </c>
+      <c r="F92" t="inlineStr">
+        <is>
+          <t>č. 1025/1 Malešice</t>
+        </is>
+      </c>
+      <c r="G92" t="n">
+        <v>1</v>
+      </c>
+      <c r="H92" t="inlineStr">
+        <is>
+          <t>číslo a KU za ním</t>
+        </is>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" t="n">
+        <v>25297</v>
+      </c>
+      <c r="B93" t="inlineStr">
+        <is>
+          <t>parcela</t>
+        </is>
+      </c>
+      <c r="C93" t="inlineStr">
+        <is>
+          <t>Hlavní město Praha</t>
+        </is>
+      </c>
+      <c r="D93" t="inlineStr">
+        <is>
+          <t>154</t>
+        </is>
+      </c>
+      <c r="E93" t="inlineStr">
+        <is>
+          <t>Malešice</t>
+        </is>
+      </c>
+      <c r="F93" t="inlineStr">
+        <is>
+          <t>č. 154 Malešice</t>
+        </is>
+      </c>
+      <c r="G93" t="n">
+        <v>1</v>
+      </c>
+      <c r="H93" t="inlineStr">
+        <is>
+          <t>číslo a KU za ním</t>
+        </is>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" t="n">
+        <v>28199</v>
+      </c>
+      <c r="B94" t="inlineStr">
+        <is>
+          <t>parcela</t>
+        </is>
+      </c>
+      <c r="C94" t="inlineStr">
+        <is>
+          <t>Hlavní město Praha</t>
+        </is>
+      </c>
+      <c r="D94" t="inlineStr">
+        <is>
+          <t>2838/64</t>
+        </is>
+      </c>
+      <c r="E94" t="inlineStr">
+        <is>
+          <t>Strašnice</t>
+        </is>
+      </c>
+      <c r="F94" t="inlineStr">
+        <is>
+          <t>č. 2838/64 Strašnice</t>
+        </is>
+      </c>
+      <c r="G94" t="n">
+        <v>1</v>
+      </c>
+      <c r="H94" t="inlineStr">
+        <is>
+          <t>číslo a KU za ním</t>
+        </is>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" t="n">
+        <v>68633</v>
+      </c>
+      <c r="B95" t="inlineStr">
+        <is>
+          <t>parcela</t>
+        </is>
+      </c>
+      <c r="C95" t="inlineStr">
+        <is>
+          <t>Hlavní město Praha</t>
+        </is>
+      </c>
+      <c r="D95" t="inlineStr">
+        <is>
+          <t>2764/37</t>
+        </is>
+      </c>
+      <c r="E95" t="inlineStr">
+        <is>
+          <t>Strašnice</t>
+        </is>
+      </c>
+      <c r="F95" t="inlineStr">
+        <is>
+          <t>č. 2764/37 Strašnice</t>
+        </is>
+      </c>
+      <c r="G95" t="n">
+        <v>1</v>
+      </c>
+      <c r="H95" t="inlineStr">
+        <is>
+          <t>číslo a KU za ním</t>
+        </is>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" t="n">
+        <v>25280</v>
+      </c>
+      <c r="B96" t="inlineStr">
+        <is>
+          <t>parcela</t>
+        </is>
+      </c>
+      <c r="C96" t="inlineStr">
+        <is>
+          <t>Hlavní město Praha</t>
+        </is>
+      </c>
+      <c r="D96" t="inlineStr">
+        <is>
+          <t>1025/1</t>
+        </is>
+      </c>
+      <c r="E96" t="inlineStr">
+        <is>
+          <t>Malešice</t>
+        </is>
+      </c>
+      <c r="F96" t="inlineStr">
+        <is>
+          <t>č. 1025/1 Malešice</t>
+        </is>
+      </c>
+      <c r="G96" t="n">
+        <v>1</v>
+      </c>
+      <c r="H96" t="inlineStr">
+        <is>
+          <t>číslo a KU za ním</t>
+        </is>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" t="n">
+        <v>68652</v>
+      </c>
+      <c r="B97" t="inlineStr">
+        <is>
+          <t>parcela</t>
+        </is>
+      </c>
+      <c r="C97" t="inlineStr">
+        <is>
+          <t>Hlavní město Praha</t>
+        </is>
+      </c>
+      <c r="D97" t="inlineStr">
+        <is>
+          <t>4307/112</t>
+        </is>
+      </c>
+      <c r="E97" t="inlineStr">
+        <is>
+          <t>Strašnice</t>
+        </is>
+      </c>
+      <c r="F97" t="inlineStr">
+        <is>
+          <t>č. 4307/112 Strašnice</t>
+        </is>
+      </c>
+      <c r="G97" t="n">
+        <v>1</v>
+      </c>
+      <c r="H97" t="inlineStr">
+        <is>
+          <t>číslo a KU za ním</t>
+        </is>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" t="n">
+        <v>68597</v>
+      </c>
+      <c r="B98" t="inlineStr">
+        <is>
+          <t>parcela</t>
+        </is>
+      </c>
+      <c r="C98" t="inlineStr">
+        <is>
+          <t>Hlavní město Praha</t>
+        </is>
+      </c>
+      <c r="D98" t="inlineStr">
+        <is>
+          <t>3237/7</t>
+        </is>
+      </c>
+      <c r="E98" t="inlineStr">
+        <is>
+          <t>Strašnice</t>
+        </is>
+      </c>
+      <c r="F98" t="inlineStr">
+        <is>
+          <t>č. 3237/7 Strašnice</t>
+        </is>
+      </c>
+      <c r="G98" t="n">
+        <v>1</v>
+      </c>
+      <c r="H98" t="inlineStr">
+        <is>
+          <t>číslo a KU za ním</t>
+        </is>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" t="n">
+        <v>68565</v>
+      </c>
+      <c r="B99" t="inlineStr">
+        <is>
+          <t>parcela</t>
+        </is>
+      </c>
+      <c r="C99" t="inlineStr">
+        <is>
+          <t>Hlavní město Praha</t>
+        </is>
+      </c>
+      <c r="D99" t="inlineStr">
+        <is>
+          <t>3115/52</t>
+        </is>
+      </c>
+      <c r="E99" t="inlineStr">
+        <is>
+          <t>Strašnice</t>
+        </is>
+      </c>
+      <c r="F99" t="inlineStr">
+        <is>
+          <t>č. 3115/52 Strašnice</t>
+        </is>
+      </c>
+      <c r="G99" t="n">
+        <v>1</v>
+      </c>
+      <c r="H99" t="inlineStr">
+        <is>
+          <t>číslo a KU za ním</t>
+        </is>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" t="n">
+        <v>68613</v>
+      </c>
+      <c r="B100" t="inlineStr">
+        <is>
+          <t>parcela</t>
+        </is>
+      </c>
+      <c r="C100" t="inlineStr">
+        <is>
+          <t>Hlavní město Praha</t>
+        </is>
+      </c>
+      <c r="D100" t="inlineStr">
+        <is>
+          <t>2706</t>
+        </is>
+      </c>
+      <c r="E100" t="inlineStr">
+        <is>
+          <t>Strašnice</t>
+        </is>
+      </c>
+      <c r="F100" t="inlineStr">
+        <is>
+          <t>č. 2706 Strašnice</t>
+        </is>
+      </c>
+      <c r="G100" t="n">
+        <v>1</v>
+      </c>
+      <c r="H100" t="inlineStr">
+        <is>
+          <t>číslo a KU za ním</t>
+        </is>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" t="n">
+        <v>68477</v>
+      </c>
+      <c r="B101" t="inlineStr">
+        <is>
+          <t>parcela</t>
+        </is>
+      </c>
+      <c r="C101" t="inlineStr">
+        <is>
+          <t>Hlavní město Praha</t>
+        </is>
+      </c>
+      <c r="D101" t="inlineStr">
+        <is>
+          <t>1818/25</t>
+        </is>
+      </c>
+      <c r="E101" t="inlineStr">
+        <is>
+          <t>Hostivař</t>
+        </is>
+      </c>
+      <c r="F101" t="inlineStr">
+        <is>
+          <t>č. 1818/25 Hostivař</t>
+        </is>
+      </c>
+      <c r="G101" t="n">
+        <v>1</v>
+      </c>
+      <c r="H101" t="inlineStr">
         <is>
           <t>číslo a KU za ním</t>
         </is>

</xml_diff>